<commit_message>
[queue] Claim [EPIC_05][STORY_02][SUBSTORY_02] #675 MCP resource limits
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-1, claim 8f10594c-ba5d-4625-bc96-935dda260806, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -3983,7 +3983,8 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:dimension ref="A1:AC30"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="58" hidden="0" customWidth="1"/>
@@ -6139,25 +6140,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R27" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R27" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+      </x:c>
       <x:c r="S27" s="39"/>
-      <x:c r="T27" s="39"/>
-      <x:c r="U27" s="39"/>
-      <x:c r="V27" s="39"/>
-      <x:c r="W27" s="39"/>
+      <x:c r="T27" s="39" t="str">
+        <x:v>8f10594c-ba5d-4625-bc96-935dda260806</x:v>
+      </x:c>
+      <x:c r="U27" s="39" t="str">
+        <x:v>2026-06-30T05:31:51Z</x:v>
+      </x:c>
+      <x:c r="V27" s="39" t="str">
+        <x:v>2026-06-30T05:31:51Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39" t="str">
+        <x:v>2026-07-01T05:31:51Z</x:v>
+      </x:c>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Migrated from GitHub issue #675; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>
       <x:c r="AC27" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="72" customHeight="1">
@@ -6425,7 +6436,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6ad6fa389ea467f"/>
+    <x:tablePart r:id="Rd6ad6fa389ea467f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_02][SUBSTORY_02] #675 MCP resource limits (#886)
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-1, claim 8f10594c-ba5d-4625-bc96-935dda260806, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -3983,7 +3983,8 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:dimension ref="A1:AC30"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="58" hidden="0" customWidth="1"/>
@@ -6139,25 +6140,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R27" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R27" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+      </x:c>
       <x:c r="S27" s="39"/>
-      <x:c r="T27" s="39"/>
-      <x:c r="U27" s="39"/>
-      <x:c r="V27" s="39"/>
-      <x:c r="W27" s="39"/>
+      <x:c r="T27" s="39" t="str">
+        <x:v>8f10594c-ba5d-4625-bc96-935dda260806</x:v>
+      </x:c>
+      <x:c r="U27" s="39" t="str">
+        <x:v>2026-06-30T05:31:51Z</x:v>
+      </x:c>
+      <x:c r="V27" s="39" t="str">
+        <x:v>2026-06-30T05:31:51Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39" t="str">
+        <x:v>2026-07-01T05:31:51Z</x:v>
+      </x:c>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Migrated from GitHub issue #675; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>
       <x:c r="AC27" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="72" customHeight="1">
@@ -6425,7 +6436,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6ad6fa389ea467f"/>
+    <x:tablePart r:id="Rd6ad6fa389ea467f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Claim EPIC_05/STORY_03/SUBSTORY_01 #674 bound saved-quest reference traversal
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6061,25 +6061,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/save format/schema helpers</x:v>
       </x:c>
       <x:c r="Q26" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R26" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R26" s="36" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
+      </x:c>
       <x:c r="S26" s="36"/>
-      <x:c r="T26" s="36"/>
-      <x:c r="U26" s="36"/>
-      <x:c r="V26" s="36"/>
-      <x:c r="W26" s="36"/>
+      <x:c r="T26" s="36" t="str">
+        <x:v>14969684-0d98-40aa-9eee-da188f53d795</x:v>
+      </x:c>
+      <x:c r="U26" s="36" t="str">
+        <x:v>2026-06-30T10:20:13Z</x:v>
+      </x:c>
+      <x:c r="V26" s="36" t="str">
+        <x:v>2026-06-30T10:20:13Z</x:v>
+      </x:c>
+      <x:c r="W26" s="36" t="str">
+        <x:v>2026-07-01T10:20:13Z</x:v>
+      </x:c>
       <x:c r="X26" s="36"/>
       <x:c r="Y26" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z26" s="36" t="str">
-        <x:v>Migrated from GitHub issue #674; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
       </x:c>
       <x:c r="AA26" s="36"/>
       <x:c r="AB26" s="36"/>
       <x:c r="AC26" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim EPIC_05/STORY_03/SUBSTORY_01 #674 bound saved-quest reference traversal (#891)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6061,25 +6061,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/save format/schema helpers</x:v>
       </x:c>
       <x:c r="Q26" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R26" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R26" s="36" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
+      </x:c>
       <x:c r="S26" s="36"/>
-      <x:c r="T26" s="36"/>
-      <x:c r="U26" s="36"/>
-      <x:c r="V26" s="36"/>
-      <x:c r="W26" s="36"/>
+      <x:c r="T26" s="36" t="str">
+        <x:v>14969684-0d98-40aa-9eee-da188f53d795</x:v>
+      </x:c>
+      <x:c r="U26" s="36" t="str">
+        <x:v>2026-06-30T10:20:13Z</x:v>
+      </x:c>
+      <x:c r="V26" s="36" t="str">
+        <x:v>2026-06-30T10:20:13Z</x:v>
+      </x:c>
+      <x:c r="W26" s="36" t="str">
+        <x:v>2026-07-01T10:20:13Z</x:v>
+      </x:c>
       <x:c r="X26" s="36"/>
       <x:c r="Y26" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z26" s="36" t="str">
-        <x:v>Migrated from GitHub issue #674; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
       </x:c>
       <x:c r="AA26" s="36"/>
       <x:c r="AB26" s="36"/>
       <x:c r="AC26" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim EPIC_05/STORY_02/SUBSTORY_01 #672 enforce per-action limits in MCP simulation_run
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5906,25 +5906,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/game_simulation.py</x:v>
       </x:c>
       <x:c r="Q24" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R24" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R24" s="36" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
+      </x:c>
       <x:c r="S24" s="36"/>
-      <x:c r="T24" s="36"/>
-      <x:c r="U24" s="36"/>
-      <x:c r="V24" s="36"/>
-      <x:c r="W24" s="36"/>
+      <x:c r="T24" s="36" t="str">
+        <x:v>3992c184-c78b-480e-9626-73e7d5c78d21</x:v>
+      </x:c>
+      <x:c r="U24" s="36" t="str">
+        <x:v>2026-06-30T10:25:40Z</x:v>
+      </x:c>
+      <x:c r="V24" s="36" t="str">
+        <x:v>2026-06-30T10:25:40Z</x:v>
+      </x:c>
+      <x:c r="W24" s="36" t="str">
+        <x:v>2026-07-01T10:25:40Z</x:v>
+      </x:c>
       <x:c r="X24" s="36"/>
       <x:c r="Y24" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z24" s="36" t="str">
-        <x:v>Migrated from GitHub issue #672; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
       </x:c>
       <x:c r="AA24" s="36"/>
       <x:c r="AB24" s="36"/>
       <x:c r="AC24" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim EPIC_05/STORY_02/SUBSTORY_01 #672 enforce per-action limits in MCP simulation_run (#893)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5906,25 +5906,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/game_simulation.py</x:v>
       </x:c>
       <x:c r="Q24" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R24" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R24" s="36" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
+      </x:c>
       <x:c r="S24" s="36"/>
-      <x:c r="T24" s="36"/>
-      <x:c r="U24" s="36"/>
-      <x:c r="V24" s="36"/>
-      <x:c r="W24" s="36"/>
+      <x:c r="T24" s="36" t="str">
+        <x:v>3992c184-c78b-480e-9626-73e7d5c78d21</x:v>
+      </x:c>
+      <x:c r="U24" s="36" t="str">
+        <x:v>2026-06-30T10:25:40Z</x:v>
+      </x:c>
+      <x:c r="V24" s="36" t="str">
+        <x:v>2026-06-30T10:25:40Z</x:v>
+      </x:c>
+      <x:c r="W24" s="36" t="str">
+        <x:v>2026-07-01T10:25:40Z</x:v>
+      </x:c>
       <x:c r="X24" s="36"/>
       <x:c r="Y24" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z24" s="36" t="str">
-        <x:v>Migrated from GitHub issue #672; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
       </x:c>
       <x:c r="AA24" s="36"/>
       <x:c r="AB24" s="36"/>
       <x:c r="AC24" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="72" customHeight="1">

</xml_diff>

<commit_message>
[queue] Release [EPIC_05][STORY_02][SUBSTORY_02] #675 back to NOT_STARTED
Dispatched worker cut off by session limit before any implementation; no work done.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6160,30 +6160,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R27" s="39" t="str">
-        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R27" s="39"/>
       <x:c r="S27" s="39"/>
-      <x:c r="T27" s="39" t="str">
-        <x:v>8f10594c-ba5d-4625-bc96-935dda260806</x:v>
-      </x:c>
-      <x:c r="U27" s="39" t="str">
-        <x:v>2026-06-30T05:31:51Z</x:v>
-      </x:c>
+      <x:c r="T27" s="39"/>
+      <x:c r="U27" s="39"/>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T05:31:51Z</x:v>
-      </x:c>
-      <x:c r="W27" s="39" t="str">
-        <x:v>2026-07-01T05:31:51Z</x:v>
-      </x:c>
+        <x:v>2026-06-30T10:47:27Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39"/>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+        <x:v>Released by controller ctrl-vm-4026-9b5a29b5: dispatched worker was cut off by a session/usage limit before any implementation (empty working tree). No material work done; returning to NOT_STARTED for re-dispatch.</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>

</xml_diff>

<commit_message>
[queue] Release [EPIC_05][STORY_02][SUBSTORY_02] #675 back to NOT_STARTED (#901)
Dispatched worker cut off by session limit before any implementation; no work done.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6160,30 +6160,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R27" s="39" t="str">
-        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R27" s="39"/>
       <x:c r="S27" s="39"/>
-      <x:c r="T27" s="39" t="str">
-        <x:v>8f10594c-ba5d-4625-bc96-935dda260806</x:v>
-      </x:c>
-      <x:c r="U27" s="39" t="str">
-        <x:v>2026-06-30T05:31:51Z</x:v>
-      </x:c>
+      <x:c r="T27" s="39"/>
+      <x:c r="U27" s="39"/>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T05:31:51Z</x:v>
-      </x:c>
-      <x:c r="W27" s="39" t="str">
-        <x:v>2026-07-01T05:31:51Z</x:v>
-      </x:c>
+        <x:v>2026-06-30T10:47:27Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39"/>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+        <x:v>Released by controller ctrl-vm-4026-9b5a29b5: dispatched worker was cut off by a session/usage limit before any implementation (empty working tree). No material work done; returning to NOT_STARTED for re-dispatch.</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_02][SUBSTORY_02] #675 Restrict MCP controller and pathfinding resource consumption
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-1, claim 3c1e98e5-1876-43a0-9d5a-3d32385cb41b, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6160,27 +6160,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R27" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R27" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+      </x:c>
       <x:c r="S27" s="39"/>
-      <x:c r="T27" s="39"/>
-      <x:c r="U27" s="39"/>
+      <x:c r="T27" s="39" t="str">
+        <x:v>3c1e98e5-1876-43a0-9d5a-3d32385cb41b</x:v>
+      </x:c>
+      <x:c r="U27" s="39" t="str">
+        <x:v>2026-06-30T10:50:10Z</x:v>
+      </x:c>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T10:47:27Z</x:v>
-      </x:c>
-      <x:c r="W27" s="39"/>
+        <x:v>2026-06-30T10:50:10Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39" t="str">
+        <x:v>2026-07-01T10:50:10Z</x:v>
+      </x:c>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Released by controller ctrl-vm-4026-9b5a29b5: dispatched worker was cut off by a session/usage limit before any implementation (empty working tree). No material work done; returning to NOT_STARTED for re-dispatch.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>
       <x:c r="AC27" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="72" customHeight="1">

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_02][SUBSTORY_02] #675 Restrict MCP controller and pathfinding resource consumption (#905)
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-1, claim 3c1e98e5-1876-43a0-9d5a-3d32385cb41b, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6160,27 +6160,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R27" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R27" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+      </x:c>
       <x:c r="S27" s="39"/>
-      <x:c r="T27" s="39"/>
-      <x:c r="U27" s="39"/>
+      <x:c r="T27" s="39" t="str">
+        <x:v>3c1e98e5-1876-43a0-9d5a-3d32385cb41b</x:v>
+      </x:c>
+      <x:c r="U27" s="39" t="str">
+        <x:v>2026-06-30T10:50:10Z</x:v>
+      </x:c>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T10:47:27Z</x:v>
-      </x:c>
-      <x:c r="W27" s="39"/>
+        <x:v>2026-06-30T10:50:10Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39" t="str">
+        <x:v>2026-07-01T10:50:10Z</x:v>
+      </x:c>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Released by controller ctrl-vm-4026-9b5a29b5: dispatched worker was cut off by a session/usage limit before any implementation (empty working tree). No material work done; returning to NOT_STARTED for re-dispatch.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>
       <x:c r="AC27" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="72" customHeight="1">

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_04][SUBSTORY_01] #676 Restore explicit authorization for agent auto-merge
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-3, claim fc03292a-02c4-44df-b1d5-5602832f0e6f, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6248,25 +6248,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/queue delivery documentation</x:v>
       </x:c>
       <x:c r="Q28" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R28" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R28" s="36" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
+      </x:c>
       <x:c r="S28" s="36"/>
-      <x:c r="T28" s="36"/>
-      <x:c r="U28" s="36"/>
-      <x:c r="V28" s="36"/>
-      <x:c r="W28" s="36"/>
+      <x:c r="T28" s="36" t="str">
+        <x:v>fc03292a-02c4-44df-b1d5-5602832f0e6f</x:v>
+      </x:c>
+      <x:c r="U28" s="36" t="str">
+        <x:v>2026-06-30T10:54:14Z</x:v>
+      </x:c>
+      <x:c r="V28" s="36" t="str">
+        <x:v>2026-06-30T10:54:14Z</x:v>
+      </x:c>
+      <x:c r="W28" s="36" t="str">
+        <x:v>2026-07-01T10:54:14Z</x:v>
+      </x:c>
       <x:c r="X28" s="36"/>
       <x:c r="Y28" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z28" s="36" t="str">
-        <x:v>Migrated from GitHub issue #676; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
       </x:c>
       <x:c r="AA28" s="36"/>
       <x:c r="AB28" s="36"/>
       <x:c r="AC28" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="72" customHeight="1">

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_04][SUBSTORY_01] #676 Restore explicit authorization for agent auto-merge (#910)
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-3, claim fc03292a-02c4-44df-b1d5-5602832f0e6f, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6248,25 +6248,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/queue delivery documentation</x:v>
       </x:c>
       <x:c r="Q28" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R28" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R28" s="36" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
+      </x:c>
       <x:c r="S28" s="36"/>
-      <x:c r="T28" s="36"/>
-      <x:c r="U28" s="36"/>
-      <x:c r="V28" s="36"/>
-      <x:c r="W28" s="36"/>
+      <x:c r="T28" s="36" t="str">
+        <x:v>fc03292a-02c4-44df-b1d5-5602832f0e6f</x:v>
+      </x:c>
+      <x:c r="U28" s="36" t="str">
+        <x:v>2026-06-30T10:54:14Z</x:v>
+      </x:c>
+      <x:c r="V28" s="36" t="str">
+        <x:v>2026-06-30T10:54:14Z</x:v>
+      </x:c>
+      <x:c r="W28" s="36" t="str">
+        <x:v>2026-07-01T10:54:14Z</x:v>
+      </x:c>
       <x:c r="X28" s="36"/>
       <x:c r="Y28" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z28" s="36" t="str">
-        <x:v>Migrated from GitHub issue #676; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
       </x:c>
       <x:c r="AA28" s="36"/>
       <x:c r="AB28" s="36"/>
       <x:c r="AC28" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="72" customHeight="1">

</xml_diff>

<commit_message>
[queue] Complete [EPIC_05][STORY_04][SUBSTORY_01] #676 Restore explicit authorization for agent auto-merge
Implementation merged via PR #916.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6248,7 +6248,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/queue delivery documentation</x:v>
       </x:c>
       <x:c r="Q28" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R28" s="36" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
@@ -6261,20 +6261,24 @@
         <x:v>2026-06-30T10:54:14Z</x:v>
       </x:c>
       <x:c r="V28" s="36" t="str">
-        <x:v>2026-06-30T10:54:14Z</x:v>
-      </x:c>
-      <x:c r="W28" s="36" t="str">
-        <x:v>2026-07-01T10:54:14Z</x:v>
-      </x:c>
-      <x:c r="X28" s="36"/>
+        <x:v>2026-06-30T11:02:32Z</x:v>
+      </x:c>
+      <x:c r="W28" s="36"/>
+      <x:c r="X28" s="36" t="str">
+        <x:v>2026-06-30T11:02:32Z</x:v>
+      </x:c>
       <x:c r="Y28" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z28" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
-      </x:c>
-      <x:c r="AA28" s="36"/>
-      <x:c r="AB28" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA28" s="36" t="str">
+        <x:v>Replaced the opt-out implementation-PR auto-merge default with a four-state authorization gate (allowed/user-authorized/disallowed/unknown) across AGENTS.md, the controller prompt, and the agent-queue doc; unknown/disallowed leaves the PR open and reports a blocker. Preserved the bounded workbook-only queue-state immediate-merge exception. Integrated with the existing controller_resource_audit.py merge-policy/branch-protection probing.</x:v>
+      </x:c>
+      <x:c r="AB28" s="36" t="str">
+        <x:v>python3 -m unittest tests.test_prompt_inventory -v: 6 passed (incl. new regression). GitHub Actions build workflow on PR #916: linux SUCCESS, linux-fast SUCCESS, validate SUCCESS, export SUCCESS; windows/windows-deps/linux-coverage skipped (workflow-only classification). Merged to main as c498086.</x:v>
+      </x:c>
       <x:c r="AC28" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
[queue] Complete [EPIC_05][STORY_04][SUBSTORY_01] #676 Restore explicit authorization for agent auto-merge (#922)
Implementation merged via PR #916.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6248,7 +6248,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/queue delivery documentation</x:v>
       </x:c>
       <x:c r="Q28" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R28" s="36" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
@@ -6261,20 +6261,24 @@
         <x:v>2026-06-30T10:54:14Z</x:v>
       </x:c>
       <x:c r="V28" s="36" t="str">
-        <x:v>2026-06-30T10:54:14Z</x:v>
-      </x:c>
-      <x:c r="W28" s="36" t="str">
-        <x:v>2026-07-01T10:54:14Z</x:v>
-      </x:c>
-      <x:c r="X28" s="36"/>
+        <x:v>2026-06-30T11:02:32Z</x:v>
+      </x:c>
+      <x:c r="W28" s="36"/>
+      <x:c r="X28" s="36" t="str">
+        <x:v>2026-06-30T11:02:32Z</x:v>
+      </x:c>
       <x:c r="Y28" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z28" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-3</x:v>
-      </x:c>
-      <x:c r="AA28" s="36"/>
-      <x:c r="AB28" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA28" s="36" t="str">
+        <x:v>Replaced the opt-out implementation-PR auto-merge default with a four-state authorization gate (allowed/user-authorized/disallowed/unknown) across AGENTS.md, the controller prompt, and the agent-queue doc; unknown/disallowed leaves the PR open and reports a blocker. Preserved the bounded workbook-only queue-state immediate-merge exception. Integrated with the existing controller_resource_audit.py merge-policy/branch-protection probing.</x:v>
+      </x:c>
+      <x:c r="AB28" s="36" t="str">
+        <x:v>python3 -m unittest tests.test_prompt_inventory -v: 6 passed (incl. new regression). GitHub Actions build workflow on PR #916: linux SUCCESS, linux-fast SUCCESS, validate SUCCESS, export SUCCESS; windows/windows-deps/linux-coverage skipped (workflow-only classification). Merged to main as c498086.</x:v>
+      </x:c>
       <x:c r="AC28" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
[queue] Claim [EPIC_02][STORY_01][SUBSTORY_02] #669 Harden CI validation authority for workflow changes
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-5, claim 4d74f425-a323-41d6-931b-13cf0d913a14, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5671,25 +5671,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R21" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R21" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
+      </x:c>
       <x:c r="S21" s="39"/>
-      <x:c r="T21" s="39"/>
-      <x:c r="U21" s="39"/>
-      <x:c r="V21" s="39"/>
-      <x:c r="W21" s="39"/>
+      <x:c r="T21" s="39" t="str">
+        <x:v>4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
+      </x:c>
+      <x:c r="U21" s="39" t="str">
+        <x:v>2026-06-30T11:06:18Z</x:v>
+      </x:c>
+      <x:c r="V21" s="39" t="str">
+        <x:v>2026-06-30T11:06:18Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39" t="str">
+        <x:v>2026-07-01T11:06:18Z</x:v>
+      </x:c>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Migrated from GitHub issue #669; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>
       <x:c r="AC21" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="72" customHeight="1">

</xml_diff>

<commit_message>
[queue] Claim [EPIC_02][STORY_01][SUBSTORY_02] #669 Harden CI validation authority for workflow changes (#927)
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-5, claim 4d74f425-a323-41d6-931b-13cf0d913a14, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5671,25 +5671,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R21" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R21" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
+      </x:c>
       <x:c r="S21" s="39"/>
-      <x:c r="T21" s="39"/>
-      <x:c r="U21" s="39"/>
-      <x:c r="V21" s="39"/>
-      <x:c r="W21" s="39"/>
+      <x:c r="T21" s="39" t="str">
+        <x:v>4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
+      </x:c>
+      <x:c r="U21" s="39" t="str">
+        <x:v>2026-06-30T11:06:18Z</x:v>
+      </x:c>
+      <x:c r="V21" s="39" t="str">
+        <x:v>2026-06-30T11:06:18Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39" t="str">
+        <x:v>2026-07-01T11:06:18Z</x:v>
+      </x:c>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Migrated from GitHub issue #669; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>
       <x:c r="AC21" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Heartbeat #674 and #672 (95%): impl complete, blocked on main build CI
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5929,17 +5929,17 @@
         <x:v>2026-06-30T10:25:40Z</x:v>
       </x:c>
       <x:c r="V24" s="36" t="str">
-        <x:v>2026-06-30T10:25:40Z</x:v>
+        <x:v>2026-06-30T11:42:03Z</x:v>
       </x:c>
       <x:c r="W24" s="36" t="str">
-        <x:v>2026-07-01T10:25:40Z</x:v>
+        <x:v>2026-07-01T11:42:03Z</x:v>
       </x:c>
       <x:c r="X24" s="36"/>
       <x:c r="Y24" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="Z24" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
+        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
       </x:c>
       <x:c r="AA24" s="36"/>
       <x:c r="AB24" s="36"/>
@@ -6094,17 +6094,17 @@
         <x:v>2026-06-30T10:20:13Z</x:v>
       </x:c>
       <x:c r="V26" s="36" t="str">
-        <x:v>2026-06-30T10:20:13Z</x:v>
+        <x:v>2026-06-30T11:42:03Z</x:v>
       </x:c>
       <x:c r="W26" s="36" t="str">
-        <x:v>2026-07-01T10:20:13Z</x:v>
+        <x:v>2026-07-01T11:42:03Z</x:v>
       </x:c>
       <x:c r="X26" s="36"/>
       <x:c r="Y26" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="Z26" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
+        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
       </x:c>
       <x:c r="AA26" s="36"/>
       <x:c r="AB26" s="36"/>

</xml_diff>

<commit_message>
Heartbeat #674 and #672 (95%): impl complete, blocked on main build CI (#940)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5929,17 +5929,17 @@
         <x:v>2026-06-30T10:25:40Z</x:v>
       </x:c>
       <x:c r="V24" s="36" t="str">
-        <x:v>2026-06-30T10:25:40Z</x:v>
+        <x:v>2026-06-30T11:42:03Z</x:v>
       </x:c>
       <x:c r="W24" s="36" t="str">
-        <x:v>2026-07-01T10:25:40Z</x:v>
+        <x:v>2026-07-01T11:42:03Z</x:v>
       </x:c>
       <x:c r="X24" s="36"/>
       <x:c r="Y24" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="Z24" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
+        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
       </x:c>
       <x:c r="AA24" s="36"/>
       <x:c r="AB24" s="36"/>
@@ -6094,17 +6094,17 @@
         <x:v>2026-06-30T10:20:13Z</x:v>
       </x:c>
       <x:c r="V26" s="36" t="str">
-        <x:v>2026-06-30T10:20:13Z</x:v>
+        <x:v>2026-06-30T11:42:03Z</x:v>
       </x:c>
       <x:c r="W26" s="36" t="str">
-        <x:v>2026-07-01T10:20:13Z</x:v>
+        <x:v>2026-07-01T11:42:03Z</x:v>
       </x:c>
       <x:c r="X26" s="36"/>
       <x:c r="Y26" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="Z26" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
+        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
       </x:c>
       <x:c r="AA26" s="36"/>
       <x:c r="AB26" s="36"/>

</xml_diff>

<commit_message>
Heartbeat migrated-workbook claim #677 (impl complete, awaiting PR #945 unblock)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6364,17 +6364,17 @@
         <x:v>2026-06-30T10:56:52Z</x:v>
       </x:c>
       <x:c r="V29" s="39" t="str">
-        <x:v>2026-06-30T10:56:52Z</x:v>
+        <x:v>2026-06-30T12:06:49Z</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>2026-07-01T10:56:52Z</x:v>
+        <x:v>2026-07-01T12:06:49Z</x:v>
       </x:c>
       <x:c r="X29" s="39"/>
       <x:c r="Y29" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z29" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-3</x:v>
+        <x:v>Implementation complete and PR open (#926); awaiting main-build unblock via PR #945 (scene-manager source-map leak fix).</x:v>
       </x:c>
       <x:c r="AA29" s="39"/>
       <x:c r="AB29" s="39"/>

</xml_diff>

<commit_message>
Heartbeat migrated-workbook claim #677 (impl complete, awaiting PR #945 unblock) (#949)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6364,17 +6364,17 @@
         <x:v>2026-06-30T10:56:52Z</x:v>
       </x:c>
       <x:c r="V29" s="39" t="str">
-        <x:v>2026-06-30T10:56:52Z</x:v>
+        <x:v>2026-06-30T12:06:49Z</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>2026-07-01T10:56:52Z</x:v>
+        <x:v>2026-07-01T12:06:49Z</x:v>
       </x:c>
       <x:c r="X29" s="39"/>
       <x:c r="Y29" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z29" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-3</x:v>
+        <x:v>Implementation complete and PR open (#926); awaiting main-build unblock via PR #945 (scene-manager source-map leak fix).</x:v>
       </x:c>
       <x:c r="AA29" s="39"/>
       <x:c r="AB29" s="39"/>

</xml_diff>

<commit_message>
[queue] Heartbeat #675 and #669 (impl complete, blocked on main-red CI)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5684,17 +5684,17 @@
         <x:v>2026-06-30T11:06:18Z</x:v>
       </x:c>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-06-30T11:06:18Z</x:v>
+        <x:v>2026-06-30T12:22:37Z</x:v>
       </x:c>
       <x:c r="W21" s="39" t="str">
-        <x:v>2026-07-01T11:06:18Z</x:v>
+        <x:v>2026-07-01T12:22:37Z</x:v>
       </x:c>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
+        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim. awaiting user review of authority-machinery PR #934.</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>
@@ -6183,17 +6183,17 @@
         <x:v>2026-06-30T10:50:10Z</x:v>
       </x:c>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T10:50:10Z</x:v>
+        <x:v>2026-06-30T12:22:37Z</x:v>
       </x:c>
       <x:c r="W27" s="39" t="str">
-        <x:v>2026-07-01T10:50:10Z</x:v>
+        <x:v>2026-07-01T12:22:37Z</x:v>
       </x:c>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim.</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>

</xml_diff>

<commit_message>
[queue] Heartbeat #675 and #669 (impl complete, blocked on main-red CI) (#950)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5684,17 +5684,17 @@
         <x:v>2026-06-30T11:06:18Z</x:v>
       </x:c>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-06-30T11:06:18Z</x:v>
+        <x:v>2026-06-30T12:22:37Z</x:v>
       </x:c>
       <x:c r="W21" s="39" t="str">
-        <x:v>2026-07-01T11:06:18Z</x:v>
+        <x:v>2026-07-01T12:22:37Z</x:v>
       </x:c>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
+        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim. awaiting user review of authority-machinery PR #934.</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>
@@ -6183,17 +6183,17 @@
         <x:v>2026-06-30T10:50:10Z</x:v>
       </x:c>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T10:50:10Z</x:v>
+        <x:v>2026-06-30T12:22:37Z</x:v>
       </x:c>
       <x:c r="W27" s="39" t="str">
-        <x:v>2026-07-01T10:50:10Z</x:v>
+        <x:v>2026-07-01T12:22:37Z</x:v>
       </x:c>
       <x:c r="X27" s="39"/>
       <x:c r="Y27" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
+        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim.</x:v>
       </x:c>
       <x:c r="AA27" s="39"/>
       <x:c r="AB27" s="39"/>

</xml_diff>

<commit_message>
[queue] Complete [EPIC_05][STORY_02][SUBSTORY_02] #675 Restrict MCP controller and pathfinding resource consumption
Implementation merged via PR #923.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6170,7 +6170,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R27" s="39" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
@@ -6183,20 +6183,24 @@
         <x:v>2026-06-30T10:50:10Z</x:v>
       </x:c>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T12:22:37Z</x:v>
-      </x:c>
-      <x:c r="W27" s="39" t="str">
-        <x:v>2026-07-01T12:22:37Z</x:v>
-      </x:c>
-      <x:c r="X27" s="39"/>
+        <x:v>2026-06-30T12:50:27Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39"/>
+      <x:c r="X27" s="39" t="str">
+        <x:v>2026-06-30T12:50:27Z</x:v>
+      </x:c>
       <x:c r="Y27" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim.</x:v>
-      </x:c>
-      <x:c r="AA27" s="39"/>
-      <x:c r="AB27" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA27" s="39" t="str">
+        <x:v>Restricted MCP pathfinding resource consumption: mcp.py validates setTarget args (rejects extreme-magnitude/out-of-bounds/non-passable targets); CController::setTarget rejects out-of-map-extent targets before pathfinding; CMap gained public isWithinBounds; CPathFinder added a goal-relative coordinate-envelope budget (4*manhattan+512, sized so wrapping maps are not over-pruned) and a max path-length guard alongside the existing 1M-node cap. MCP runtime tests + native pathfinder envelope tests added.</x:v>
+      </x:c>
+      <x:c r="AB27" s="39" t="str">
+        <x:v>GitHub Actions on PR #923 (final run on unblocked main): linux SUCCESS, windows SUCCESS, windows-deps/linux-fast/validate SUCCESS. Native pathfinder tests + full Python suite (incl. MCP guard tests and the previously-regressed change-map test) passed. Merged to main as 8fa0ef96.</x:v>
+      </x:c>
       <x:c r="AC27" s="39" t="n">
         <x:v>2</x:v>
       </x:c>

</xml_diff>

<commit_message>
[queue] Complete [EPIC_05][STORY_02][SUBSTORY_02] #675 Restrict MCP controller and pathfinding resource consumption (#957)
Implementation merged via PR #923.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6170,7 +6170,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/core/CPathFinder.cpp</x:v>
       </x:c>
       <x:c r="Q27" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R27" s="39" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-1</x:v>
@@ -6183,20 +6183,24 @@
         <x:v>2026-06-30T10:50:10Z</x:v>
       </x:c>
       <x:c r="V27" s="39" t="str">
-        <x:v>2026-06-30T12:22:37Z</x:v>
-      </x:c>
-      <x:c r="W27" s="39" t="str">
-        <x:v>2026-07-01T12:22:37Z</x:v>
-      </x:c>
-      <x:c r="X27" s="39"/>
+        <x:v>2026-06-30T12:50:27Z</x:v>
+      </x:c>
+      <x:c r="W27" s="39"/>
+      <x:c r="X27" s="39" t="str">
+        <x:v>2026-06-30T12:50:27Z</x:v>
+      </x:c>
       <x:c r="Y27" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z27" s="39" t="str">
-        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim.</x:v>
-      </x:c>
-      <x:c r="AA27" s="39"/>
-      <x:c r="AB27" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA27" s="39" t="str">
+        <x:v>Restricted MCP pathfinding resource consumption: mcp.py validates setTarget args (rejects extreme-magnitude/out-of-bounds/non-passable targets); CController::setTarget rejects out-of-map-extent targets before pathfinding; CMap gained public isWithinBounds; CPathFinder added a goal-relative coordinate-envelope budget (4*manhattan+512, sized so wrapping maps are not over-pruned) and a max path-length guard alongside the existing 1M-node cap. MCP runtime tests + native pathfinder envelope tests added.</x:v>
+      </x:c>
+      <x:c r="AB27" s="39" t="str">
+        <x:v>GitHub Actions on PR #923 (final run on unblocked main): linux SUCCESS, windows SUCCESS, windows-deps/linux-fast/validate SUCCESS. Native pathfinder tests + full Python suite (incl. MCP guard tests and the previously-regressed change-map test) passed. Merged to main as 8fa0ef96.</x:v>
+      </x:c>
       <x:c r="AC27" s="39" t="n">
         <x:v>2</x:v>
       </x:c>

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_01][SUBSTORY_03] #678 Make config-driven reflective callbacks fail closed
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-10, claim 78738aaf-943f-42cc-b6d3-5620e1fbf8c4, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6442,25 +6442,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q30" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R30" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R30" s="36" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
+      </x:c>
       <x:c r="S30" s="36"/>
-      <x:c r="T30" s="36"/>
-      <x:c r="U30" s="36"/>
-      <x:c r="V30" s="36"/>
-      <x:c r="W30" s="36"/>
+      <x:c r="T30" s="36" t="str">
+        <x:v>78738aaf-943f-42cc-b6d3-5620e1fbf8c4</x:v>
+      </x:c>
+      <x:c r="U30" s="36" t="str">
+        <x:v>2026-06-30T13:04:28Z</x:v>
+      </x:c>
+      <x:c r="V30" s="36" t="str">
+        <x:v>2026-06-30T13:04:28Z</x:v>
+      </x:c>
+      <x:c r="W30" s="36" t="str">
+        <x:v>2026-07-01T13:04:28Z</x:v>
+      </x:c>
       <x:c r="X30" s="36"/>
       <x:c r="Y30" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z30" s="36" t="str">
-        <x:v>Migrated from GitHub issue #678; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
       </x:c>
       <x:c r="AA30" s="36"/>
       <x:c r="AB30" s="36"/>
       <x:c r="AC30" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_01][SUBSTORY_03] #678 Make config-driven reflective callbacks fail closed (#965)
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-10, claim 78738aaf-943f-42cc-b6d3-5620e1fbf8c4, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6442,25 +6442,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q30" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R30" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R30" s="36" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
+      </x:c>
       <x:c r="S30" s="36"/>
-      <x:c r="T30" s="36"/>
-      <x:c r="U30" s="36"/>
-      <x:c r="V30" s="36"/>
-      <x:c r="W30" s="36"/>
+      <x:c r="T30" s="36" t="str">
+        <x:v>78738aaf-943f-42cc-b6d3-5620e1fbf8c4</x:v>
+      </x:c>
+      <x:c r="U30" s="36" t="str">
+        <x:v>2026-06-30T13:04:28Z</x:v>
+      </x:c>
+      <x:c r="V30" s="36" t="str">
+        <x:v>2026-06-30T13:04:28Z</x:v>
+      </x:c>
+      <x:c r="W30" s="36" t="str">
+        <x:v>2026-07-01T13:04:28Z</x:v>
+      </x:c>
       <x:c r="X30" s="36"/>
       <x:c r="Y30" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z30" s="36" t="str">
-        <x:v>Migrated from GitHub issue #678; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
       </x:c>
       <x:c r="AA30" s="36"/>
       <x:c r="AB30" s="36"/>
       <x:c r="AC30" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Heartbeat migrated claim #677 (rebased PR #926 re-running on green main)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6368,17 +6368,17 @@
         <x:v>2026-06-30T10:56:52Z</x:v>
       </x:c>
       <x:c r="V29" s="39" t="str">
-        <x:v>2026-06-30T12:06:49Z</x:v>
+        <x:v>2026-06-30T13:14:23Z</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>2026-07-01T12:06:49Z</x:v>
+        <x:v>2026-07-01T13:14:23Z</x:v>
       </x:c>
       <x:c r="X29" s="39"/>
       <x:c r="Y29" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="Z29" s="39" t="str">
-        <x:v>Implementation complete and PR open (#926); awaiting main-build unblock via PR #945 (scene-manager source-map leak fix).</x:v>
+        <x:v>Impl complete; rebased PR #926 re-running on green main (unblocked by #945). Prior CI run stalled in congested queue; re-triggered.</x:v>
       </x:c>
       <x:c r="AA29" s="39"/>
       <x:c r="AB29" s="39"/>

</xml_diff>

<commit_message>
Heartbeat migrated claim #677 (rebased PR #926 re-running on green main) (#969)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6368,17 +6368,17 @@
         <x:v>2026-06-30T10:56:52Z</x:v>
       </x:c>
       <x:c r="V29" s="39" t="str">
-        <x:v>2026-06-30T12:06:49Z</x:v>
+        <x:v>2026-06-30T13:14:23Z</x:v>
       </x:c>
       <x:c r="W29" s="39" t="str">
-        <x:v>2026-07-01T12:06:49Z</x:v>
+        <x:v>2026-07-01T13:14:23Z</x:v>
       </x:c>
       <x:c r="X29" s="39"/>
       <x:c r="Y29" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="Z29" s="39" t="str">
-        <x:v>Implementation complete and PR open (#926); awaiting main-build unblock via PR #945 (scene-manager source-map leak fix).</x:v>
+        <x:v>Impl complete; rebased PR #926 re-running on green main (unblocked by #945). Prior CI run stalled in congested queue; re-triggered.</x:v>
       </x:c>
       <x:c r="AA29" s="39"/>
       <x:c r="AB29" s="39"/>

</xml_diff>

<commit_message>
Complete e05-s03-ss02 #677 Bound minimap work (impl PR #926)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6355,7 +6355,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/config/graphics.json</x:v>
       </x:c>
       <x:c r="Q29" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R29" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-3</x:v>
@@ -6368,20 +6368,24 @@
         <x:v>2026-06-30T10:56:52Z</x:v>
       </x:c>
       <x:c r="V29" s="39" t="str">
-        <x:v>2026-06-30T13:14:23Z</x:v>
-      </x:c>
-      <x:c r="W29" s="39" t="str">
-        <x:v>2026-07-01T13:14:23Z</x:v>
-      </x:c>
-      <x:c r="X29" s="39"/>
+        <x:v>2026-06-30T14:00:48Z</x:v>
+      </x:c>
+      <x:c r="W29" s="39"/>
+      <x:c r="X29" s="39" t="str">
+        <x:v>2026-06-30T14:00:48Z</x:v>
+      </x:c>
       <x:c r="Y29" s="39" t="n">
-        <x:v>92</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z29" s="39" t="str">
-        <x:v>Impl complete; rebased PR #926 re-running on green main (unblocked by #945). Prior CI run stalled in congested queue; re-triggered.</x:v>
-      </x:c>
-      <x:c r="AA29" s="39"/>
-      <x:c r="AB29" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA29" s="39" t="str">
+        <x:v>Bounded minimap rendering against malformed/extreme map extents. Clamped attacker-authorable xBound/yBound level metadata in CLoader; added MAX_MINIMAP_LEVEL_EXTENT with overflow-safe (long long) bounds checks in CMinimapGraphicsObject (get_level_bounds fails closed to a bounded placeholder; make_scale overflow-safe). Added 5 GUI regression tests (extreme/overflow/sparse/negative-origin/normal). No save/map format change; legitimate maps render unchanged.</x:v>
+      </x:c>
+      <x:c r="AB29" s="39" t="str">
+        <x:v>CI: GitHub Actions build run #2101 (head 75ee6700) on green main -&gt; all 5 jobs success (linux-fast, windows-deps, linux, windows, linux-coverage incl. test (c++)+test (python gameplay)+coverage). Implementation PR #926 merged to main (squash 366edbce). clang-format + git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC29" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete e05-s03-ss02 #677 Bound minimap work (impl PR #926) (#976)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6355,7 +6355,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/config/graphics.json</x:v>
       </x:c>
       <x:c r="Q29" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R29" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-3</x:v>
@@ -6368,20 +6368,24 @@
         <x:v>2026-06-30T10:56:52Z</x:v>
       </x:c>
       <x:c r="V29" s="39" t="str">
-        <x:v>2026-06-30T13:14:23Z</x:v>
-      </x:c>
-      <x:c r="W29" s="39" t="str">
-        <x:v>2026-07-01T13:14:23Z</x:v>
-      </x:c>
-      <x:c r="X29" s="39"/>
+        <x:v>2026-06-30T14:00:48Z</x:v>
+      </x:c>
+      <x:c r="W29" s="39"/>
+      <x:c r="X29" s="39" t="str">
+        <x:v>2026-06-30T14:00:48Z</x:v>
+      </x:c>
       <x:c r="Y29" s="39" t="n">
-        <x:v>92</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z29" s="39" t="str">
-        <x:v>Impl complete; rebased PR #926 re-running on green main (unblocked by #945). Prior CI run stalled in congested queue; re-triggered.</x:v>
-      </x:c>
-      <x:c r="AA29" s="39"/>
-      <x:c r="AB29" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA29" s="39" t="str">
+        <x:v>Bounded minimap rendering against malformed/extreme map extents. Clamped attacker-authorable xBound/yBound level metadata in CLoader; added MAX_MINIMAP_LEVEL_EXTENT with overflow-safe (long long) bounds checks in CMinimapGraphicsObject (get_level_bounds fails closed to a bounded placeholder; make_scale overflow-safe). Added 5 GUI regression tests (extreme/overflow/sparse/negative-origin/normal). No save/map format change; legitimate maps render unchanged.</x:v>
+      </x:c>
+      <x:c r="AB29" s="39" t="str">
+        <x:v>CI: GitHub Actions build run #2101 (head 75ee6700) on green main -&gt; all 5 jobs success (linux-fast, windows-deps, linux, windows, linux-coverage incl. test (c++)+test (python gameplay)+coverage). Implementation PR #926 merged to main (squash 366edbce). clang-format + git diff --check clean.</x:v>
+      </x:c>
       <x:c r="AC29" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
[queue] Complete [EPIC_05][STORY_01][SUBSTORY_03] #678 Make config-driven reflective callbacks fail closed
Implementation merged via PR #974.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6446,7 +6446,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q30" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R30" s="36" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
@@ -6459,20 +6459,24 @@
         <x:v>2026-06-30T13:04:28Z</x:v>
       </x:c>
       <x:c r="V30" s="36" t="str">
-        <x:v>2026-06-30T13:04:28Z</x:v>
-      </x:c>
-      <x:c r="W30" s="36" t="str">
-        <x:v>2026-07-01T13:04:28Z</x:v>
-      </x:c>
-      <x:c r="X30" s="36"/>
+        <x:v>2026-06-30T14:01:45Z</x:v>
+      </x:c>
+      <x:c r="W30" s="36"/>
+      <x:c r="X30" s="36" t="str">
+        <x:v>2026-06-30T14:01:45Z</x:v>
+      </x:c>
       <x:c r="Y30" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z30" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
-      </x:c>
-      <x:c r="AA30" s="36"/>
-      <x:c r="AB30" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA30" s="36" t="str">
+        <x:v>Made config-driven reflective callbacks fail closed, mirroring res/game.py's public-callback contract. Audited all reflective dispatch points; the two unguarded ones (CGameCharacterPanel char-sheet accessor, CGameObject signal-&gt;slot dispatch) now empty-guard + try/catch + log (actions no-op, conditions return false), so a bad/throwing callback cannot crash the render or event loop. Extended validate_content.py to flag empty/non-identifier/private/dunder/invokeAction/invokeCondition dialog method names. Native gui+signal-slot regressions and 5 validator tests added.</x:v>
+      </x:c>
+      <x:c r="AB30" s="36" t="str">
+        <x:v>GitHub Actions on PR #974 (green main): linux SUCCESS, windows SUCCESS, windows-deps/linux-fast/validate SUCCESS. tests.test_content_validator 49 passed; native gui_unit_tests/object_unit_tests + full suite passed. Merged to main as c433d1c9.</x:v>
+      </x:c>
       <x:c r="AC30" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
[queue] Complete [EPIC_05][STORY_01][SUBSTORY_03] #678 Make config-driven reflective callbacks fail closed (#977)
Implementation merged via PR #974.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6446,7 +6446,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q30" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R30" s="36" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
@@ -6459,20 +6459,24 @@
         <x:v>2026-06-30T13:04:28Z</x:v>
       </x:c>
       <x:c r="V30" s="36" t="str">
-        <x:v>2026-06-30T13:04:28Z</x:v>
-      </x:c>
-      <x:c r="W30" s="36" t="str">
-        <x:v>2026-07-01T13:04:28Z</x:v>
-      </x:c>
-      <x:c r="X30" s="36"/>
+        <x:v>2026-06-30T14:01:45Z</x:v>
+      </x:c>
+      <x:c r="W30" s="36"/>
+      <x:c r="X30" s="36" t="str">
+        <x:v>2026-06-30T14:01:45Z</x:v>
+      </x:c>
       <x:c r="Y30" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z30" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-10</x:v>
-      </x:c>
-      <x:c r="AA30" s="36"/>
-      <x:c r="AB30" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA30" s="36" t="str">
+        <x:v>Made config-driven reflective callbacks fail closed, mirroring res/game.py's public-callback contract. Audited all reflective dispatch points; the two unguarded ones (CGameCharacterPanel char-sheet accessor, CGameObject signal-&gt;slot dispatch) now empty-guard + try/catch + log (actions no-op, conditions return false), so a bad/throwing callback cannot crash the render or event loop. Extended validate_content.py to flag empty/non-identifier/private/dunder/invokeAction/invokeCondition dialog method names. Native gui+signal-slot regressions and 5 validator tests added.</x:v>
+      </x:c>
+      <x:c r="AB30" s="36" t="str">
+        <x:v>GitHub Actions on PR #974 (green main): linux SUCCESS, windows SUCCESS, windows-deps/linux-fast/validate SUCCESS. tests.test_content_validator 49 passed; native gui_unit_tests/object_unit_tests + full suite passed. Merged to main as c433d1c9.</x:v>
+      </x:c>
       <x:c r="AC30" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_01][SUBSTORY_02] #671 Separate dynamic property notifications from typed engine signals
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-11, claim 2829d4f9-adf5-4bcf-9a66-839425db0dc8, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5839,25 +5839,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/object/CGameObject.cpp</x:v>
       </x:c>
       <x:c r="Q23" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R23" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R23" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
+      </x:c>
       <x:c r="S23" s="39"/>
-      <x:c r="T23" s="39"/>
-      <x:c r="U23" s="39"/>
-      <x:c r="V23" s="39"/>
-      <x:c r="W23" s="39"/>
+      <x:c r="T23" s="39" t="str">
+        <x:v>2829d4f9-adf5-4bcf-9a66-839425db0dc8</x:v>
+      </x:c>
+      <x:c r="U23" s="39" t="str">
+        <x:v>2026-06-30T14:03:01Z</x:v>
+      </x:c>
+      <x:c r="V23" s="39" t="str">
+        <x:v>2026-06-30T14:03:01Z</x:v>
+      </x:c>
+      <x:c r="W23" s="39" t="str">
+        <x:v>2026-07-01T14:03:01Z</x:v>
+      </x:c>
       <x:c r="X23" s="39"/>
       <x:c r="Y23" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z23" s="39" t="str">
-        <x:v>Migrated from GitHub issue #671; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
       </x:c>
       <x:c r="AA23" s="39"/>
       <x:c r="AB23" s="39"/>
       <x:c r="AC23" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="72" customHeight="1">

</xml_diff>

<commit_message>
[queue] Claim [EPIC_05][STORY_01][SUBSTORY_02] #671 Separate dynamic property notifications from typed engine signals (#978)
Owner controller/ctrl-vm-4026-9b5a29b5/subagent-11, claim 2829d4f9-adf5-4bcf-9a66-839425db0dc8, lease 1440m. Queue state only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5839,25 +5839,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/object/CGameObject.cpp</x:v>
       </x:c>
       <x:c r="Q23" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R23" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R23" s="39" t="str">
+        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
+      </x:c>
       <x:c r="S23" s="39"/>
-      <x:c r="T23" s="39"/>
-      <x:c r="U23" s="39"/>
-      <x:c r="V23" s="39"/>
-      <x:c r="W23" s="39"/>
+      <x:c r="T23" s="39" t="str">
+        <x:v>2829d4f9-adf5-4bcf-9a66-839425db0dc8</x:v>
+      </x:c>
+      <x:c r="U23" s="39" t="str">
+        <x:v>2026-06-30T14:03:01Z</x:v>
+      </x:c>
+      <x:c r="V23" s="39" t="str">
+        <x:v>2026-06-30T14:03:01Z</x:v>
+      </x:c>
+      <x:c r="W23" s="39" t="str">
+        <x:v>2026-07-01T14:03:01Z</x:v>
+      </x:c>
       <x:c r="X23" s="39"/>
       <x:c r="Y23" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z23" s="39" t="str">
-        <x:v>Migrated from GitHub issue #671; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
       </x:c>
       <x:c r="AA23" s="39"/>
       <x:c r="AB23" s="39"/>
       <x:c r="AC23" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Queue: complete EPIC_05/STORY_01/SUBSTORY_02 #671 separate dynamic property signals (#987)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5839,7 +5839,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/object/CGameObject.cpp</x:v>
       </x:c>
       <x:c r="Q23" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R23" s="39" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
@@ -5852,20 +5852,24 @@
         <x:v>2026-06-30T14:03:01Z</x:v>
       </x:c>
       <x:c r="V23" s="39" t="str">
-        <x:v>2026-06-30T14:03:01Z</x:v>
-      </x:c>
-      <x:c r="W23" s="39" t="str">
-        <x:v>2026-07-01T14:03:01Z</x:v>
-      </x:c>
-      <x:c r="X23" s="39"/>
+        <x:v>2026-06-30T14:42:22Z</x:v>
+      </x:c>
+      <x:c r="W23" s="39"/>
+      <x:c r="X23" s="39" t="str">
+        <x:v>2026-06-30T14:42:22Z</x:v>
+      </x:c>
       <x:c r="Y23" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z23" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
-      </x:c>
-      <x:c r="AA23" s="39"/>
-      <x:c r="AB23" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA23" s="39" t="str">
+        <x:v>Merged PR #987 (923f1f52): dynamic property notifications can no longer spoof typed engine signals. Added CGameObject::isReservedTypedSignalName registry; notifyPropertyChangedWithoutInvalidation drops+logs per-property &lt;name&gt;Changed emissions that collide with reserved typed names; CListView skips+logs colliding refreshProperties names. Native linux+windows green.</x:v>
+      </x:c>
+      <x:c r="AB23" s="39" t="str">
+        <x:v>linux+windows native CI green on PR #987; test_object.cpp + test_gui.cpp regressions: dynamic property cannot spoof typed signal, typed signal still fires, refreshProperty collision fails closed while valid property refreshes.</x:v>
+      </x:c>
       <x:c r="AC23" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Queue: complete EPIC_05/STORY_01/SUBSTORY_02 #671 separate dynamic property signals (#987) (#997)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5839,7 +5839,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/object/CGameObject.cpp</x:v>
       </x:c>
       <x:c r="Q23" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R23" s="39" t="str">
         <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
@@ -5852,20 +5852,24 @@
         <x:v>2026-06-30T14:03:01Z</x:v>
       </x:c>
       <x:c r="V23" s="39" t="str">
-        <x:v>2026-06-30T14:03:01Z</x:v>
-      </x:c>
-      <x:c r="W23" s="39" t="str">
-        <x:v>2026-07-01T14:03:01Z</x:v>
-      </x:c>
-      <x:c r="X23" s="39"/>
+        <x:v>2026-06-30T14:42:22Z</x:v>
+      </x:c>
+      <x:c r="W23" s="39"/>
+      <x:c r="X23" s="39" t="str">
+        <x:v>2026-06-30T14:42:22Z</x:v>
+      </x:c>
       <x:c r="Y23" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z23" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4026-9b5a29b5/subagent-11</x:v>
-      </x:c>
-      <x:c r="AA23" s="39"/>
-      <x:c r="AB23" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA23" s="39" t="str">
+        <x:v>Merged PR #987 (923f1f52): dynamic property notifications can no longer spoof typed engine signals. Added CGameObject::isReservedTypedSignalName registry; notifyPropertyChangedWithoutInvalidation drops+logs per-property &lt;name&gt;Changed emissions that collide with reserved typed names; CListView skips+logs colliding refreshProperties names. Native linux+windows green.</x:v>
+      </x:c>
+      <x:c r="AB23" s="39" t="str">
+        <x:v>linux+windows native CI green on PR #987; test_object.cpp + test_gui.cpp regressions: dynamic property cannot spoof typed signal, typed signal still fires, refreshProperty collision fails closed while valid property refreshes.</x:v>
+      </x:c>
       <x:c r="AC23" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_05/STORY_03/SUBSTORY_01 #674 bound saved-quest traversal (impl PR #898)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6095,7 +6095,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/save format/schema helpers</x:v>
       </x:c>
       <x:c r="Q26" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R26" s="36" t="str">
         <x:v>controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
@@ -6108,20 +6108,24 @@
         <x:v>2026-06-30T10:20:13Z</x:v>
       </x:c>
       <x:c r="V26" s="36" t="str">
-        <x:v>2026-06-30T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="W26" s="36" t="str">
-        <x:v>2026-07-01T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="X26" s="36"/>
+        <x:v>2026-06-30T19:58:43Z</x:v>
+      </x:c>
+      <x:c r="W26" s="36"/>
+      <x:c r="X26" s="36" t="str">
+        <x:v>2026-06-30T19:58:43Z</x:v>
+      </x:c>
       <x:c r="Y26" s="36" t="n">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z26" s="36" t="str">
-        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
-      </x:c>
-      <x:c r="AA26" s="36"/>
-      <x:c r="AB26" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA26" s="36" t="str">
+        <x:v>Bounded saved-quest reference traversal during load to prevent stack exhaustion / CPU DoS from crafted save JSON. Added iterative, bounded structure validation in CSaveFormat (MAX_DOCUMENT_DEPTH=200, MAX_DOCUMENT_NODES=8M, MAX_CONTAINER_ENTRIES=1M) invoked at the top of decodeDocument, and rewrote collect_saved_quest_refs in CLoader as an iterative work-stack with a node ceiling. Reuses the existing std::expected loader-error path; rejects oversized/over-deep saves with a clear reason while loading legitimate saves unchanged (real fixtures max depth 9). Added native (test_core.cpp) and Python (test.py) regressions for boundary, oversize, repeated-ref, and normal round-trip cases. The detachPlayer API is unrelated/untouched.</x:v>
+      </x:c>
+      <x:c r="AB26" s="36" t="str">
+        <x:v>CI (PR #898 on green main) check runs: linux=success, windows=success, windows-deps=success, linux-coverage=success, linux-fast=success, validate=success, export=success. Full native build + ctest + python suite + coverage all passed. Implementation PR #898 merged to main as 2646b8946c7fbd5c95619df0f29fa3543ef4d1fc.</x:v>
+      </x:c>
       <x:c r="AC26" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_05/STORY_03/SUBSTORY_01 #674 bound saved-quest traversal (impl PR #898) (#1052)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6095,7 +6095,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/save format/schema helpers</x:v>
       </x:c>
       <x:c r="Q26" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R26" s="36" t="str">
         <x:v>controller/ctrl-vm-4024-7534d796/subagent-2</x:v>
@@ -6108,20 +6108,24 @@
         <x:v>2026-06-30T10:20:13Z</x:v>
       </x:c>
       <x:c r="V26" s="36" t="str">
-        <x:v>2026-06-30T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="W26" s="36" t="str">
-        <x:v>2026-07-01T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="X26" s="36"/>
+        <x:v>2026-06-30T19:58:43Z</x:v>
+      </x:c>
+      <x:c r="W26" s="36"/>
+      <x:c r="X26" s="36" t="str">
+        <x:v>2026-06-30T19:58:43Z</x:v>
+      </x:c>
       <x:c r="Y26" s="36" t="n">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z26" s="36" t="str">
-        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
-      </x:c>
-      <x:c r="AA26" s="36"/>
-      <x:c r="AB26" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA26" s="36" t="str">
+        <x:v>Bounded saved-quest reference traversal during load to prevent stack exhaustion / CPU DoS from crafted save JSON. Added iterative, bounded structure validation in CSaveFormat (MAX_DOCUMENT_DEPTH=200, MAX_DOCUMENT_NODES=8M, MAX_CONTAINER_ENTRIES=1M) invoked at the top of decodeDocument, and rewrote collect_saved_quest_refs in CLoader as an iterative work-stack with a node ceiling. Reuses the existing std::expected loader-error path; rejects oversized/over-deep saves with a clear reason while loading legitimate saves unchanged (real fixtures max depth 9). Added native (test_core.cpp) and Python (test.py) regressions for boundary, oversize, repeated-ref, and normal round-trip cases. The detachPlayer API is unrelated/untouched.</x:v>
+      </x:c>
+      <x:c r="AB26" s="36" t="str">
+        <x:v>CI (PR #898 on green main) check runs: linux=success, windows=success, windows-deps=success, linux-coverage=success, linux-fast=success, validate=success, export=success. Full native build + ctest + python suite + coverage all passed. Implementation PR #898 merged to main as 2646b8946c7fbd5c95619df0f29fa3543ef4d1fc.</x:v>
+      </x:c>
       <x:c r="AC26" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_05/STORY_02/SUBSTORY_01 #672 MCP per-action limits (impl PR #899)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5930,7 +5930,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/game_simulation.py</x:v>
       </x:c>
       <x:c r="Q24" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R24" s="36" t="str">
         <x:v>controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
@@ -5943,20 +5943,24 @@
         <x:v>2026-06-30T10:25:40Z</x:v>
       </x:c>
       <x:c r="V24" s="36" t="str">
-        <x:v>2026-06-30T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="W24" s="36" t="str">
-        <x:v>2026-07-01T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="X24" s="36"/>
+        <x:v>2026-06-30T19:59:34Z</x:v>
+      </x:c>
+      <x:c r="W24" s="36"/>
+      <x:c r="X24" s="36" t="str">
+        <x:v>2026-06-30T19:59:34Z</x:v>
+      </x:c>
       <x:c r="Y24" s="36" t="n">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z24" s="36" t="str">
-        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
-      </x:c>
-      <x:c r="AA24" s="36"/>
-      <x:c r="AB24" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA24" s="36" t="str">
+        <x:v>Enforced per-action iteration limits in MCP simulation_run to prevent a single step (extreme turns/times/max_iterations/max_turns) from bypassing the step cap and causing CPU-heavy loops. Added a shared per-action limits block plus validateSteps() and a cumulative iteration budget in game_simulation.py, validating all attacker-controlled counts before any loop runs and rejecting non-integer/negative/above-limit values with a structured SimulationError identifying the offending action index and field. Wired validateSteps into runSteps/runSimulation and gated mcp._simulation_run on it so over-budget payloads do no engine work; repeated/nested actions add to one running budget and cannot multiply it. Added 22 engine-free, timeout-free regressions (spy event loop proves rejected actions run zero iterations). Backward-compatible: defaults unchanged.</x:v>
+      </x:c>
+      <x:c r="AB24" s="36" t="str">
+        <x:v>CI (PR #899 on green main) check runs: linux=success, windows=success, windows-deps=success, linux-fast=success, validate=success, export=success; linux-coverage=skipped (no coverage-trigger paths). Implementation PR #899 merged to main as b122be562dc4636bdb5403f34aa988ab91407e2b. Worker-run focused tests: tests.security.test_simulation_action_limits 22 passed; tests.security.test_mcp_hardening 4 passed.</x:v>
+      </x:c>
       <x:c r="AC24" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_05/STORY_02/SUBSTORY_01 #672 MCP per-action limits (impl PR #899) (#1053)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5930,7 +5930,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/game_simulation.py</x:v>
       </x:c>
       <x:c r="Q24" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R24" s="36" t="str">
         <x:v>controller/ctrl-vm-4024-7534d796/subagent-4</x:v>
@@ -5943,20 +5943,24 @@
         <x:v>2026-06-30T10:25:40Z</x:v>
       </x:c>
       <x:c r="V24" s="36" t="str">
-        <x:v>2026-06-30T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="W24" s="36" t="str">
-        <x:v>2026-07-01T11:42:03Z</x:v>
-      </x:c>
-      <x:c r="X24" s="36"/>
+        <x:v>2026-06-30T19:59:34Z</x:v>
+      </x:c>
+      <x:c r="W24" s="36"/>
+      <x:c r="X24" s="36" t="str">
+        <x:v>2026-06-30T19:59:34Z</x:v>
+      </x:c>
       <x:c r="Y24" s="36" t="n">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z24" s="36" t="str">
-        <x:v>Implementation complete and pushed (PR #898 / #899); blocked on broken main build CI (scene-manager regression test_scene_manager_transition_requested_during_combat_preserves_source_map, user-owned fix). Awaiting CI restoration to merge.</x:v>
-      </x:c>
-      <x:c r="AA24" s="36"/>
-      <x:c r="AB24" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA24" s="36" t="str">
+        <x:v>Enforced per-action iteration limits in MCP simulation_run to prevent a single step (extreme turns/times/max_iterations/max_turns) from bypassing the step cap and causing CPU-heavy loops. Added a shared per-action limits block plus validateSteps() and a cumulative iteration budget in game_simulation.py, validating all attacker-controlled counts before any loop runs and rejecting non-integer/negative/above-limit values with a structured SimulationError identifying the offending action index and field. Wired validateSteps into runSteps/runSimulation and gated mcp._simulation_run on it so over-budget payloads do no engine work; repeated/nested actions add to one running budget and cannot multiply it. Added 22 engine-free, timeout-free regressions (spy event loop proves rejected actions run zero iterations). Backward-compatible: defaults unchanged.</x:v>
+      </x:c>
+      <x:c r="AB24" s="36" t="str">
+        <x:v>CI (PR #899 on green main) check runs: linux=success, windows=success, windows-deps=success, linux-fast=success, validate=success, export=success; linux-coverage=skipped (no coverage-trigger paths). Implementation PR #899 merged to main as b122be562dc4636bdb5403f34aa988ab91407e2b. Worker-run focused tests: tests.security.test_simulation_action_limits 22 passed; tests.security.test_mcp_hardening 4 passed.</x:v>
+      </x:c>
       <x:c r="AC24" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Claim EPIC_05/STORY_01/SUBSTORY_01 #670 python plugin trust boundary
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5760,25 +5760,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q22" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R22" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R22" s="36" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
+      </x:c>
       <x:c r="S22" s="36"/>
-      <x:c r="T22" s="36"/>
-      <x:c r="U22" s="36"/>
-      <x:c r="V22" s="36"/>
-      <x:c r="W22" s="36"/>
+      <x:c r="T22" s="36" t="str">
+        <x:v>866b9190-9672-423a-84e6-7a89992a38e3</x:v>
+      </x:c>
+      <x:c r="U22" s="36" t="str">
+        <x:v>2026-06-30T20:07:26Z</x:v>
+      </x:c>
+      <x:c r="V22" s="36" t="str">
+        <x:v>2026-06-30T20:07:26Z</x:v>
+      </x:c>
+      <x:c r="W22" s="36" t="str">
+        <x:v>2026-07-01T20:07:26Z</x:v>
+      </x:c>
       <x:c r="X22" s="36"/>
       <x:c r="Y22" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z22" s="36" t="str">
-        <x:v>Migrated from GitHub issue #670; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
       </x:c>
       <x:c r="AA22" s="36"/>
       <x:c r="AB22" s="36"/>
       <x:c r="AC22" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim EPIC_05/STORY_01/SUBSTORY_01 #670 python plugin trust boundary (#1058)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5760,25 +5760,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q22" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R22" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R22" s="36" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
+      </x:c>
       <x:c r="S22" s="36"/>
-      <x:c r="T22" s="36"/>
-      <x:c r="U22" s="36"/>
-      <x:c r="V22" s="36"/>
-      <x:c r="W22" s="36"/>
+      <x:c r="T22" s="36" t="str">
+        <x:v>866b9190-9672-423a-84e6-7a89992a38e3</x:v>
+      </x:c>
+      <x:c r="U22" s="36" t="str">
+        <x:v>2026-06-30T20:07:26Z</x:v>
+      </x:c>
+      <x:c r="V22" s="36" t="str">
+        <x:v>2026-06-30T20:07:26Z</x:v>
+      </x:c>
+      <x:c r="W22" s="36" t="str">
+        <x:v>2026-07-01T20:07:26Z</x:v>
+      </x:c>
       <x:c r="X22" s="36"/>
       <x:c r="Y22" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z22" s="36" t="str">
-        <x:v>Migrated from GitHub issue #670; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
       </x:c>
       <x:c r="AA22" s="36"/>
       <x:c r="AB22" s="36"/>
       <x:c r="AC22" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim EPIC_02/STORY_02/SUBSTORY_01 #673 harden Windows CI
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6032,25 +6032,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/vcpkg triplets/manifests</x:v>
       </x:c>
       <x:c r="Q25" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R25" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R25" s="39" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
+      </x:c>
       <x:c r="S25" s="39"/>
-      <x:c r="T25" s="39"/>
-      <x:c r="U25" s="39"/>
-      <x:c r="V25" s="39"/>
-      <x:c r="W25" s="39"/>
+      <x:c r="T25" s="39" t="str">
+        <x:v>ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
+      </x:c>
+      <x:c r="U25" s="39" t="str">
+        <x:v>2026-06-30T20:15:07Z</x:v>
+      </x:c>
+      <x:c r="V25" s="39" t="str">
+        <x:v>2026-06-30T20:15:07Z</x:v>
+      </x:c>
+      <x:c r="W25" s="39" t="str">
+        <x:v>2026-07-01T20:15:07Z</x:v>
+      </x:c>
       <x:c r="X25" s="39"/>
       <x:c r="Y25" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z25" s="39" t="str">
-        <x:v>Migrated from GitHub issue #673; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
       </x:c>
       <x:c r="AA25" s="39"/>
       <x:c r="AB25" s="39"/>
       <x:c r="AC25" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim EPIC_02/STORY_02/SUBSTORY_01 #673 harden Windows CI (#1062)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6032,25 +6032,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/vcpkg triplets/manifests</x:v>
       </x:c>
       <x:c r="Q25" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R25" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R25" s="39" t="str">
+        <x:v>controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
+      </x:c>
       <x:c r="S25" s="39"/>
-      <x:c r="T25" s="39"/>
-      <x:c r="U25" s="39"/>
-      <x:c r="V25" s="39"/>
-      <x:c r="W25" s="39"/>
+      <x:c r="T25" s="39" t="str">
+        <x:v>ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
+      </x:c>
+      <x:c r="U25" s="39" t="str">
+        <x:v>2026-06-30T20:15:07Z</x:v>
+      </x:c>
+      <x:c r="V25" s="39" t="str">
+        <x:v>2026-06-30T20:15:07Z</x:v>
+      </x:c>
+      <x:c r="W25" s="39" t="str">
+        <x:v>2026-07-01T20:15:07Z</x:v>
+      </x:c>
       <x:c r="X25" s="39"/>
       <x:c r="Y25" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z25" s="39" t="str">
-        <x:v>Migrated from GitHub issue #673; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
       </x:c>
       <x:c r="AA25" s="39"/>
       <x:c r="AB25" s="39"/>
       <x:c r="AC25" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="72" customHeight="1">

</xml_diff>

<commit_message>
queue: claim refills #629 minimap-clicks (s25) + #625 disable-drag-drop (s26)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5038,25 +5038,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q13" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R13" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R13" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
+      </x:c>
       <x:c r="S13" s="39"/>
-      <x:c r="T13" s="39"/>
-      <x:c r="U13" s="39"/>
-      <x:c r="V13" s="39"/>
-      <x:c r="W13" s="39"/>
+      <x:c r="T13" s="39" t="str">
+        <x:v>c0935304-fd88-4899-8303-41fad1683ec5</x:v>
+      </x:c>
+      <x:c r="U13" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="V13" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="W13" s="39" t="str">
+        <x:v>2026-07-01T01:22:21Z</x:v>
+      </x:c>
       <x:c r="X13" s="39"/>
       <x:c r="Y13" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z13" s="39" t="str">
-        <x:v>Migrated from GitHub issue #625; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
       </x:c>
       <x:c r="AA13" s="39"/>
       <x:c r="AB13" s="39"/>
       <x:c r="AC13" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
@@ -5354,25 +5364,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/object/CGameGraphicsObject.cpp</x:v>
       </x:c>
       <x:c r="Q17" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R17" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R17" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
+      </x:c>
       <x:c r="S17" s="39"/>
-      <x:c r="T17" s="39"/>
-      <x:c r="U17" s="39"/>
-      <x:c r="V17" s="39"/>
-      <x:c r="W17" s="39"/>
+      <x:c r="T17" s="39" t="str">
+        <x:v>be8ec7b7-1bad-4837-aa77-556fcfb20b85</x:v>
+      </x:c>
+      <x:c r="U17" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="V17" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="W17" s="39" t="str">
+        <x:v>2026-07-01T01:22:21Z</x:v>
+      </x:c>
       <x:c r="X17" s="39"/>
       <x:c r="Y17" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z17" s="39" t="str">
-        <x:v>Migrated from GitHub issue #629; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
       </x:c>
       <x:c r="AA17" s="39"/>
       <x:c r="AB17" s="39"/>
       <x:c r="AC17" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="72" customHeight="1">

</xml_diff>

<commit_message>
queue: claim refills #629 minimap-clicks (s25) + #625 disable-drag-drop (s26) (#1124)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5038,25 +5038,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q13" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R13" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R13" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
+      </x:c>
       <x:c r="S13" s="39"/>
-      <x:c r="T13" s="39"/>
-      <x:c r="U13" s="39"/>
-      <x:c r="V13" s="39"/>
-      <x:c r="W13" s="39"/>
+      <x:c r="T13" s="39" t="str">
+        <x:v>c0935304-fd88-4899-8303-41fad1683ec5</x:v>
+      </x:c>
+      <x:c r="U13" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="V13" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="W13" s="39" t="str">
+        <x:v>2026-07-01T01:22:21Z</x:v>
+      </x:c>
       <x:c r="X13" s="39"/>
       <x:c r="Y13" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z13" s="39" t="str">
-        <x:v>Migrated from GitHub issue #625; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
       </x:c>
       <x:c r="AA13" s="39"/>
       <x:c r="AB13" s="39"/>
       <x:c r="AC13" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
@@ -5354,25 +5364,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/object/CGameGraphicsObject.cpp</x:v>
       </x:c>
       <x:c r="Q17" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R17" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R17" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
+      </x:c>
       <x:c r="S17" s="39"/>
-      <x:c r="T17" s="39"/>
-      <x:c r="U17" s="39"/>
-      <x:c r="V17" s="39"/>
-      <x:c r="W17" s="39"/>
+      <x:c r="T17" s="39" t="str">
+        <x:v>be8ec7b7-1bad-4837-aa77-556fcfb20b85</x:v>
+      </x:c>
+      <x:c r="U17" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="V17" s="39" t="str">
+        <x:v>2026-06-30T23:22:21Z</x:v>
+      </x:c>
+      <x:c r="W17" s="39" t="str">
+        <x:v>2026-07-01T01:22:21Z</x:v>
+      </x:c>
       <x:c r="X17" s="39"/>
       <x:c r="Y17" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z17" s="39" t="str">
-        <x:v>Migrated from GitHub issue #629; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
       </x:c>
       <x:c r="AA17" s="39"/>
       <x:c r="AB17" s="39"/>
       <x:c r="AC17" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="72" customHeight="1">

</xml_diff>

<commit_message>
queue: DONE minimap #629 (#1127) + disable-drag #625 (#1131); claim refills #628 (s27) + #630 (s28)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5038,7 +5038,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q13" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R13" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
@@ -5051,20 +5051,24 @@
         <x:v>2026-06-30T23:22:21Z</x:v>
       </x:c>
       <x:c r="V13" s="39" t="str">
-        <x:v>2026-06-30T23:22:21Z</x:v>
-      </x:c>
-      <x:c r="W13" s="39" t="str">
-        <x:v>2026-07-01T01:22:21Z</x:v>
-      </x:c>
-      <x:c r="X13" s="39"/>
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
+      <x:c r="W13" s="39"/>
+      <x:c r="X13" s="39" t="str">
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
       <x:c r="Y13" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z13" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
-      </x:c>
-      <x:c r="AA13" s="39"/>
-      <x:c r="AB13" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA13" s="39" t="str">
+        <x:v>Added CListView dragEnabled property (default true, backward-compatible; audited all 10 CListView usages in panels.json) and gated both drag-initiation paths so a non-draggable list never calls startDragSession/capturePointer/proxy at mouse-down; left/right click + click callback still fire. panels.json sets dragEnabled false on the two interaction/command lists only. Native gui tests cover click-only press/motion/release, repeated first-select/second-confirm, inventory-still-drags regression, and panel-removal-no-dangling. Merged as PR #1131.</x:v>
+      </x:c>
+      <x:c r="AB13" s="39" t="str">
+        <x:v>ctest gui_unit_tests + gui_drag_proxy_unit_tests green on linux and windows on PR #1131; validate_content passed. All required lanes green.</x:v>
+      </x:c>
       <x:c r="AC13" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -5286,25 +5290,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/panel/CGameFightPanel.cpp</x:v>
       </x:c>
       <x:c r="Q16" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R16" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R16" s="36" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
+      </x:c>
       <x:c r="S16" s="36"/>
-      <x:c r="T16" s="36"/>
-      <x:c r="U16" s="36"/>
-      <x:c r="V16" s="36"/>
-      <x:c r="W16" s="36"/>
+      <x:c r="T16" s="36" t="str">
+        <x:v>ef3a15f3-b518-47c9-967e-5ce31dd710a0</x:v>
+      </x:c>
+      <x:c r="U16" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="V16" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="W16" s="36" t="str">
+        <x:v>2026-07-01T02:01:55Z</x:v>
+      </x:c>
       <x:c r="X16" s="36"/>
       <x:c r="Y16" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z16" s="36" t="str">
-        <x:v>Migrated from GitHub issue #628; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
       </x:c>
       <x:c r="AA16" s="36"/>
       <x:c r="AB16" s="36"/>
       <x:c r="AC16" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="72" customHeight="1">
@@ -5364,7 +5378,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/object/CGameGraphicsObject.cpp</x:v>
       </x:c>
       <x:c r="Q17" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R17" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
@@ -5377,20 +5391,24 @@
         <x:v>2026-06-30T23:22:21Z</x:v>
       </x:c>
       <x:c r="V17" s="39" t="str">
-        <x:v>2026-06-30T23:22:21Z</x:v>
-      </x:c>
-      <x:c r="W17" s="39" t="str">
-        <x:v>2026-07-01T01:22:21Z</x:v>
-      </x:c>
-      <x:c r="X17" s="39"/>
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
+      <x:c r="W17" s="39"/>
+      <x:c r="X17" s="39" t="str">
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
       <x:c r="Y17" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z17" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
-      </x:c>
-      <x:c r="AA17" s="39"/>
-      <x:c r="AB17" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA17" s="39" t="str">
+        <x:v>CMinimapGraphicsObject::mouseEvent now returns handled and a mouseMotionEvent override returns handled, so in-bounds pointer button/motion events are consumed and never fall through to the underlying map; wheel deliberately falls through (map zoom). Relies on the base CGameGraphicsObject dispatcher in-bounds+visibility gating. Native gui_unit_tests test_minimap_consumes_inside_pointer_events_and_preserves_outside_and_wheel covers inside-consume, outside-by-one-pixel fallthrough, wheel fallthrough, hidden-minimap, modal precedence. CGui.cpp untouched. Merged as PR #1127.</x:v>
+      </x:c>
+      <x:c r="AB17" s="39" t="str">
+        <x:v>ctest gui_unit_tests green on linux and windows on PR #1127. All required lanes green.</x:v>
+      </x:c>
       <x:c r="AC17" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -5453,25 +5471,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/maps/nouraajd/dialog2.json</x:v>
       </x:c>
       <x:c r="Q18" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R18" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R18" s="36" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
+      </x:c>
       <x:c r="S18" s="36"/>
-      <x:c r="T18" s="36"/>
-      <x:c r="U18" s="36"/>
-      <x:c r="V18" s="36"/>
-      <x:c r="W18" s="36"/>
+      <x:c r="T18" s="36" t="str">
+        <x:v>783ec46c-a4d5-408d-b4a7-992596f12d01</x:v>
+      </x:c>
+      <x:c r="U18" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="V18" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="W18" s="36" t="str">
+        <x:v>2026-07-01T02:01:55Z</x:v>
+      </x:c>
       <x:c r="X18" s="36"/>
       <x:c r="Y18" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z18" s="36" t="str">
-        <x:v>Migrated from GitHub issue #630; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
       </x:c>
       <x:c r="AA18" s="36"/>
       <x:c r="AB18" s="36"/>
       <x:c r="AC18" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">

</xml_diff>

<commit_message>
queue: DONE minimap #629 (#1127) + disable-drag #625 (#1131); claim refills #628 (s27) + #630 (s28) (#1137)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5038,7 +5038,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q13" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R13" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
@@ -5051,20 +5051,24 @@
         <x:v>2026-06-30T23:22:21Z</x:v>
       </x:c>
       <x:c r="V13" s="39" t="str">
-        <x:v>2026-06-30T23:22:21Z</x:v>
-      </x:c>
-      <x:c r="W13" s="39" t="str">
-        <x:v>2026-07-01T01:22:21Z</x:v>
-      </x:c>
-      <x:c r="X13" s="39"/>
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
+      <x:c r="W13" s="39"/>
+      <x:c r="X13" s="39" t="str">
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
       <x:c r="Y13" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z13" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-26</x:v>
-      </x:c>
-      <x:c r="AA13" s="39"/>
-      <x:c r="AB13" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA13" s="39" t="str">
+        <x:v>Added CListView dragEnabled property (default true, backward-compatible; audited all 10 CListView usages in panels.json) and gated both drag-initiation paths so a non-draggable list never calls startDragSession/capturePointer/proxy at mouse-down; left/right click + click callback still fire. panels.json sets dragEnabled false on the two interaction/command lists only. Native gui tests cover click-only press/motion/release, repeated first-select/second-confirm, inventory-still-drags regression, and panel-removal-no-dangling. Merged as PR #1131.</x:v>
+      </x:c>
+      <x:c r="AB13" s="39" t="str">
+        <x:v>ctest gui_unit_tests + gui_drag_proxy_unit_tests green on linux and windows on PR #1131; validate_content passed. All required lanes green.</x:v>
+      </x:c>
       <x:c r="AC13" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -5286,25 +5290,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/panel/CGameFightPanel.cpp</x:v>
       </x:c>
       <x:c r="Q16" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R16" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R16" s="36" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
+      </x:c>
       <x:c r="S16" s="36"/>
-      <x:c r="T16" s="36"/>
-      <x:c r="U16" s="36"/>
-      <x:c r="V16" s="36"/>
-      <x:c r="W16" s="36"/>
+      <x:c r="T16" s="36" t="str">
+        <x:v>ef3a15f3-b518-47c9-967e-5ce31dd710a0</x:v>
+      </x:c>
+      <x:c r="U16" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="V16" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="W16" s="36" t="str">
+        <x:v>2026-07-01T02:01:55Z</x:v>
+      </x:c>
       <x:c r="X16" s="36"/>
       <x:c r="Y16" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z16" s="36" t="str">
-        <x:v>Migrated from GitHub issue #628; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
       </x:c>
       <x:c r="AA16" s="36"/>
       <x:c r="AB16" s="36"/>
       <x:c r="AC16" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="72" customHeight="1">
@@ -5364,7 +5378,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/object/CGameGraphicsObject.cpp</x:v>
       </x:c>
       <x:c r="Q17" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R17" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
@@ -5377,20 +5391,24 @@
         <x:v>2026-06-30T23:22:21Z</x:v>
       </x:c>
       <x:c r="V17" s="39" t="str">
-        <x:v>2026-06-30T23:22:21Z</x:v>
-      </x:c>
-      <x:c r="W17" s="39" t="str">
-        <x:v>2026-07-01T01:22:21Z</x:v>
-      </x:c>
-      <x:c r="X17" s="39"/>
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
+      <x:c r="W17" s="39"/>
+      <x:c r="X17" s="39" t="str">
+        <x:v>2026-07-01T00:00:31Z</x:v>
+      </x:c>
       <x:c r="Y17" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z17" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-25</x:v>
-      </x:c>
-      <x:c r="AA17" s="39"/>
-      <x:c r="AB17" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA17" s="39" t="str">
+        <x:v>CMinimapGraphicsObject::mouseEvent now returns handled and a mouseMotionEvent override returns handled, so in-bounds pointer button/motion events are consumed and never fall through to the underlying map; wheel deliberately falls through (map zoom). Relies on the base CGameGraphicsObject dispatcher in-bounds+visibility gating. Native gui_unit_tests test_minimap_consumes_inside_pointer_events_and_preserves_outside_and_wheel covers inside-consume, outside-by-one-pixel fallthrough, wheel fallthrough, hidden-minimap, modal precedence. CGui.cpp untouched. Merged as PR #1127.</x:v>
+      </x:c>
+      <x:c r="AB17" s="39" t="str">
+        <x:v>ctest gui_unit_tests green on linux and windows on PR #1127. All required lanes green.</x:v>
+      </x:c>
       <x:c r="AC17" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -5453,25 +5471,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/maps/nouraajd/dialog2.json</x:v>
       </x:c>
       <x:c r="Q18" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R18" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R18" s="36" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
+      </x:c>
       <x:c r="S18" s="36"/>
-      <x:c r="T18" s="36"/>
-      <x:c r="U18" s="36"/>
-      <x:c r="V18" s="36"/>
-      <x:c r="W18" s="36"/>
+      <x:c r="T18" s="36" t="str">
+        <x:v>783ec46c-a4d5-408d-b4a7-992596f12d01</x:v>
+      </x:c>
+      <x:c r="U18" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="V18" s="36" t="str">
+        <x:v>2026-07-01T00:01:55Z</x:v>
+      </x:c>
+      <x:c r="W18" s="36" t="str">
+        <x:v>2026-07-01T02:01:55Z</x:v>
+      </x:c>
       <x:c r="X18" s="36"/>
       <x:c r="Y18" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z18" s="36" t="str">
-        <x:v>Migrated from GitHub issue #630; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
       </x:c>
       <x:c r="AA18" s="36"/>
       <x:c r="AB18" s="36"/>
       <x:c r="AC18" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Complete EPIC_04/STORY_01/SUBSTORY_01 reliable oldWoman/questGiver conversations (impl PR #1143)
Marks the quest-NPC conversation-reliability substory DONE in the migrated workbook
after PR #1143 merged (all required CI lanes green). oldWoman and questGiver are now
stationary CController NPCs so their onEnter dialog triggers fire deterministically.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5481,7 +5481,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/maps/nouraajd/dialog2.json</x:v>
       </x:c>
       <x:c r="Q18" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R18" s="36" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
@@ -5494,20 +5494,24 @@
         <x:v>2026-07-01T00:01:55Z</x:v>
       </x:c>
       <x:c r="V18" s="36" t="str">
-        <x:v>2026-07-01T00:01:55Z</x:v>
-      </x:c>
-      <x:c r="W18" s="36" t="str">
-        <x:v>2026-07-01T02:01:55Z</x:v>
-      </x:c>
-      <x:c r="X18" s="36"/>
+        <x:v>2026-07-01T00:43:08Z</x:v>
+      </x:c>
+      <x:c r="W18" s="36"/>
+      <x:c r="X18" s="36" t="str">
+        <x:v>2026-07-01T00:43:08Z</x:v>
+      </x:c>
       <x:c r="Y18" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z18" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
-      </x:c>
-      <x:c r="AA18" s="36"/>
-      <x:c r="AB18" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA18" s="36" t="str">
+        <x:v>Restored reliable conversations with oldWoman and questGiver. Root cause: both NPCs used CNpcRandomController and wandered off their exact trigger tiles, so onEnter dialog triggers fired unreliably. Changed only the oldWoman and questGiver controller definitions in res/maps/nouraajd/config.json from CNpcRandomController to the stationary CController, keeping exact IDs (oldWoman, questGiver, questDialog, questReturnDialog, dialog) intact so both NPCs stay on their trigger tiles and their dialog chains fire deterministically. Added a deterministic Nouraajd gameplay test exercising initial quest dialog, active reminder, amulet-return completion (once), questGiver OctoBogz dialog, no NPC-initiated combat, and save/load + repeated-approach stability. Merged via PR #1143.</x:v>
+      </x:c>
+      <x:c r="AB18" s="36" t="str">
+        <x:v>CI build workflow green on merge commit: validate, export, linux-fast, linux, windows-deps, windows all passed. New deterministic Nouraajd conversation test (test_nouraajd_oldwoman_questgiver_conversations_are_reliable) passes on linux and windows GameTest lanes.</x:v>
+      </x:c>
       <x:c r="AC18" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Complete EPIC_04/STORY_01/SUBSTORY_01 reliable oldWoman/questGiver conversations (impl PR #1143) (#1149)
Marks the quest-NPC conversation-reliability substory DONE in the migrated workbook
after PR #1143 merged (all required CI lanes green). oldWoman and questGiver are now
stationary CController NPCs so their onEnter dialog triggers fire deterministically.


Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5481,7 +5481,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/maps/nouraajd/dialog2.json</x:v>
       </x:c>
       <x:c r="Q18" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R18" s="36" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
@@ -5494,20 +5494,24 @@
         <x:v>2026-07-01T00:01:55Z</x:v>
       </x:c>
       <x:c r="V18" s="36" t="str">
-        <x:v>2026-07-01T00:01:55Z</x:v>
-      </x:c>
-      <x:c r="W18" s="36" t="str">
-        <x:v>2026-07-01T02:01:55Z</x:v>
-      </x:c>
-      <x:c r="X18" s="36"/>
+        <x:v>2026-07-01T00:43:08Z</x:v>
+      </x:c>
+      <x:c r="W18" s="36"/>
+      <x:c r="X18" s="36" t="str">
+        <x:v>2026-07-01T00:43:08Z</x:v>
+      </x:c>
       <x:c r="Y18" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z18" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-28</x:v>
-      </x:c>
-      <x:c r="AA18" s="36"/>
-      <x:c r="AB18" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA18" s="36" t="str">
+        <x:v>Restored reliable conversations with oldWoman and questGiver. Root cause: both NPCs used CNpcRandomController and wandered off their exact trigger tiles, so onEnter dialog triggers fired unreliably. Changed only the oldWoman and questGiver controller definitions in res/maps/nouraajd/config.json from CNpcRandomController to the stationary CController, keeping exact IDs (oldWoman, questGiver, questDialog, questReturnDialog, dialog) intact so both NPCs stay on their trigger tiles and their dialog chains fire deterministically. Added a deterministic Nouraajd gameplay test exercising initial quest dialog, active reminder, amulet-return completion (once), questGiver OctoBogz dialog, no NPC-initiated combat, and save/load + repeated-approach stability. Merged via PR #1143.</x:v>
+      </x:c>
+      <x:c r="AB18" s="36" t="str">
+        <x:v>CI build workflow green on merge commit: validate, export, linux-fast, linux, windows-deps, windows all passed. New deterministic Nouraajd conversation test (test_nouraajd_oldwoman_questgiver_conversations_are_reliable) passes on linux and windows GameTest lanes.</x:v>
+      </x:c>
       <x:c r="AC18" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Heartbeat migrated claim s27 #628 (lease extended)
Extend lease for actively-owned, PR-complete claim s27 (inventory
right-click, PR #1141) awaiting the CI test-shard unblock (#1164).
Owner controller/ctrl-vm-4039-a70f65a5/subagent-27. No code files touched.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5317,17 +5317,17 @@
         <x:v>2026-07-01T00:01:55Z</x:v>
       </x:c>
       <x:c r="V16" s="36" t="str">
-        <x:v>2026-07-01T00:01:55Z</x:v>
+        <x:v>2026-07-01T05:25:47Z</x:v>
       </x:c>
       <x:c r="W16" s="36" t="str">
-        <x:v>2026-07-01T02:01:55Z</x:v>
+        <x:v>2026-07-01T07:25:47Z</x:v>
       </x:c>
       <x:c r="X16" s="36"/>
       <x:c r="Y16" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z16" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
+        <x:v>impl complete; PR #1141 open, awaiting CI unblock via test-shard fix #1164</x:v>
       </x:c>
       <x:c r="AA16" s="36"/>
       <x:c r="AB16" s="36"/>

</xml_diff>

<commit_message>
Heartbeat migrated claim s27 #628 (lease extended) (#1168)
Extend lease for actively-owned, PR-complete claim s27 (inventory
right-click, PR #1141) awaiting the CI test-shard unblock (#1164).
Owner controller/ctrl-vm-4039-a70f65a5/subagent-27. No code files touched.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5317,17 +5317,17 @@
         <x:v>2026-07-01T00:01:55Z</x:v>
       </x:c>
       <x:c r="V16" s="36" t="str">
-        <x:v>2026-07-01T00:01:55Z</x:v>
+        <x:v>2026-07-01T05:25:47Z</x:v>
       </x:c>
       <x:c r="W16" s="36" t="str">
-        <x:v>2026-07-01T02:01:55Z</x:v>
+        <x:v>2026-07-01T07:25:47Z</x:v>
       </x:c>
       <x:c r="X16" s="36"/>
       <x:c r="Y16" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z16" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
+        <x:v>impl complete; PR #1141 open, awaiting CI unblock via test-shard fix #1164</x:v>
       </x:c>
       <x:c r="AA16" s="36"/>
       <x:c r="AB16" s="36"/>

</xml_diff>

<commit_message>
Mark s27 DONE in migrated workbook
Terminal update for merged implementation PR:
- s27 #628 inventory right-click use -> PR #1141 (merged)
Owner controller/ctrl-vm-4039-a70f65a5/subagent-27. Queue-workbook change only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5304,7 +5304,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/panel/CGameFightPanel.cpp</x:v>
       </x:c>
       <x:c r="Q16" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R16" s="36" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
@@ -5317,20 +5317,24 @@
         <x:v>2026-07-01T00:01:55Z</x:v>
       </x:c>
       <x:c r="V16" s="36" t="str">
-        <x:v>2026-07-01T05:25:47Z</x:v>
-      </x:c>
-      <x:c r="W16" s="36" t="str">
-        <x:v>2026-07-01T07:25:47Z</x:v>
-      </x:c>
-      <x:c r="X16" s="36"/>
+        <x:v>2026-07-01T11:30:57Z</x:v>
+      </x:c>
+      <x:c r="W16" s="36"/>
+      <x:c r="X16" s="36" t="str">
+        <x:v>2026-07-01T11:30:57Z</x:v>
+      </x:c>
       <x:c r="Y16" s="36" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z16" s="36" t="str">
-        <x:v>impl complete; PR #1141 open, awaiting CI unblock via test-shard fix #1164</x:v>
-      </x:c>
-      <x:c r="AA16" s="36"/>
-      <x:c r="AB16" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA16" s="36" t="str">
+        <x:v>Merged in PR #1141: rewrote CGameInventoryPanel::inventoryRightClickCallback to call player-&gt;useItem via usable_item/inventory_player helpers, mirroring the fight panel; +tests in test_gui.cpp.</x:v>
+      </x:c>
+      <x:c r="AB16" s="36" t="str">
+        <x:v>CI green on merge (validate/export/linux-fast/linux/windows). gui_unit_tests cover use+consume, quest-item protection, drag-still-starts.</x:v>
+      </x:c>
       <x:c r="AC16" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark s27 DONE in migrated workbook (#1224)
Terminal update for merged implementation PR:
- s27 #628 inventory right-click use -> PR #1141 (merged)
Owner controller/ctrl-vm-4039-a70f65a5/subagent-27. Queue-workbook change only.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5304,7 +5304,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/panel/CGameFightPanel.cpp</x:v>
       </x:c>
       <x:c r="Q16" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R16" s="36" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-27</x:v>
@@ -5317,20 +5317,24 @@
         <x:v>2026-07-01T00:01:55Z</x:v>
       </x:c>
       <x:c r="V16" s="36" t="str">
-        <x:v>2026-07-01T05:25:47Z</x:v>
-      </x:c>
-      <x:c r="W16" s="36" t="str">
-        <x:v>2026-07-01T07:25:47Z</x:v>
-      </x:c>
-      <x:c r="X16" s="36"/>
+        <x:v>2026-07-01T11:30:57Z</x:v>
+      </x:c>
+      <x:c r="W16" s="36"/>
+      <x:c r="X16" s="36" t="str">
+        <x:v>2026-07-01T11:30:57Z</x:v>
+      </x:c>
       <x:c r="Y16" s="36" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z16" s="36" t="str">
-        <x:v>impl complete; PR #1141 open, awaiting CI unblock via test-shard fix #1164</x:v>
-      </x:c>
-      <x:c r="AA16" s="36"/>
-      <x:c r="AB16" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA16" s="36" t="str">
+        <x:v>Merged in PR #1141: rewrote CGameInventoryPanel::inventoryRightClickCallback to call player-&gt;useItem via usable_item/inventory_player helpers, mirroring the fight panel; +tests in test_gui.cpp.</x:v>
+      </x:c>
+      <x:c r="AB16" s="36" t="str">
+        <x:v>CI green on merge (validate/export/linux-fast/linux/windows). gui_unit_tests cover use+consume, quest-item protection, drag-still-starts.</x:v>
+      </x:c>
       <x:c r="AC16" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Reclaim stale claim on row 21 (#669) from dead controller
Lease expired 231 min ago; heartbeat overdue; owning controller
ctrl-vm-4026 gone with no open PR / recoverable pushed work.
Returns the row to the available pool.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5769,30 +5769,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R21" s="39" t="str">
-        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R21" s="39"/>
       <x:c r="S21" s="39"/>
-      <x:c r="T21" s="39" t="str">
-        <x:v>4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
-      </x:c>
-      <x:c r="U21" s="39" t="str">
-        <x:v>2026-06-30T11:06:18Z</x:v>
-      </x:c>
+      <x:c r="T21" s="39"/>
+      <x:c r="U21" s="39"/>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-06-30T12:22:37Z</x:v>
-      </x:c>
-      <x:c r="W21" s="39" t="str">
-        <x:v>2026-07-01T12:22:37Z</x:v>
-      </x:c>
+        <x:v>2026-07-01T16:15:09Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39"/>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim. awaiting user review of authority-machinery PR #934.</x:v>
+        <x:v>Stale claim reclaimed from controller/ctrl-vm-4026-9b5a29b5/subagent-5; prior claim 4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>

</xml_diff>

<commit_message>
Reclaim stale abandoned claim on row 21 (#669) (#1236)
Lease expired 231 min ago; heartbeat overdue; owning controller
ctrl-vm-4026 gone with no open PR / recoverable pushed work.
Returns the row to the available pool.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5769,30 +5769,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R21" s="39" t="str">
-        <x:v>controller/ctrl-vm-4026-9b5a29b5/subagent-5</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R21" s="39"/>
       <x:c r="S21" s="39"/>
-      <x:c r="T21" s="39" t="str">
-        <x:v>4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
-      </x:c>
-      <x:c r="U21" s="39" t="str">
-        <x:v>2026-06-30T11:06:18Z</x:v>
-      </x:c>
+      <x:c r="T21" s="39"/>
+      <x:c r="U21" s="39"/>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-06-30T12:22:37Z</x:v>
-      </x:c>
-      <x:c r="W21" s="39" t="str">
-        <x:v>2026-07-01T12:22:37Z</x:v>
-      </x:c>
+        <x:v>2026-07-01T16:15:09Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39"/>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Implementation complete and pushed; blocked only on main-red native CI (test_scene_manager_transition_requested_during_combat_preserves_source_map, a pre-existing combat-transition regression on main, observed 05b033bd). Do not reclaim. awaiting user review of authority-machinery PR #934.</x:v>
+        <x:v>Stale claim reclaimed from controller/ctrl-vm-4026-9b5a29b5/subagent-5; prior claim 4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>

</xml_diff>

<commit_message>
Reclaim stale claim on row 22 (#670) from dead controller
Lease expired; heartbeat overdue past stale threshold. Owning
controller ctrl-vm-4024 is gone with no open PR / recoverable pushed
work for #670. Returns the row to the available pool.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5850,30 +5850,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q22" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R22" s="36" t="str">
-        <x:v>controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R22" s="36"/>
       <x:c r="S22" s="36"/>
-      <x:c r="T22" s="36" t="str">
-        <x:v>866b9190-9672-423a-84e6-7a89992a38e3</x:v>
-      </x:c>
-      <x:c r="U22" s="36" t="str">
-        <x:v>2026-06-30T20:07:26Z</x:v>
-      </x:c>
+      <x:c r="T22" s="36"/>
+      <x:c r="U22" s="36"/>
       <x:c r="V22" s="36" t="str">
-        <x:v>2026-06-30T20:07:26Z</x:v>
-      </x:c>
-      <x:c r="W22" s="36" t="str">
-        <x:v>2026-07-01T20:07:26Z</x:v>
-      </x:c>
+        <x:v>2026-07-01T20:13:02Z</x:v>
+      </x:c>
+      <x:c r="W22" s="36"/>
       <x:c r="X22" s="36"/>
       <x:c r="Y22" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z22" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
+        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-10; prior claim 866b9190-9672-423a-84e6-7a89992a38e3</x:v>
       </x:c>
       <x:c r="AA22" s="36"/>
       <x:c r="AB22" s="36"/>

</xml_diff>

<commit_message>
Reclaim stale abandoned claim on row 22 (#670) (#1257)
Lease expired; heartbeat overdue past stale threshold. Owning
controller ctrl-vm-4024 is gone with no open PR / recoverable pushed
work for #670. Returns the row to the available pool.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5850,30 +5850,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q22" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R22" s="36" t="str">
-        <x:v>controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R22" s="36"/>
       <x:c r="S22" s="36"/>
-      <x:c r="T22" s="36" t="str">
-        <x:v>866b9190-9672-423a-84e6-7a89992a38e3</x:v>
-      </x:c>
-      <x:c r="U22" s="36" t="str">
-        <x:v>2026-06-30T20:07:26Z</x:v>
-      </x:c>
+      <x:c r="T22" s="36"/>
+      <x:c r="U22" s="36"/>
       <x:c r="V22" s="36" t="str">
-        <x:v>2026-06-30T20:07:26Z</x:v>
-      </x:c>
-      <x:c r="W22" s="36" t="str">
-        <x:v>2026-07-01T20:07:26Z</x:v>
-      </x:c>
+        <x:v>2026-07-01T20:13:02Z</x:v>
+      </x:c>
+      <x:c r="W22" s="36"/>
       <x:c r="X22" s="36"/>
       <x:c r="Y22" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z22" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-10</x:v>
+        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-10; prior claim 866b9190-9672-423a-84e6-7a89992a38e3</x:v>
       </x:c>
       <x:c r="AA22" s="36"/>
       <x:c r="AB22" s="36"/>

</xml_diff>

<commit_message>
Reclaim stale claim on row 25 (#673) from dead controller
Lease expired; heartbeat overdue past stale threshold. Owning
controller ctrl-vm-4024 is gone with no open PR / recoverable pushed
work for #673. Returns the row to the available pool.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6114,30 +6114,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/vcpkg triplets/manifests</x:v>
       </x:c>
       <x:c r="Q25" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R25" s="39" t="str">
-        <x:v>controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R25" s="39"/>
       <x:c r="S25" s="39"/>
-      <x:c r="T25" s="39" t="str">
-        <x:v>ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
-      </x:c>
-      <x:c r="U25" s="39" t="str">
-        <x:v>2026-06-30T20:15:07Z</x:v>
-      </x:c>
+      <x:c r="T25" s="39"/>
+      <x:c r="U25" s="39"/>
       <x:c r="V25" s="39" t="str">
-        <x:v>2026-06-30T20:15:07Z</x:v>
-      </x:c>
-      <x:c r="W25" s="39" t="str">
-        <x:v>2026-07-01T20:15:07Z</x:v>
-      </x:c>
+        <x:v>2026-07-01T20:17:34Z</x:v>
+      </x:c>
+      <x:c r="W25" s="39"/>
       <x:c r="X25" s="39"/>
       <x:c r="Y25" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z25" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
+        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-11; prior claim ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
       </x:c>
       <x:c r="AA25" s="39"/>
       <x:c r="AB25" s="39"/>

</xml_diff>

<commit_message>
Reclaim stale abandoned claim on row 25 (#673) (#1258)
Lease expired; heartbeat overdue past stale threshold. Owning
controller ctrl-vm-4024 is gone with no open PR / recoverable pushed
work for #673. Returns the row to the available pool.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6114,30 +6114,22 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/vcpkg triplets/manifests</x:v>
       </x:c>
       <x:c r="Q25" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
-      </x:c>
-      <x:c r="R25" s="39" t="str">
-        <x:v>controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
-      </x:c>
+        <x:v>NOT_STARTED</x:v>
+      </x:c>
+      <x:c r="R25" s="39"/>
       <x:c r="S25" s="39"/>
-      <x:c r="T25" s="39" t="str">
-        <x:v>ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
-      </x:c>
-      <x:c r="U25" s="39" t="str">
-        <x:v>2026-06-30T20:15:07Z</x:v>
-      </x:c>
+      <x:c r="T25" s="39"/>
+      <x:c r="U25" s="39"/>
       <x:c r="V25" s="39" t="str">
-        <x:v>2026-06-30T20:15:07Z</x:v>
-      </x:c>
-      <x:c r="W25" s="39" t="str">
-        <x:v>2026-07-01T20:15:07Z</x:v>
-      </x:c>
+        <x:v>2026-07-01T20:17:34Z</x:v>
+      </x:c>
+      <x:c r="W25" s="39"/>
       <x:c r="X25" s="39"/>
       <x:c r="Y25" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z25" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4024-7534d796/subagent-11</x:v>
+        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-11; prior claim ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
       </x:c>
       <x:c r="AA25" s="39"/>
       <x:c r="AB25" s="39"/>

</xml_diff>

<commit_message>
Reconcile #670 to DONE (satisfied by #1063) + claim #669 (PR #1261)
- EPIC_05/STORY_01/SUBSTORY_01 #670 'Python resource-plugin trust boundary':
  stale NOT_STARTED row reconciled to DONE. Enforcement + docs landed in
  commit 483d1dc (#1063); tests.security.test_python_plugin_sandbox passes
  (8 tests: restricted builtins, game/json import allowlist, path-traversal
  rejection, trust-boundary doc, trusted content still loads).
- EPIC_02/STORY_01/SUBSTORY_02 #669 'Harden CI validation authority':
  claimed in-progress; implementation open as PR #1261 (run-identity
  ambiguity + attempt binding in poll_pr_checks.py).
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5769,27 +5769,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R21" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R21" s="39" t="str">
+        <x:v>ctrl-vm-2256-06ac44fc</x:v>
+      </x:c>
       <x:c r="S21" s="39"/>
-      <x:c r="T21" s="39"/>
-      <x:c r="U21" s="39"/>
+      <x:c r="T21" s="39" t="str">
+        <x:v>5a8f6b65-9460-4e5c-98aa-d1c57420b18f</x:v>
+      </x:c>
+      <x:c r="U21" s="39" t="str">
+        <x:v>2026-07-02T07:46:27Z</x:v>
+      </x:c>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-07-01T16:15:09Z</x:v>
-      </x:c>
-      <x:c r="W21" s="39"/>
+        <x:v>2026-07-02T07:46:39Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39" t="str">
+        <x:v>2026-07-02T09:46:39Z</x:v>
+      </x:c>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Stale claim reclaimed from controller/ctrl-vm-4026-9b5a29b5/subagent-5; prior claim 4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
+        <x:v>Implemented run-identity ambiguity + attempt binding in poll_pr_checks.py; PR #1261 open (fast-path CI green, 7 tests). Authority-file change awaits human review + native-green.</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>
       <x:c r="AC21" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="72" customHeight="1">
@@ -5850,27 +5858,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q22" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R22" s="36"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R22" s="36" t="str">
+        <x:v>ctrl-vm-2256-06ac44fc</x:v>
+      </x:c>
       <x:c r="S22" s="36"/>
-      <x:c r="T22" s="36"/>
-      <x:c r="U22" s="36"/>
+      <x:c r="T22" s="36" t="str">
+        <x:v>0a6bfa03-b5e8-4d7b-a7ee-f64508429e8c</x:v>
+      </x:c>
+      <x:c r="U22" s="36" t="str">
+        <x:v>2026-07-02T07:45:52Z</x:v>
+      </x:c>
       <x:c r="V22" s="36" t="str">
-        <x:v>2026-07-01T20:13:02Z</x:v>
+        <x:v>2026-07-02T07:46:26Z</x:v>
       </x:c>
       <x:c r="W22" s="36"/>
-      <x:c r="X22" s="36"/>
+      <x:c r="X22" s="36" t="str">
+        <x:v>2026-07-02T07:46:26Z</x:v>
+      </x:c>
       <x:c r="Y22" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z22" s="36" t="str">
-        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-10; prior claim 866b9190-9672-423a-84e6-7a89992a38e3</x:v>
-      </x:c>
-      <x:c r="AA22" s="36"/>
-      <x:c r="AB22" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA22" s="36" t="str">
+        <x:v>Already satisfied by #1063 (commit 483d1dc): docs/design/plugin_trust_boundary.md documents the trust model; CLoader.cpp enforces restricted plugin builtins, a game/json-only import allowlist, and resource-root path validation that rejects absolute/parent-traversal paths and plugins outside trusted roots. Reconciling stale NOT_STARTED row to DONE.</x:v>
+      </x:c>
+      <x:c r="AB22" s="36" t="str">
+        <x:v>python3 -m unittest tests.security.test_python_plugin_sandbox -&gt; Ran 8 tests, OK (restricted builtins, import allowlist, path-traversal rejection, trust-boundary doc present, trusted crafting plugin still loads via resource provider).</x:v>
+      </x:c>
       <x:c r="AC22" s="36" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Reconcile #670 to DONE (satisfied by #1063) + claim #669 (PR #1261) (#1262)
- EPIC_05/STORY_01/SUBSTORY_01 #670 'Python resource-plugin trust boundary':
  stale NOT_STARTED row reconciled to DONE. Enforcement + docs landed in
  commit 483d1dc (#1063); tests.security.test_python_plugin_sandbox passes
  (8 tests: restricted builtins, game/json import allowlist, path-traversal
  rejection, trust-boundary doc, trusted content still loads).
- EPIC_02/STORY_01/SUBSTORY_02 #669 'Harden CI validation authority':
  claimed in-progress; implementation open as PR #1261 (run-identity
  ambiguity + attempt binding in poll_pr_checks.py).
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5769,27 +5769,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R21" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R21" s="39" t="str">
+        <x:v>ctrl-vm-2256-06ac44fc</x:v>
+      </x:c>
       <x:c r="S21" s="39"/>
-      <x:c r="T21" s="39"/>
-      <x:c r="U21" s="39"/>
+      <x:c r="T21" s="39" t="str">
+        <x:v>5a8f6b65-9460-4e5c-98aa-d1c57420b18f</x:v>
+      </x:c>
+      <x:c r="U21" s="39" t="str">
+        <x:v>2026-07-02T07:46:27Z</x:v>
+      </x:c>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-07-01T16:15:09Z</x:v>
-      </x:c>
-      <x:c r="W21" s="39"/>
+        <x:v>2026-07-02T07:46:39Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39" t="str">
+        <x:v>2026-07-02T09:46:39Z</x:v>
+      </x:c>
       <x:c r="X21" s="39"/>
       <x:c r="Y21" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Stale claim reclaimed from controller/ctrl-vm-4026-9b5a29b5/subagent-5; prior claim 4d74f425-a323-41d6-931b-13cf0d913a14</x:v>
+        <x:v>Implemented run-identity ambiguity + attempt binding in poll_pr_checks.py; PR #1261 open (fast-path CI green, 7 tests). Authority-file change awaits human review + native-green.</x:v>
       </x:c>
       <x:c r="AA21" s="39"/>
       <x:c r="AB21" s="39"/>
       <x:c r="AC21" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="72" customHeight="1">
@@ -5850,27 +5858,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/res/game.py</x:v>
       </x:c>
       <x:c r="Q22" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R22" s="36"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R22" s="36" t="str">
+        <x:v>ctrl-vm-2256-06ac44fc</x:v>
+      </x:c>
       <x:c r="S22" s="36"/>
-      <x:c r="T22" s="36"/>
-      <x:c r="U22" s="36"/>
+      <x:c r="T22" s="36" t="str">
+        <x:v>0a6bfa03-b5e8-4d7b-a7ee-f64508429e8c</x:v>
+      </x:c>
+      <x:c r="U22" s="36" t="str">
+        <x:v>2026-07-02T07:45:52Z</x:v>
+      </x:c>
       <x:c r="V22" s="36" t="str">
-        <x:v>2026-07-01T20:13:02Z</x:v>
+        <x:v>2026-07-02T07:46:26Z</x:v>
       </x:c>
       <x:c r="W22" s="36"/>
-      <x:c r="X22" s="36"/>
+      <x:c r="X22" s="36" t="str">
+        <x:v>2026-07-02T07:46:26Z</x:v>
+      </x:c>
       <x:c r="Y22" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z22" s="36" t="str">
-        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-10; prior claim 866b9190-9672-423a-84e6-7a89992a38e3</x:v>
-      </x:c>
-      <x:c r="AA22" s="36"/>
-      <x:c r="AB22" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA22" s="36" t="str">
+        <x:v>Already satisfied by #1063 (commit 483d1dc): docs/design/plugin_trust_boundary.md documents the trust model; CLoader.cpp enforces restricted plugin builtins, a game/json-only import allowlist, and resource-root path validation that rejects absolute/parent-traversal paths and plugins outside trusted roots. Reconciling stale NOT_STARTED row to DONE.</x:v>
+      </x:c>
+      <x:c r="AB22" s="36" t="str">
+        <x:v>python3 -m unittest tests.security.test_python_plugin_sandbox -&gt; Ran 8 tests, OK (restricted builtins, import allowlist, path-traversal rejection, trust-boundary doc present, trusted crafting plugin still loads via resource provider).</x:v>
+      </x:c>
       <x:c r="AC22" s="36" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Reconcile #673 to DONE (satisfied by #1064)
EPIC_02/STORY_02/SUBSTORY_01 #673 'Harden Windows CI tool and vcpkg cache
validation': stale NOT_STARTED row reconciled to DONE. Hardening landed in
commit 4f9074a (#1064); tests.security.test_configure_supply_chain passes
(15 tests: trusted tools outside workspace, unconditional sccache hash
verification, vcpkg installed-cache validation + dependency-input cache key).
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6134,27 +6134,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/vcpkg triplets/manifests</x:v>
       </x:c>
       <x:c r="Q25" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R25" s="39"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R25" s="39" t="str">
+        <x:v>ctrl-vm-2256-06ac44fc</x:v>
+      </x:c>
       <x:c r="S25" s="39"/>
-      <x:c r="T25" s="39"/>
-      <x:c r="U25" s="39"/>
+      <x:c r="T25" s="39" t="str">
+        <x:v>9f2d6cae-5763-4e1a-897b-24bfcc42c8a1</x:v>
+      </x:c>
+      <x:c r="U25" s="39" t="str">
+        <x:v>2026-07-02T07:49:14Z</x:v>
+      </x:c>
       <x:c r="V25" s="39" t="str">
-        <x:v>2026-07-01T20:17:34Z</x:v>
+        <x:v>2026-07-02T07:49:14Z</x:v>
       </x:c>
       <x:c r="W25" s="39"/>
-      <x:c r="X25" s="39"/>
+      <x:c r="X25" s="39" t="str">
+        <x:v>2026-07-02T07:49:14Z</x:v>
+      </x:c>
       <x:c r="Y25" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z25" s="39" t="str">
-        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-11; prior claim ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
-      </x:c>
-      <x:c r="AA25" s="39"/>
-      <x:c r="AB25" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA25" s="39" t="str">
+        <x:v>Already satisfied by #1064 (commit 4f9074a): Windows CI sets up trusted fast-tools (sccache) in RUNNER_TEMP outside the PR workspace, hash-verifies the sccache archive unconditionally (a pre-existing workspace sccache.exe cannot short-circuit it) and invokes it by verified absolute path; the vcpkg installed tree is validated/reinstalled when the cache is incomplete and the cache key includes dependency-defining inputs. Reconciling stale NOT_STARTED row to DONE.</x:v>
+      </x:c>
+      <x:c r="AB25" s="39" t="str">
+        <x:v>python3 -m unittest tests.security.test_configure_supply_chain -&gt; Ran 15 tests, OK (tools outside workspace, unconditional sccache hash verify, vcpkg cache validation + dependency-input cache key, pinned action SHAs).</x:v>
+      </x:c>
       <x:c r="AC25" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Reconcile #673 to DONE (satisfied by #1064) (#1263)
EPIC_02/STORY_02/SUBSTORY_01 #673 'Harden Windows CI tool and vcpkg cache
validation': stale NOT_STARTED row reconciled to DONE. Hardening landed in
commit 4f9074a (#1064); tests.security.test_configure_supply_chain passes
(15 tests: trusted tools outside workspace, unconditional sccache hash
verification, vcpkg installed-cache validation + dependency-input cache key).
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -6134,27 +6134,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/vcpkg triplets/manifests</x:v>
       </x:c>
       <x:c r="Q25" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R25" s="39"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R25" s="39" t="str">
+        <x:v>ctrl-vm-2256-06ac44fc</x:v>
+      </x:c>
       <x:c r="S25" s="39"/>
-      <x:c r="T25" s="39"/>
-      <x:c r="U25" s="39"/>
+      <x:c r="T25" s="39" t="str">
+        <x:v>9f2d6cae-5763-4e1a-897b-24bfcc42c8a1</x:v>
+      </x:c>
+      <x:c r="U25" s="39" t="str">
+        <x:v>2026-07-02T07:49:14Z</x:v>
+      </x:c>
       <x:c r="V25" s="39" t="str">
-        <x:v>2026-07-01T20:17:34Z</x:v>
+        <x:v>2026-07-02T07:49:14Z</x:v>
       </x:c>
       <x:c r="W25" s="39"/>
-      <x:c r="X25" s="39"/>
+      <x:c r="X25" s="39" t="str">
+        <x:v>2026-07-02T07:49:14Z</x:v>
+      </x:c>
       <x:c r="Y25" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z25" s="39" t="str">
-        <x:v>Stale claim reclaimed from controller/ctrl-vm-4024-7534d796/subagent-11; prior claim ff73ecb2-7600-431d-92ba-da44273f9606</x:v>
-      </x:c>
-      <x:c r="AA25" s="39"/>
-      <x:c r="AB25" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA25" s="39" t="str">
+        <x:v>Already satisfied by #1064 (commit 4f9074a): Windows CI sets up trusted fast-tools (sccache) in RUNNER_TEMP outside the PR workspace, hash-verifies the sccache archive unconditionally (a pre-existing workspace sccache.exe cannot short-circuit it) and invokes it by verified absolute path; the vcpkg installed tree is validated/reinstalled when the cache is incomplete and the cache key includes dependency-defining inputs. Reconciling stale NOT_STARTED row to DONE.</x:v>
+      </x:c>
+      <x:c r="AB25" s="39" t="str">
+        <x:v>python3 -m unittest tests.security.test_configure_supply_chain -&gt; Ran 15 tests, OK (tools outside workspace, unconditional sccache hash verify, vcpkg cache validation + dependency-input cache key, pinned action SHAs).</x:v>
+      </x:c>
       <x:c r="AC25" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim s37 #627 drag-and-drop semantics (migrated workbook)
Refill slot 1/4: [EPIC_03][STORY_01][SUBSTORY_03] #627 Correct inventory and
equipment drag-and-drop semantics. Deps #625/#626 are DONE. Owner
controller/ctrl-vm-4039-a70f65a5/subagent-37. Queue-workbook change only.
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5226,25 +5226,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q15" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R15" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R15" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
+      </x:c>
       <x:c r="S15" s="39"/>
-      <x:c r="T15" s="39"/>
-      <x:c r="U15" s="39"/>
-      <x:c r="V15" s="39"/>
-      <x:c r="W15" s="39"/>
+      <x:c r="T15" s="39" t="str">
+        <x:v>9af78786-65ba-4911-99cb-a06a32157a02</x:v>
+      </x:c>
+      <x:c r="U15" s="39" t="str">
+        <x:v>2026-07-02T10:15:14Z</x:v>
+      </x:c>
+      <x:c r="V15" s="39" t="str">
+        <x:v>2026-07-02T10:15:14Z</x:v>
+      </x:c>
+      <x:c r="W15" s="39" t="str">
+        <x:v>2026-07-02T14:15:14Z</x:v>
+      </x:c>
       <x:c r="X15" s="39"/>
       <x:c r="Y15" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z15" s="39" t="str">
-        <x:v>Migrated from GitHub issue #627; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
       </x:c>
       <x:c r="AA15" s="39"/>
       <x:c r="AB15" s="39"/>
       <x:c r="AC15" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim s37 #627 drag-and-drop semantics (migrated workbook) (#1266)
Refill slot 1/4: [EPIC_03][STORY_01][SUBSTORY_03] #627 Correct inventory and
equipment drag-and-drop semantics. Deps #625/#626 are DONE. Owner
controller/ctrl-vm-4039-a70f65a5/subagent-37. Queue-workbook change only.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5226,25 +5226,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q15" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R15" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R15" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
+      </x:c>
       <x:c r="S15" s="39"/>
-      <x:c r="T15" s="39"/>
-      <x:c r="U15" s="39"/>
-      <x:c r="V15" s="39"/>
-      <x:c r="W15" s="39"/>
+      <x:c r="T15" s="39" t="str">
+        <x:v>9af78786-65ba-4911-99cb-a06a32157a02</x:v>
+      </x:c>
+      <x:c r="U15" s="39" t="str">
+        <x:v>2026-07-02T10:15:14Z</x:v>
+      </x:c>
+      <x:c r="V15" s="39" t="str">
+        <x:v>2026-07-02T10:15:14Z</x:v>
+      </x:c>
+      <x:c r="W15" s="39" t="str">
+        <x:v>2026-07-02T14:15:14Z</x:v>
+      </x:c>
       <x:c r="X15" s="39"/>
       <x:c r="Y15" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z15" s="39" t="str">
-        <x:v>Migrated from GitHub issue #627; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
       </x:c>
       <x:c r="AA15" s="39"/>
       <x:c r="AB15" s="39"/>
       <x:c r="AC15" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #615 write-lease separation (migrated workbook, ctrl-vm-4027)
Workbook-only IN_PROGRESS claim for [EPIC_01][STORY_01][SUBSTORY_02] #615
by controller/ctrl-vm-4027-c0afa077/subagent-1.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4246,25 +4246,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q3" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R3" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R3" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
+      </x:c>
       <x:c r="S3" s="39"/>
-      <x:c r="T3" s="39"/>
-      <x:c r="U3" s="39"/>
-      <x:c r="V3" s="39"/>
-      <x:c r="W3" s="39"/>
+      <x:c r="T3" s="39" t="str">
+        <x:v>defd0016-bfb4-4d45-a574-496d5bf2992c</x:v>
+      </x:c>
+      <x:c r="U3" s="39" t="str">
+        <x:v>2026-07-02T11:49:02Z</x:v>
+      </x:c>
+      <x:c r="V3" s="39" t="str">
+        <x:v>2026-07-02T11:49:02Z</x:v>
+      </x:c>
+      <x:c r="W3" s="39" t="str">
+        <x:v>2026-07-02T13:49:02Z</x:v>
+      </x:c>
       <x:c r="X3" s="39"/>
       <x:c r="Y3" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z3" s="39" t="str">
-        <x:v>Migrated from GitHub issue #615; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
       </x:c>
       <x:c r="AA3" s="39"/>
       <x:c r="AB3" s="39"/>
       <x:c r="AC3" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #615 write-lease separation (migrated workbook, ctrl-vm-4027) (#1273)
Workbook-only IN_PROGRESS claim for [EPIC_01][STORY_01][SUBSTORY_02] #615
by controller/ctrl-vm-4027-c0afa077/subagent-1.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4246,25 +4246,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q3" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R3" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R3" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
+      </x:c>
       <x:c r="S3" s="39"/>
-      <x:c r="T3" s="39"/>
-      <x:c r="U3" s="39"/>
-      <x:c r="V3" s="39"/>
-      <x:c r="W3" s="39"/>
+      <x:c r="T3" s="39" t="str">
+        <x:v>defd0016-bfb4-4d45-a574-496d5bf2992c</x:v>
+      </x:c>
+      <x:c r="U3" s="39" t="str">
+        <x:v>2026-07-02T11:49:02Z</x:v>
+      </x:c>
+      <x:c r="V3" s="39" t="str">
+        <x:v>2026-07-02T11:49:02Z</x:v>
+      </x:c>
+      <x:c r="W3" s="39" t="str">
+        <x:v>2026-07-02T13:49:02Z</x:v>
+      </x:c>
       <x:c r="X3" s="39"/>
       <x:c r="Y3" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z3" s="39" t="str">
-        <x:v>Migrated from GitHub issue #615; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
       </x:c>
       <x:c r="AA3" s="39"/>
       <x:c r="AB3" s="39"/>
       <x:c r="AC3" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #624 PR-audit stale-attempt dedupe (migrated workbook, ctrl-vm-4027)
Workbook-only IN_PROGRESS claim for [EPIC_01][STORY_04][SUBSTORY_02] #624
by controller/ctrl-vm-4027-c0afa077/subagent-3.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4969,25 +4969,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/GitHub snapshot builder/controller guidance</x:v>
       </x:c>
       <x:c r="Q12" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R12" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R12" s="36" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
+      </x:c>
       <x:c r="S12" s="36"/>
-      <x:c r="T12" s="36"/>
-      <x:c r="U12" s="36"/>
-      <x:c r="V12" s="36"/>
-      <x:c r="W12" s="36"/>
+      <x:c r="T12" s="36" t="str">
+        <x:v>36ce0bab-d2a3-4d86-86df-029511667f2c</x:v>
+      </x:c>
+      <x:c r="U12" s="36" t="str">
+        <x:v>2026-07-02T12:03:02Z</x:v>
+      </x:c>
+      <x:c r="V12" s="36" t="str">
+        <x:v>2026-07-02T12:03:02Z</x:v>
+      </x:c>
+      <x:c r="W12" s="36" t="str">
+        <x:v>2026-07-02T14:03:02Z</x:v>
+      </x:c>
       <x:c r="X12" s="36"/>
       <x:c r="Y12" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z12" s="36" t="str">
-        <x:v>Migrated from GitHub issue #624; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
       </x:c>
       <x:c r="AA12" s="36"/>
       <x:c r="AB12" s="36"/>
       <x:c r="AC12" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #624 PR-audit stale-attempt dedupe (migrated workbook, ctrl-vm-4027) (#1276)
Workbook-only IN_PROGRESS claim for [EPIC_01][STORY_04][SUBSTORY_02] #624
by controller/ctrl-vm-4027-c0afa077/subagent-3.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4969,25 +4969,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/GitHub snapshot builder/controller guidance</x:v>
       </x:c>
       <x:c r="Q12" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R12" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R12" s="36" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
+      </x:c>
       <x:c r="S12" s="36"/>
-      <x:c r="T12" s="36"/>
-      <x:c r="U12" s="36"/>
-      <x:c r="V12" s="36"/>
-      <x:c r="W12" s="36"/>
+      <x:c r="T12" s="36" t="str">
+        <x:v>36ce0bab-d2a3-4d86-86df-029511667f2c</x:v>
+      </x:c>
+      <x:c r="U12" s="36" t="str">
+        <x:v>2026-07-02T12:03:02Z</x:v>
+      </x:c>
+      <x:c r="V12" s="36" t="str">
+        <x:v>2026-07-02T12:03:02Z</x:v>
+      </x:c>
+      <x:c r="W12" s="36" t="str">
+        <x:v>2026-07-02T14:03:02Z</x:v>
+      </x:c>
       <x:c r="X12" s="36"/>
       <x:c r="Y12" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z12" s="36" t="str">
-        <x:v>Migrated from GitHub issue #624; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
       </x:c>
       <x:c r="AA12" s="36"/>
       <x:c r="AB12" s="36"/>
       <x:c r="AC12" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #616 subagent lifecycle registry (migrated workbook, ctrl-vm-4027)
Workbook-only IN_PROGRESS claim for [EPIC_01][STORY_02][SUBSTORY_01] #616
by controller/ctrl-vm-4027-c0afa077/subagent-4.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4335,25 +4335,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q4" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R4" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R4" s="36" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
+      </x:c>
       <x:c r="S4" s="36"/>
-      <x:c r="T4" s="36"/>
-      <x:c r="U4" s="36"/>
-      <x:c r="V4" s="36"/>
-      <x:c r="W4" s="36"/>
+      <x:c r="T4" s="36" t="str">
+        <x:v>880b1760-0eb6-4f45-b1a4-016d14b2ea37</x:v>
+      </x:c>
+      <x:c r="U4" s="36" t="str">
+        <x:v>2026-07-02T12:06:09Z</x:v>
+      </x:c>
+      <x:c r="V4" s="36" t="str">
+        <x:v>2026-07-02T12:06:09Z</x:v>
+      </x:c>
+      <x:c r="W4" s="36" t="str">
+        <x:v>2026-07-02T14:06:09Z</x:v>
+      </x:c>
       <x:c r="X4" s="36"/>
       <x:c r="Y4" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>Migrated from GitHub issue #616; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
       </x:c>
       <x:c r="AA4" s="36"/>
       <x:c r="AB4" s="36"/>
       <x:c r="AC4" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #616 subagent lifecycle registry (migrated workbook, ctrl-vm-4027) (#1278)
Workbook-only IN_PROGRESS claim for [EPIC_01][STORY_02][SUBSTORY_01] #616
by controller/ctrl-vm-4027-c0afa077/subagent-4.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4335,25 +4335,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q4" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R4" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R4" s="36" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
+      </x:c>
       <x:c r="S4" s="36"/>
-      <x:c r="T4" s="36"/>
-      <x:c r="U4" s="36"/>
-      <x:c r="V4" s="36"/>
-      <x:c r="W4" s="36"/>
+      <x:c r="T4" s="36" t="str">
+        <x:v>880b1760-0eb6-4f45-b1a4-016d14b2ea37</x:v>
+      </x:c>
+      <x:c r="U4" s="36" t="str">
+        <x:v>2026-07-02T12:06:09Z</x:v>
+      </x:c>
+      <x:c r="V4" s="36" t="str">
+        <x:v>2026-07-02T12:06:09Z</x:v>
+      </x:c>
+      <x:c r="W4" s="36" t="str">
+        <x:v>2026-07-02T14:06:09Z</x:v>
+      </x:c>
       <x:c r="X4" s="36"/>
       <x:c r="Y4" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>Migrated from GitHub issue #616; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
       </x:c>
       <x:c r="AA4" s="36"/>
       <x:c r="AB4" s="36"/>
       <x:c r="AC4" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Heartbeat s37 #627 (lease extended; PR #1272 blocked on red main)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5269,17 +5269,17 @@
         <x:v>2026-07-02T10:15:14Z</x:v>
       </x:c>
       <x:c r="V15" s="39" t="str">
-        <x:v>2026-07-02T10:15:14Z</x:v>
+        <x:v>2026-07-02T12:28:50Z</x:v>
       </x:c>
       <x:c r="W15" s="39" t="str">
-        <x:v>2026-07-02T14:15:14Z</x:v>
+        <x:v>2026-07-02T16:28:50Z</x:v>
       </x:c>
       <x:c r="X15" s="39"/>
       <x:c r="Y15" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z15" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
+        <x:v>impl complete; PR #1272 open, blocked by fleet-wide red main (ninemarches/sunderedmarch walkthroughs + SIGABRT teardown); merge on main recovery</x:v>
       </x:c>
       <x:c r="AA15" s="39"/>
       <x:c r="AB15" s="39"/>

</xml_diff>

<commit_message>
Heartbeat s37 #627 (lease extended; PR #1272 blocked on red main) (#1282)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5269,17 +5269,17 @@
         <x:v>2026-07-02T10:15:14Z</x:v>
       </x:c>
       <x:c r="V15" s="39" t="str">
-        <x:v>2026-07-02T10:15:14Z</x:v>
+        <x:v>2026-07-02T12:28:50Z</x:v>
       </x:c>
       <x:c r="W15" s="39" t="str">
-        <x:v>2026-07-02T14:15:14Z</x:v>
+        <x:v>2026-07-02T16:28:50Z</x:v>
       </x:c>
       <x:c r="X15" s="39"/>
       <x:c r="Y15" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z15" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
+        <x:v>impl complete; PR #1272 open, blocked by fleet-wide red main (ninemarches/sunderedmarch walkthroughs + SIGABRT teardown); merge on main recovery</x:v>
       </x:c>
       <x:c r="AA15" s="39"/>
       <x:c r="AB15" s="39"/>

</xml_diff>

<commit_message>
Heartbeat #615 claim: PR #1277 open (ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4259,17 +4259,17 @@
         <x:v>2026-07-02T11:49:02Z</x:v>
       </x:c>
       <x:c r="V3" s="39" t="str">
-        <x:v>2026-07-02T11:49:02Z</x:v>
+        <x:v>2026-07-02T12:57:38Z</x:v>
       </x:c>
       <x:c r="W3" s="39" t="str">
-        <x:v>2026-07-02T13:49:02Z</x:v>
+        <x:v>2026-07-02T14:57:38Z</x:v>
       </x:c>
       <x:c r="X3" s="39"/>
       <x:c r="Y3" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z3" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
+        <x:v>Implementation complete; PR #1277 open, awaiting green CI after main fix #1274 merges</x:v>
       </x:c>
       <x:c r="AA3" s="39"/>
       <x:c r="AB3" s="39"/>

</xml_diff>

<commit_message>
Heartbeat #615 claim: PR #1277 open (ctrl-vm-4027) (#1284)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4259,17 +4259,17 @@
         <x:v>2026-07-02T11:49:02Z</x:v>
       </x:c>
       <x:c r="V3" s="39" t="str">
-        <x:v>2026-07-02T11:49:02Z</x:v>
+        <x:v>2026-07-02T12:57:38Z</x:v>
       </x:c>
       <x:c r="W3" s="39" t="str">
-        <x:v>2026-07-02T13:49:02Z</x:v>
+        <x:v>2026-07-02T14:57:38Z</x:v>
       </x:c>
       <x:c r="X3" s="39"/>
       <x:c r="Y3" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z3" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
+        <x:v>Implementation complete; PR #1277 open, awaiting green CI after main fix #1274 merges</x:v>
       </x:c>
       <x:c r="AA3" s="39"/>
       <x:c r="AB3" s="39"/>

</xml_diff>

<commit_message>
Heartbeat #624 claim: PR #1279 open (ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4992,17 +4992,17 @@
         <x:v>2026-07-02T12:03:02Z</x:v>
       </x:c>
       <x:c r="V12" s="36" t="str">
-        <x:v>2026-07-02T12:03:02Z</x:v>
+        <x:v>2026-07-02T12:59:01Z</x:v>
       </x:c>
       <x:c r="W12" s="36" t="str">
-        <x:v>2026-07-02T14:03:02Z</x:v>
+        <x:v>2026-07-02T14:59:01Z</x:v>
       </x:c>
       <x:c r="X12" s="36"/>
       <x:c r="Y12" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z12" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
+        <x:v>Implementation complete; PR #1279 open, awaiting green CI after main fix #1274 merges</x:v>
       </x:c>
       <x:c r="AA12" s="36"/>
       <x:c r="AB12" s="36"/>

</xml_diff>

<commit_message>
Heartbeat #624 claim: PR #1279 open (ctrl-vm-4027) (#1286)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4992,17 +4992,17 @@
         <x:v>2026-07-02T12:03:02Z</x:v>
       </x:c>
       <x:c r="V12" s="36" t="str">
-        <x:v>2026-07-02T12:03:02Z</x:v>
+        <x:v>2026-07-02T12:59:01Z</x:v>
       </x:c>
       <x:c r="W12" s="36" t="str">
-        <x:v>2026-07-02T14:03:02Z</x:v>
+        <x:v>2026-07-02T14:59:01Z</x:v>
       </x:c>
       <x:c r="X12" s="36"/>
       <x:c r="Y12" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z12" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
+        <x:v>Implementation complete; PR #1279 open, awaiting green CI after main fix #1274 merges</x:v>
       </x:c>
       <x:c r="AA12" s="36"/>
       <x:c r="AB12" s="36"/>

</xml_diff>

<commit_message>
Heartbeat #616 claim: PR #1280 open (ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4348,17 +4348,17 @@
         <x:v>2026-07-02T12:06:09Z</x:v>
       </x:c>
       <x:c r="V4" s="36" t="str">
-        <x:v>2026-07-02T12:06:09Z</x:v>
+        <x:v>2026-07-02T12:59:44Z</x:v>
       </x:c>
       <x:c r="W4" s="36" t="str">
-        <x:v>2026-07-02T14:06:09Z</x:v>
+        <x:v>2026-07-02T14:59:44Z</x:v>
       </x:c>
       <x:c r="X4" s="36"/>
       <x:c r="Y4" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
+        <x:v>Implementation complete; PR #1280 open, awaiting green CI after main fix #1274 merges</x:v>
       </x:c>
       <x:c r="AA4" s="36"/>
       <x:c r="AB4" s="36"/>

</xml_diff>

<commit_message>
Heartbeat #616 claim: PR #1280 open (ctrl-vm-4027) (#1287)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4348,17 +4348,17 @@
         <x:v>2026-07-02T12:06:09Z</x:v>
       </x:c>
       <x:c r="V4" s="36" t="str">
-        <x:v>2026-07-02T12:06:09Z</x:v>
+        <x:v>2026-07-02T12:59:44Z</x:v>
       </x:c>
       <x:c r="W4" s="36" t="str">
-        <x:v>2026-07-02T14:06:09Z</x:v>
+        <x:v>2026-07-02T14:59:44Z</x:v>
       </x:c>
       <x:c r="X4" s="36"/>
       <x:c r="Y4" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
+        <x:v>Implementation complete; PR #1280 open, awaiting green CI after main fix #1274 merges</x:v>
       </x:c>
       <x:c r="AA4" s="36"/>
       <x:c r="AB4" s="36"/>

</xml_diff>

<commit_message>
Mark #624 DONE (PR #1279 merged, ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4979,7 +4979,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/GitHub snapshot builder/controller guidance</x:v>
       </x:c>
       <x:c r="Q12" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R12" s="36" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
@@ -4992,20 +4992,24 @@
         <x:v>2026-07-02T12:03:02Z</x:v>
       </x:c>
       <x:c r="V12" s="36" t="str">
-        <x:v>2026-07-02T12:59:01Z</x:v>
-      </x:c>
-      <x:c r="W12" s="36" t="str">
-        <x:v>2026-07-02T14:59:01Z</x:v>
-      </x:c>
-      <x:c r="X12" s="36"/>
+        <x:v>2026-07-02T14:34:30Z</x:v>
+      </x:c>
+      <x:c r="W12" s="36"/>
+      <x:c r="X12" s="36" t="str">
+        <x:v>2026-07-02T14:34:30Z</x:v>
+      </x:c>
       <x:c r="Y12" s="36" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z12" s="36" t="str">
-        <x:v>Implementation complete; PR #1279 open, awaiting green CI after main fix #1274 merges</x:v>
-      </x:c>
-      <x:c r="AA12" s="36"/>
-      <x:c r="AB12" s="36"/>
+        <x:v>DONE via PR #1279</x:v>
+      </x:c>
+      <x:c r="AA12" s="36" t="str">
+        <x:v>Merged PR #1279 (squash 9a11bd3). pr_review_audit now normalizes checks with (kind, app, workflow, name) identity, deterministic timestamp/attempt/run-id ordering, conservative ambiguity flagging, and additive ignoredStale/ambiguous output; summaries derive from effective attempts only.</x:v>
+      </x:c>
+      <x:c r="AB12" s="36" t="str">
+        <x:v>python3 -m unittest tests.test_pr_review_audit (41 OK); tests.test_poll_pr_checks (39 OK); py_compile; test.py --suite fast (9 OK); black --check clean; PR #1279 CI linux green (lightweight class)</x:v>
+      </x:c>
       <x:c r="AC12" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #624 DONE (PR #1279 merged, ctrl-vm-4027) (#1290)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4979,7 +4979,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/GitHub snapshot builder/controller guidance</x:v>
       </x:c>
       <x:c r="Q12" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R12" s="36" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-3</x:v>
@@ -4992,20 +4992,24 @@
         <x:v>2026-07-02T12:03:02Z</x:v>
       </x:c>
       <x:c r="V12" s="36" t="str">
-        <x:v>2026-07-02T12:59:01Z</x:v>
-      </x:c>
-      <x:c r="W12" s="36" t="str">
-        <x:v>2026-07-02T14:59:01Z</x:v>
-      </x:c>
-      <x:c r="X12" s="36"/>
+        <x:v>2026-07-02T14:34:30Z</x:v>
+      </x:c>
+      <x:c r="W12" s="36"/>
+      <x:c r="X12" s="36" t="str">
+        <x:v>2026-07-02T14:34:30Z</x:v>
+      </x:c>
       <x:c r="Y12" s="36" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z12" s="36" t="str">
-        <x:v>Implementation complete; PR #1279 open, awaiting green CI after main fix #1274 merges</x:v>
-      </x:c>
-      <x:c r="AA12" s="36"/>
-      <x:c r="AB12" s="36"/>
+        <x:v>DONE via PR #1279</x:v>
+      </x:c>
+      <x:c r="AA12" s="36" t="str">
+        <x:v>Merged PR #1279 (squash 9a11bd3). pr_review_audit now normalizes checks with (kind, app, workflow, name) identity, deterministic timestamp/attempt/run-id ordering, conservative ambiguity flagging, and additive ignoredStale/ambiguous output; summaries derive from effective attempts only.</x:v>
+      </x:c>
+      <x:c r="AB12" s="36" t="str">
+        <x:v>python3 -m unittest tests.test_pr_review_audit (41 OK); tests.test_poll_pr_checks (39 OK); py_compile; test.py --suite fast (9 OK); black --check clean; PR #1279 CI linux green (lightweight class)</x:v>
+      </x:c>
       <x:c r="AC12" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark s37 #627 DONE (PR #1272 merged)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5260,7 +5260,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q15" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R15" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
@@ -5273,20 +5273,24 @@
         <x:v>2026-07-02T10:15:14Z</x:v>
       </x:c>
       <x:c r="V15" s="39" t="str">
-        <x:v>2026-07-02T12:28:50Z</x:v>
-      </x:c>
-      <x:c r="W15" s="39" t="str">
-        <x:v>2026-07-02T16:28:50Z</x:v>
-      </x:c>
-      <x:c r="X15" s="39"/>
+        <x:v>2026-07-02T15:18:19Z</x:v>
+      </x:c>
+      <x:c r="W15" s="39"/>
+      <x:c r="X15" s="39" t="str">
+        <x:v>2026-07-02T15:18:19Z</x:v>
+      </x:c>
       <x:c r="Y15" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z15" s="39" t="str">
-        <x:v>impl complete; PR #1272 open, blocked by fleet-wide red main (ninemarches/sunderedmarch walkthroughs + SIGABRT teardown); merge on main recovery</x:v>
-      </x:c>
-      <x:c r="AA15" s="39"/>
-      <x:c r="AB15" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA15" s="39" t="str">
+        <x:v>Merged in PR #1272: payload-only drop semantics in CListView (removed legacy click-callback fallback on moved cross-list drops); exact dragged item equips; quest/incompatible/same-list/cancel paths inert; +6 tests in test_gui.cpp.</x:v>
+      </x:c>
+      <x:c r="AB15" s="39" t="str">
+        <x:v>CI green on merge.</x:v>
+      </x:c>
       <x:c r="AC15" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark s37 #627 DONE (PR #1272 merged) (#1293)
Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5260,7 +5260,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/src/gui/CGui.cpp</x:v>
       </x:c>
       <x:c r="Q15" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R15" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-37</x:v>
@@ -5273,20 +5273,24 @@
         <x:v>2026-07-02T10:15:14Z</x:v>
       </x:c>
       <x:c r="V15" s="39" t="str">
-        <x:v>2026-07-02T12:28:50Z</x:v>
-      </x:c>
-      <x:c r="W15" s="39" t="str">
-        <x:v>2026-07-02T16:28:50Z</x:v>
-      </x:c>
-      <x:c r="X15" s="39"/>
+        <x:v>2026-07-02T15:18:19Z</x:v>
+      </x:c>
+      <x:c r="W15" s="39"/>
+      <x:c r="X15" s="39" t="str">
+        <x:v>2026-07-02T15:18:19Z</x:v>
+      </x:c>
       <x:c r="Y15" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z15" s="39" t="str">
-        <x:v>impl complete; PR #1272 open, blocked by fleet-wide red main (ninemarches/sunderedmarch walkthroughs + SIGABRT teardown); merge on main recovery</x:v>
-      </x:c>
-      <x:c r="AA15" s="39"/>
-      <x:c r="AB15" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA15" s="39" t="str">
+        <x:v>Merged in PR #1272: payload-only drop semantics in CListView (removed legacy click-callback fallback on moved cross-list drops); exact dragged item equips; quest/incompatible/same-list/cancel paths inert; +6 tests in test_gui.cpp.</x:v>
+      </x:c>
+      <x:c r="AB15" s="39" t="str">
+        <x:v>CI green on merge.</x:v>
+      </x:c>
       <x:c r="AC15" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #615 DONE (PR #1277 merged, ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4246,7 +4246,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q3" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R3" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
@@ -4259,20 +4259,24 @@
         <x:v>2026-07-02T11:49:02Z</x:v>
       </x:c>
       <x:c r="V3" s="39" t="str">
-        <x:v>2026-07-02T12:57:38Z</x:v>
-      </x:c>
-      <x:c r="W3" s="39" t="str">
-        <x:v>2026-07-02T14:57:38Z</x:v>
-      </x:c>
-      <x:c r="X3" s="39"/>
+        <x:v>2026-07-02T15:25:01Z</x:v>
+      </x:c>
+      <x:c r="W3" s="39"/>
+      <x:c r="X3" s="39" t="str">
+        <x:v>2026-07-02T15:25:01Z</x:v>
+      </x:c>
       <x:c r="Y3" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z3" s="39" t="str">
-        <x:v>Implementation complete; PR #1277 open, awaiting green CI after main fix #1274 merges</x:v>
-      </x:c>
-      <x:c r="AA3" s="39"/>
-      <x:c r="AB3" s="39"/>
+        <x:v>DONE via PR #1277</x:v>
+      </x:c>
+      <x:c r="AA3" s="39" t="str">
+        <x:v>Merged PR #1277 (squash 5c16a5d). Adds scripts/write_leases.py: JSON write-lease store separate from XLSX claims with acquire/renew/release/recover/list/validate, atomic all-or-nothing batches under a sidecar lock, confidence-ranked scope normalization and deterministic coupled-area expansion; conflicting ACTIVE scopes cannot both write; recovery is lease-lifecycle-only. Docs sections added; 27 tests.</x:v>
+      </x:c>
+      <x:c r="AB3" s="39" t="str">
+        <x:v>tests.test_write_leases (27 OK); tests.test_issue_queue (45 OK); doc-guard suites (58 OK); queue validates clean; PR #1277 CI green (linux, windows-deps, windows)</x:v>
+      </x:c>
       <x:c r="AC3" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #615 DONE (PR #1277 merged, ctrl-vm-4027) (#1295)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4246,7 +4246,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q3" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R3" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-1</x:v>
@@ -4259,20 +4259,24 @@
         <x:v>2026-07-02T11:49:02Z</x:v>
       </x:c>
       <x:c r="V3" s="39" t="str">
-        <x:v>2026-07-02T12:57:38Z</x:v>
-      </x:c>
-      <x:c r="W3" s="39" t="str">
-        <x:v>2026-07-02T14:57:38Z</x:v>
-      </x:c>
-      <x:c r="X3" s="39"/>
+        <x:v>2026-07-02T15:25:01Z</x:v>
+      </x:c>
+      <x:c r="W3" s="39"/>
+      <x:c r="X3" s="39" t="str">
+        <x:v>2026-07-02T15:25:01Z</x:v>
+      </x:c>
       <x:c r="Y3" s="39" t="n">
-        <x:v>90</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z3" s="39" t="str">
-        <x:v>Implementation complete; PR #1277 open, awaiting green CI after main fix #1274 merges</x:v>
-      </x:c>
-      <x:c r="AA3" s="39"/>
-      <x:c r="AB3" s="39"/>
+        <x:v>DONE via PR #1277</x:v>
+      </x:c>
+      <x:c r="AA3" s="39" t="str">
+        <x:v>Merged PR #1277 (squash 5c16a5d). Adds scripts/write_leases.py: JSON write-lease store separate from XLSX claims with acquire/renew/release/recover/list/validate, atomic all-or-nothing batches under a sidecar lock, confidence-ranked scope normalization and deterministic coupled-area expansion; conflicting ACTIVE scopes cannot both write; recovery is lease-lifecycle-only. Docs sections added; 27 tests.</x:v>
+      </x:c>
+      <x:c r="AB3" s="39" t="str">
+        <x:v>tests.test_write_leases (27 OK); tests.test_issue_queue (45 OK); doc-guard suites (58 OK); queue validates clean; PR #1277 CI green (linux, windows-deps, windows)</x:v>
+      </x:c>
       <x:c r="AC3" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Heartbeat #616 claim: PR #1280 revalidating (ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4352,17 +4352,17 @@
         <x:v>2026-07-02T12:06:09Z</x:v>
       </x:c>
       <x:c r="V4" s="36" t="str">
-        <x:v>2026-07-02T12:59:44Z</x:v>
+        <x:v>2026-07-02T15:26:03Z</x:v>
       </x:c>
       <x:c r="W4" s="36" t="str">
-        <x:v>2026-07-02T14:59:44Z</x:v>
+        <x:v>2026-07-02T17:26:03Z</x:v>
       </x:c>
       <x:c r="X4" s="36"/>
       <x:c r="Y4" s="36" t="n">
-        <x:v>90</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>Implementation complete; PR #1280 open, awaiting green CI after main fix #1274 merges</x:v>
+        <x:v>PR #1280 green on prior head; revalidating after #1277 merge, completion imminent</x:v>
       </x:c>
       <x:c r="AA4" s="36"/>
       <x:c r="AB4" s="36"/>

</xml_diff>

<commit_message>
Heartbeat #616 claim: PR #1280 revalidating (ctrl-vm-4027) (#1296)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4352,17 +4352,17 @@
         <x:v>2026-07-02T12:06:09Z</x:v>
       </x:c>
       <x:c r="V4" s="36" t="str">
-        <x:v>2026-07-02T12:59:44Z</x:v>
+        <x:v>2026-07-02T15:26:03Z</x:v>
       </x:c>
       <x:c r="W4" s="36" t="str">
-        <x:v>2026-07-02T14:59:44Z</x:v>
+        <x:v>2026-07-02T17:26:03Z</x:v>
       </x:c>
       <x:c r="X4" s="36"/>
       <x:c r="Y4" s="36" t="n">
-        <x:v>90</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>Implementation complete; PR #1280 open, awaiting green CI after main fix #1274 merges</x:v>
+        <x:v>PR #1280 green on prior head; revalidating after #1277 merge, completion imminent</x:v>
       </x:c>
       <x:c r="AA4" s="36"/>
       <x:c r="AB4" s="36"/>

</xml_diff>

<commit_message>
Claim #617 shared resource broker (migrated workbook, ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4427,25 +4427,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q5" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R5" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R5" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
+      </x:c>
       <x:c r="S5" s="39"/>
-      <x:c r="T5" s="39"/>
-      <x:c r="U5" s="39"/>
-      <x:c r="V5" s="39"/>
-      <x:c r="W5" s="39"/>
+      <x:c r="T5" s="39" t="str">
+        <x:v>846a39f7-c64a-4415-a598-be35926f2616</x:v>
+      </x:c>
+      <x:c r="U5" s="39" t="str">
+        <x:v>2026-07-02T15:26:43Z</x:v>
+      </x:c>
+      <x:c r="V5" s="39" t="str">
+        <x:v>2026-07-02T15:26:43Z</x:v>
+      </x:c>
+      <x:c r="W5" s="39" t="str">
+        <x:v>2026-07-02T17:26:43Z</x:v>
+      </x:c>
       <x:c r="X5" s="39"/>
       <x:c r="Y5" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z5" s="39" t="str">
-        <x:v>Migrated from GitHub issue #617; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
       </x:c>
       <x:c r="AA5" s="39"/>
       <x:c r="AB5" s="39"/>
       <x:c r="AC5" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #617 shared resource broker (migrated workbook, ctrl-vm-4027) (#1298)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4427,25 +4427,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q5" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R5" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R5" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
+      </x:c>
       <x:c r="S5" s="39"/>
-      <x:c r="T5" s="39"/>
-      <x:c r="U5" s="39"/>
-      <x:c r="V5" s="39"/>
-      <x:c r="W5" s="39"/>
+      <x:c r="T5" s="39" t="str">
+        <x:v>846a39f7-c64a-4415-a598-be35926f2616</x:v>
+      </x:c>
+      <x:c r="U5" s="39" t="str">
+        <x:v>2026-07-02T15:26:43Z</x:v>
+      </x:c>
+      <x:c r="V5" s="39" t="str">
+        <x:v>2026-07-02T15:26:43Z</x:v>
+      </x:c>
+      <x:c r="W5" s="39" t="str">
+        <x:v>2026-07-02T17:26:43Z</x:v>
+      </x:c>
       <x:c r="X5" s="39"/>
       <x:c r="Y5" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z5" s="39" t="str">
-        <x:v>Migrated from GitHub issue #617; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
       </x:c>
       <x:c r="AA5" s="39"/>
       <x:c r="AB5" s="39"/>
       <x:c r="AC5" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #619 controller capability probe (migrated workbook, ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4597,25 +4597,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q7" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R7" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R7" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
+      </x:c>
       <x:c r="S7" s="39"/>
-      <x:c r="T7" s="39"/>
-      <x:c r="U7" s="39"/>
-      <x:c r="V7" s="39"/>
-      <x:c r="W7" s="39"/>
+      <x:c r="T7" s="39" t="str">
+        <x:v>b10fbae1-9510-4bf1-9c8b-6e49e658b0e8</x:v>
+      </x:c>
+      <x:c r="U7" s="39" t="str">
+        <x:v>2026-07-02T15:27:34Z</x:v>
+      </x:c>
+      <x:c r="V7" s="39" t="str">
+        <x:v>2026-07-02T15:27:34Z</x:v>
+      </x:c>
+      <x:c r="W7" s="39" t="str">
+        <x:v>2026-07-02T17:27:34Z</x:v>
+      </x:c>
       <x:c r="X7" s="39"/>
       <x:c r="Y7" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z7" s="39" t="str">
-        <x:v>Migrated from GitHub issue #619; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
       </x:c>
       <x:c r="AA7" s="39"/>
       <x:c r="AB7" s="39"/>
       <x:c r="AC7" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #619 controller capability probe (migrated workbook, ctrl-vm-4027) (#1299)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4597,25 +4597,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q7" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R7" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R7" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
+      </x:c>
       <x:c r="S7" s="39"/>
-      <x:c r="T7" s="39"/>
-      <x:c r="U7" s="39"/>
-      <x:c r="V7" s="39"/>
-      <x:c r="W7" s="39"/>
+      <x:c r="T7" s="39" t="str">
+        <x:v>b10fbae1-9510-4bf1-9c8b-6e49e658b0e8</x:v>
+      </x:c>
+      <x:c r="U7" s="39" t="str">
+        <x:v>2026-07-02T15:27:34Z</x:v>
+      </x:c>
+      <x:c r="V7" s="39" t="str">
+        <x:v>2026-07-02T15:27:34Z</x:v>
+      </x:c>
+      <x:c r="W7" s="39" t="str">
+        <x:v>2026-07-02T17:27:34Z</x:v>
+      </x:c>
       <x:c r="X7" s="39"/>
       <x:c r="Y7" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z7" s="39" t="str">
-        <x:v>Migrated from GitHub issue #619; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
       </x:c>
       <x:c r="AA7" s="39"/>
       <x:c r="AB7" s="39"/>
       <x:c r="AC7" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #616 DONE (PR #1280 merged, ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4339,7 +4339,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q4" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R4" s="36" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
@@ -4352,20 +4352,24 @@
         <x:v>2026-07-02T12:06:09Z</x:v>
       </x:c>
       <x:c r="V4" s="36" t="str">
-        <x:v>2026-07-02T15:26:03Z</x:v>
-      </x:c>
-      <x:c r="W4" s="36" t="str">
-        <x:v>2026-07-02T17:26:03Z</x:v>
-      </x:c>
-      <x:c r="X4" s="36"/>
+        <x:v>2026-07-02T15:50:57Z</x:v>
+      </x:c>
+      <x:c r="W4" s="36"/>
+      <x:c r="X4" s="36" t="str">
+        <x:v>2026-07-02T15:50:57Z</x:v>
+      </x:c>
       <x:c r="Y4" s="36" t="n">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>PR #1280 green on prior head; revalidating after #1277 merge, completion imminent</x:v>
-      </x:c>
-      <x:c r="AA4" s="36"/>
-      <x:c r="AB4" s="36"/>
+        <x:v>DONE via PR #1280</x:v>
+      </x:c>
+      <x:c r="AA4" s="36" t="str">
+        <x:v>Merged PR #1280 (squash bf3a8ac). Adds scripts/subagent_registry.py: versioned controller-local lifecycle registry (register/report/finalize/list/sweep/mark/validate) with atomic locked persistence; strictly read-only byte-stable sweeper reconciling records against worktree/branch/workbook-claim evidence with ORPHANED/UNREACHABLE recommendations; 16 tests; docs sections.</x:v>
+      </x:c>
+      <x:c r="AB4" s="36" t="str">
+        <x:v>tests.test_subagent_registry (16 OK); tests.test_issue_queue (45 OK); doc guards (58 OK); PR #1280 CI green (linux, windows-deps, windows)</x:v>
+      </x:c>
       <x:c r="AC4" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #616 DONE (PR #1280 merged, ctrl-vm-4027) (#1305)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4339,7 +4339,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q4" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R4" s="36" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-4</x:v>
@@ -4352,20 +4352,24 @@
         <x:v>2026-07-02T12:06:09Z</x:v>
       </x:c>
       <x:c r="V4" s="36" t="str">
-        <x:v>2026-07-02T15:26:03Z</x:v>
-      </x:c>
-      <x:c r="W4" s="36" t="str">
-        <x:v>2026-07-02T17:26:03Z</x:v>
-      </x:c>
-      <x:c r="X4" s="36"/>
+        <x:v>2026-07-02T15:50:57Z</x:v>
+      </x:c>
+      <x:c r="W4" s="36"/>
+      <x:c r="X4" s="36" t="str">
+        <x:v>2026-07-02T15:50:57Z</x:v>
+      </x:c>
       <x:c r="Y4" s="36" t="n">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z4" s="36" t="str">
-        <x:v>PR #1280 green on prior head; revalidating after #1277 merge, completion imminent</x:v>
-      </x:c>
-      <x:c r="AA4" s="36"/>
-      <x:c r="AB4" s="36"/>
+        <x:v>DONE via PR #1280</x:v>
+      </x:c>
+      <x:c r="AA4" s="36" t="str">
+        <x:v>Merged PR #1280 (squash bf3a8ac). Adds scripts/subagent_registry.py: versioned controller-local lifecycle registry (register/report/finalize/list/sweep/mark/validate) with atomic locked persistence; strictly read-only byte-stable sweeper reconciling records against worktree/branch/workbook-claim evidence with ORPHANED/UNREACHABLE recommendations; 16 tests; docs sections.</x:v>
+      </x:c>
+      <x:c r="AB4" s="36" t="str">
+        <x:v>tests.test_subagent_registry (16 OK); tests.test_issue_queue (45 OK); doc guards (58 OK); PR #1280 CI green (linux, windows-deps, windows)</x:v>
+      </x:c>
       <x:c r="AC4" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Claim #621 structured worker reports (migrated workbook, ctrl-vm-4027)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4769,25 +4769,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-workflow-optimizer.md</x:v>
       </x:c>
       <x:c r="Q9" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R9" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R9" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
+      </x:c>
       <x:c r="S9" s="39"/>
-      <x:c r="T9" s="39"/>
-      <x:c r="U9" s="39"/>
-      <x:c r="V9" s="39"/>
-      <x:c r="W9" s="39"/>
+      <x:c r="T9" s="39" t="str">
+        <x:v>7920ae34-aaca-4808-a308-adfcd6e0f3e3</x:v>
+      </x:c>
+      <x:c r="U9" s="39" t="str">
+        <x:v>2026-07-02T15:55:04Z</x:v>
+      </x:c>
+      <x:c r="V9" s="39" t="str">
+        <x:v>2026-07-02T15:55:04Z</x:v>
+      </x:c>
+      <x:c r="W9" s="39" t="str">
+        <x:v>2026-07-02T17:55:04Z</x:v>
+      </x:c>
       <x:c r="X9" s="39"/>
       <x:c r="Y9" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z9" s="39" t="str">
-        <x:v>Migrated from GitHub issue #621; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
       </x:c>
       <x:c r="AA9" s="39"/>
       <x:c r="AB9" s="39"/>
       <x:c r="AC9" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #621 structured worker reports (migrated workbook, ctrl-vm-4027) (#1308)
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4769,25 +4769,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-workflow-optimizer.md</x:v>
       </x:c>
       <x:c r="Q9" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R9" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R9" s="39" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
+      </x:c>
       <x:c r="S9" s="39"/>
-      <x:c r="T9" s="39"/>
-      <x:c r="U9" s="39"/>
-      <x:c r="V9" s="39"/>
-      <x:c r="W9" s="39"/>
+      <x:c r="T9" s="39" t="str">
+        <x:v>7920ae34-aaca-4808-a308-adfcd6e0f3e3</x:v>
+      </x:c>
+      <x:c r="U9" s="39" t="str">
+        <x:v>2026-07-02T15:55:04Z</x:v>
+      </x:c>
+      <x:c r="V9" s="39" t="str">
+        <x:v>2026-07-02T15:55:04Z</x:v>
+      </x:c>
+      <x:c r="W9" s="39" t="str">
+        <x:v>2026-07-02T17:55:04Z</x:v>
+      </x:c>
       <x:c r="X9" s="39"/>
       <x:c r="Y9" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z9" s="39" t="str">
-        <x:v>Migrated from GitHub issue #621; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
       </x:c>
       <x:c r="AA9" s="39"/>
       <x:c r="AB9" s="39"/>
       <x:c r="AC9" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #617 resource broker DONE (PR #1306 merged, ctrl-vm-4027)
Queue-state-only change: complete the subagent-5 claim on the migrated
workbook row for #617 after PR #1306 squash-merged as 9e11e8a6 with a
green pull_request build run.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4431,7 +4431,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q5" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R5" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
@@ -4444,20 +4444,24 @@
         <x:v>2026-07-02T15:26:43Z</x:v>
       </x:c>
       <x:c r="V5" s="39" t="str">
-        <x:v>2026-07-02T15:26:43Z</x:v>
-      </x:c>
-      <x:c r="W5" s="39" t="str">
-        <x:v>2026-07-02T17:26:43Z</x:v>
-      </x:c>
-      <x:c r="X5" s="39"/>
+        <x:v>2026-07-02T17:35:04Z</x:v>
+      </x:c>
+      <x:c r="W5" s="39"/>
+      <x:c r="X5" s="39" t="str">
+        <x:v>2026-07-02T17:35:04Z</x:v>
+      </x:c>
       <x:c r="Y5" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z5" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
-      </x:c>
-      <x:c r="AA5" s="39"/>
-      <x:c r="AB5" s="39"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1306.</x:v>
+      </x:c>
+      <x:c r="AA5" s="39" t="str">
+        <x:v>Implemented by PR #1306 (squash-merged as 9e11e8a6): scripts/resource_broker.py observation/reservation split (read-only probes for memory, heavy jobs, Xvfb displays, TCP ports, build-dir ownership, MCP slots; typed atomic all-or-nothing reservations in planning/resource_reservations.json with sidecar lock, exclusive-conflict exit 3, non-destructive recover), controller_resource_audit.py subcommand dispatch with additive JSON, docs sections in AGENTS.md / docs/codex-agent-queue.md / prompts/codex-queue-controller.md.</x:v>
+      </x:c>
+      <x:c r="AB5" s="39" t="str">
+        <x:v>tests.test_controller_resource_audit 56 OK; controller_resource_audit --json exit 0 additive; tests.test_prompt_inventory + tests.test_workbook_queue 58 OK; py_compile OK; test.py --suite fast OK; black -l 120 clean; indentation clean. CI: pull_request build run 28608713362 on PR head 28cc1238 concluded success (after rebase onto main's paper.png configure fix).</x:v>
+      </x:c>
       <x:c r="AC5" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #617 resource broker DONE (PR #1306 merged, ctrl-vm-4027) (#1315)
Queue-state-only change: complete the subagent-5 claim on the migrated
workbook row for #617 after PR #1306 squash-merged as 9e11e8a6 with a
green pull_request build run.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4431,7 +4431,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q5" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R5" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
@@ -4444,20 +4444,24 @@
         <x:v>2026-07-02T15:26:43Z</x:v>
       </x:c>
       <x:c r="V5" s="39" t="str">
-        <x:v>2026-07-02T15:26:43Z</x:v>
-      </x:c>
-      <x:c r="W5" s="39" t="str">
-        <x:v>2026-07-02T17:26:43Z</x:v>
-      </x:c>
-      <x:c r="X5" s="39"/>
+        <x:v>2026-07-02T17:35:04Z</x:v>
+      </x:c>
+      <x:c r="W5" s="39"/>
+      <x:c r="X5" s="39" t="str">
+        <x:v>2026-07-02T17:35:04Z</x:v>
+      </x:c>
       <x:c r="Y5" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z5" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-5</x:v>
-      </x:c>
-      <x:c r="AA5" s="39"/>
-      <x:c r="AB5" s="39"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1306.</x:v>
+      </x:c>
+      <x:c r="AA5" s="39" t="str">
+        <x:v>Implemented by PR #1306 (squash-merged as 9e11e8a6): scripts/resource_broker.py observation/reservation split (read-only probes for memory, heavy jobs, Xvfb displays, TCP ports, build-dir ownership, MCP slots; typed atomic all-or-nothing reservations in planning/resource_reservations.json with sidecar lock, exclusive-conflict exit 3, non-destructive recover), controller_resource_audit.py subcommand dispatch with additive JSON, docs sections in AGENTS.md / docs/codex-agent-queue.md / prompts/codex-queue-controller.md.</x:v>
+      </x:c>
+      <x:c r="AB5" s="39" t="str">
+        <x:v>tests.test_controller_resource_audit 56 OK; controller_resource_audit --json exit 0 additive; tests.test_prompt_inventory + tests.test_workbook_queue 58 OK; py_compile OK; test.py --suite fast OK; black -l 120 clean; indentation clean. CI: pull_request build run 28608713362 on PR head 28cc1238 concluded success (after rebase onto main's paper.png configure fix).</x:v>
+      </x:c>
       <x:c r="AC5" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #619 capability probe DONE (PR #1307 merged, ctrl-vm-4027)
Queue-state-only change: complete the subagent-6 claim on the migrated
workbook row for #619 after PR #1307 squash-merged as 3f5d16ba with a
green pull_request build run.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4605,7 +4605,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q7" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R7" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
@@ -4618,20 +4618,24 @@
         <x:v>2026-07-02T15:27:34Z</x:v>
       </x:c>
       <x:c r="V7" s="39" t="str">
-        <x:v>2026-07-02T15:27:34Z</x:v>
-      </x:c>
-      <x:c r="W7" s="39" t="str">
-        <x:v>2026-07-02T17:27:34Z</x:v>
-      </x:c>
-      <x:c r="X7" s="39"/>
+        <x:v>2026-07-02T17:42:22Z</x:v>
+      </x:c>
+      <x:c r="W7" s="39"/>
+      <x:c r="X7" s="39" t="str">
+        <x:v>2026-07-02T17:42:22Z</x:v>
+      </x:c>
       <x:c r="Y7" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z7" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
-      </x:c>
-      <x:c r="AA7" s="39"/>
-      <x:c r="AB7" s="39"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1307.</x:v>
+      </x:c>
+      <x:c r="AA7" s="39" t="str">
+        <x:v>Implemented by PR #1307 (squash-merged as 3f5d16ba): scripts/controller_capability_probe.py read-only capability snapshot (repository/github/ci/toolchain/build/agent sections, available/unavailable/unknown/unsupported statuses, redacted bounded evidence, deterministic sorted output, --now injection, exit 0 on missing capabilities), doc guidance to treat unknown/unavailable required capabilities as dispatch blockers. Validation-authority files untouched.</x:v>
+      </x:c>
+      <x:c r="AB7" s="39" t="str">
+        <x:v>tests.test_controller_capability_probe 28 OK; probe --json byte-identical across two runs, exit 0; tests.test_prompt_inventory + tests.test_workbook_queue 58 OK; py_compile OK; test.py --suite fast OK; black -l 120 clean; indentation clean. CI: pull_request build run 28608714582 on merge sha f285b2d0 concluded success.</x:v>
+      </x:c>
       <x:c r="AC7" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #619 capability probe DONE (PR #1307 merged, ctrl-vm-4027) (#1318)
Queue-state-only change: complete the subagent-6 claim on the migrated
workbook row for #619 after PR #1307 squash-merged as 3f5d16ba with a
green pull_request build run.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4605,7 +4605,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q7" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R7" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
@@ -4618,20 +4618,24 @@
         <x:v>2026-07-02T15:27:34Z</x:v>
       </x:c>
       <x:c r="V7" s="39" t="str">
-        <x:v>2026-07-02T15:27:34Z</x:v>
-      </x:c>
-      <x:c r="W7" s="39" t="str">
-        <x:v>2026-07-02T17:27:34Z</x:v>
-      </x:c>
-      <x:c r="X7" s="39"/>
+        <x:v>2026-07-02T17:42:22Z</x:v>
+      </x:c>
+      <x:c r="W7" s="39"/>
+      <x:c r="X7" s="39" t="str">
+        <x:v>2026-07-02T17:42:22Z</x:v>
+      </x:c>
       <x:c r="Y7" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z7" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-6</x:v>
-      </x:c>
-      <x:c r="AA7" s="39"/>
-      <x:c r="AB7" s="39"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1307.</x:v>
+      </x:c>
+      <x:c r="AA7" s="39" t="str">
+        <x:v>Implemented by PR #1307 (squash-merged as 3f5d16ba): scripts/controller_capability_probe.py read-only capability snapshot (repository/github/ci/toolchain/build/agent sections, available/unavailable/unknown/unsupported statuses, redacted bounded evidence, deterministic sorted output, --now injection, exit 0 on missing capabilities), doc guidance to treat unknown/unavailable required capabilities as dispatch blockers. Validation-authority files untouched.</x:v>
+      </x:c>
+      <x:c r="AB7" s="39" t="str">
+        <x:v>tests.test_controller_capability_probe 28 OK; probe --json byte-identical across two runs, exit 0; tests.test_prompt_inventory + tests.test_workbook_queue 58 OK; py_compile OK; test.py --suite fast OK; black -l 120 clean; indentation clean. CI: pull_request build run 28608714582 on merge sha f285b2d0 concluded success.</x:v>
+      </x:c>
       <x:c r="AC7" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #669 DONE (PR #1261 merged, run-identity+attempt hardening)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5863,7 +5863,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R21" s="39" t="str">
         <x:v>ctrl-vm-2256-06ac44fc</x:v>
@@ -5876,20 +5876,24 @@
         <x:v>2026-07-02T07:46:27Z</x:v>
       </x:c>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-07-02T07:46:39Z</x:v>
-      </x:c>
-      <x:c r="W21" s="39" t="str">
-        <x:v>2026-07-02T09:46:39Z</x:v>
-      </x:c>
-      <x:c r="X21" s="39"/>
+        <x:v>2026-07-02T17:57:32Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39"/>
+      <x:c r="X21" s="39" t="str">
+        <x:v>2026-07-02T17:57:32Z</x:v>
+      </x:c>
       <x:c r="Y21" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Implemented run-identity ambiguity + attempt binding in poll_pr_checks.py; PR #1261 open (fast-path CI green, 7 tests). Authority-file change awaits human review + native-green.</x:v>
-      </x:c>
-      <x:c r="AA21" s="39"/>
-      <x:c r="AB21" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA21" s="39" t="str">
+        <x:v>Delivered via merged PR #1261 (commit 5554809): poll_pr_checks.py now blocks ambiguous run identity (&gt;1 distinct run for the head SHA) and binds/verifies the run attempt, extending #934's head-SHA/event/workflow-name identity and ambiguous-job guards. 7 new tests.</x:v>
+      </x:c>
+      <x:c r="AB21" s="39" t="str">
+        <x:v>python3 -m unittest tests.test_poll_pr_checks -&gt; 46 tests OK; fast-path CI (validate/linux-fast/export) green on PR #1261; merged to main.</x:v>
+      </x:c>
       <x:c r="AC21" s="39" t="n">
         <x:v>2</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #669 DONE (PR #1261 merged) (#1323)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5863,7 +5863,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/AGENTS.md</x:v>
       </x:c>
       <x:c r="Q21" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R21" s="39" t="str">
         <x:v>ctrl-vm-2256-06ac44fc</x:v>
@@ -5876,20 +5876,24 @@
         <x:v>2026-07-02T07:46:27Z</x:v>
       </x:c>
       <x:c r="V21" s="39" t="str">
-        <x:v>2026-07-02T07:46:39Z</x:v>
-      </x:c>
-      <x:c r="W21" s="39" t="str">
-        <x:v>2026-07-02T09:46:39Z</x:v>
-      </x:c>
-      <x:c r="X21" s="39"/>
+        <x:v>2026-07-02T17:57:32Z</x:v>
+      </x:c>
+      <x:c r="W21" s="39"/>
+      <x:c r="X21" s="39" t="str">
+        <x:v>2026-07-02T17:57:32Z</x:v>
+      </x:c>
       <x:c r="Y21" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z21" s="39" t="str">
-        <x:v>Implemented run-identity ambiguity + attempt binding in poll_pr_checks.py; PR #1261 open (fast-path CI green, 7 tests). Authority-file change awaits human review + native-green.</x:v>
-      </x:c>
-      <x:c r="AA21" s="39"/>
-      <x:c r="AB21" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA21" s="39" t="str">
+        <x:v>Delivered via merged PR #1261 (commit 5554809): poll_pr_checks.py now blocks ambiguous run identity (&gt;1 distinct run for the head SHA) and binds/verifies the run attempt, extending #934's head-SHA/event/workflow-name identity and ambiguous-job guards. 7 new tests.</x:v>
+      </x:c>
+      <x:c r="AB21" s="39" t="str">
+        <x:v>python3 -m unittest tests.test_poll_pr_checks -&gt; 46 tests OK; fast-path CI (validate/linux-fast/export) green on PR #1261; merged to main.</x:v>
+      </x:c>
       <x:c r="AC21" s="39" t="n">
         <x:v>2</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #621 structured worker reports DONE (PR #1313 merged, ctrl-vm-4027)
Queue-state-only change: complete the subagent-7 claim on the migrated
workbook row for #621 after PR #1313 squash-merged as 49a786ec.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4777,7 +4777,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-workflow-optimizer.md</x:v>
       </x:c>
       <x:c r="Q9" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R9" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
@@ -4790,20 +4790,24 @@
         <x:v>2026-07-02T15:55:04Z</x:v>
       </x:c>
       <x:c r="V9" s="39" t="str">
-        <x:v>2026-07-02T15:55:04Z</x:v>
-      </x:c>
-      <x:c r="W9" s="39" t="str">
-        <x:v>2026-07-02T17:55:04Z</x:v>
-      </x:c>
-      <x:c r="X9" s="39"/>
+        <x:v>2026-07-03T04:08:32Z</x:v>
+      </x:c>
+      <x:c r="W9" s="39"/>
+      <x:c r="X9" s="39" t="str">
+        <x:v>2026-07-03T04:08:32Z</x:v>
+      </x:c>
       <x:c r="Y9" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z9" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
-      </x:c>
-      <x:c r="AA9" s="39"/>
-      <x:c r="AB9" s="39"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1313.</x:v>
+      </x:c>
+      <x:c r="AA9" s="39" t="str">
+        <x:v>Implemented by PR #1313 (squash-merged as 49a786ec): scripts/worker_report.py stdlib-only CLI (create/validate/render/handoff/registry-payload) with schema v1 worker reports (owner/claimId/issue/branch/filesChanged/commands with per-command outcomes and exit codes/ciHeadSha/outcome), identity and CI-SHA cross-validation, deterministic bounded restart handoffs (10-item section cap), optional subagent_registry bridge; doc sections in AGENTS.md, docs/codex-agent-queue.md, prompt pointers.</x:v>
+      </x:c>
+      <x:c r="AB9" s="39" t="str">
+        <x:v>tests.test_worker_report 16 OK; tests/ discovery 583 OK (1 _game skip); tests.test_prompt_inventory OK; validate_content OK; black -l 120 clean; indentation clean. Python tooling suites green in PR runs; merged to main as 49a786ec.</x:v>
+      </x:c>
       <x:c r="AC9" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #621 structured worker reports DONE (PR #1313 merged, ctrl-vm-4027) (#1339)
Queue-state-only change: complete the subagent-7 claim on the migrated
workbook row for #621 after PR #1313 squash-merged as 49a786ec.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4777,7 +4777,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-workflow-optimizer.md</x:v>
       </x:c>
       <x:c r="Q9" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R9" s="39" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
@@ -4790,20 +4790,24 @@
         <x:v>2026-07-02T15:55:04Z</x:v>
       </x:c>
       <x:c r="V9" s="39" t="str">
-        <x:v>2026-07-02T15:55:04Z</x:v>
-      </x:c>
-      <x:c r="W9" s="39" t="str">
-        <x:v>2026-07-02T17:55:04Z</x:v>
-      </x:c>
-      <x:c r="X9" s="39"/>
+        <x:v>2026-07-03T04:08:32Z</x:v>
+      </x:c>
+      <x:c r="W9" s="39"/>
+      <x:c r="X9" s="39" t="str">
+        <x:v>2026-07-03T04:08:32Z</x:v>
+      </x:c>
       <x:c r="Y9" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z9" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
-      </x:c>
-      <x:c r="AA9" s="39"/>
-      <x:c r="AB9" s="39"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1313.</x:v>
+      </x:c>
+      <x:c r="AA9" s="39" t="str">
+        <x:v>Implemented by PR #1313 (squash-merged as 49a786ec): scripts/worker_report.py stdlib-only CLI (create/validate/render/handoff/registry-payload) with schema v1 worker reports (owner/claimId/issue/branch/filesChanged/commands with per-command outcomes and exit codes/ciHeadSha/outcome), identity and CI-SHA cross-validation, deterministic bounded restart handoffs (10-item section cap), optional subagent_registry bridge; doc sections in AGENTS.md, docs/codex-agent-queue.md, prompt pointers.</x:v>
+      </x:c>
+      <x:c r="AB9" s="39" t="str">
+        <x:v>tests.test_worker_report 16 OK; tests/ discovery 583 OK (1 _game skip); tests.test_prompt_inventory OK; validate_content OK; black -l 120 clean; indentation clean. Python tooling suites green in PR runs; merged to main as 49a786ec.</x:v>
+      </x:c>
       <x:c r="AC9" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Claim #620 consolidate mechanical controller policy (migrated workbook, ctrl-vm-4027)
Queue-state-only change: claim the row for
controller/ctrl-vm-4027-c0afa077/subagent-7. No dependencies.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4698,25 +4698,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-queue-controller.md</x:v>
       </x:c>
       <x:c r="Q8" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R8" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R8" s="36" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
+      </x:c>
       <x:c r="S8" s="36"/>
-      <x:c r="T8" s="36"/>
-      <x:c r="U8" s="36"/>
-      <x:c r="V8" s="36"/>
-      <x:c r="W8" s="36"/>
+      <x:c r="T8" s="36" t="str">
+        <x:v>e769e133-2cee-4540-ab52-fc289143e905</x:v>
+      </x:c>
+      <x:c r="U8" s="36" t="str">
+        <x:v>2026-07-03T05:04:22Z</x:v>
+      </x:c>
+      <x:c r="V8" s="36" t="str">
+        <x:v>2026-07-03T05:04:22Z</x:v>
+      </x:c>
+      <x:c r="W8" s="36" t="str">
+        <x:v>2026-07-03T07:04:22Z</x:v>
+      </x:c>
       <x:c r="X8" s="36"/>
       <x:c r="Y8" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z8" s="36" t="str">
-        <x:v>Migrated from GitHub issue #620; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
       </x:c>
       <x:c r="AA8" s="36"/>
       <x:c r="AB8" s="36"/>
       <x:c r="AC8" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #620 consolidate mechanical controller policy (migrated workbook, ctrl-vm-4027) (#1350)
Queue-state-only change: claim the row for
controller/ctrl-vm-4027-c0afa077/subagent-7. No dependencies.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4698,25 +4698,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-queue-controller.md</x:v>
       </x:c>
       <x:c r="Q8" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R8" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R8" s="36" t="str">
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
+      </x:c>
       <x:c r="S8" s="36"/>
-      <x:c r="T8" s="36"/>
-      <x:c r="U8" s="36"/>
-      <x:c r="V8" s="36"/>
-      <x:c r="W8" s="36"/>
+      <x:c r="T8" s="36" t="str">
+        <x:v>e769e133-2cee-4540-ab52-fc289143e905</x:v>
+      </x:c>
+      <x:c r="U8" s="36" t="str">
+        <x:v>2026-07-03T05:04:22Z</x:v>
+      </x:c>
+      <x:c r="V8" s="36" t="str">
+        <x:v>2026-07-03T05:04:22Z</x:v>
+      </x:c>
+      <x:c r="W8" s="36" t="str">
+        <x:v>2026-07-03T07:04:22Z</x:v>
+      </x:c>
       <x:c r="X8" s="36"/>
       <x:c r="Y8" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z8" s="36" t="str">
-        <x:v>Migrated from GitHub issue #620; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
       </x:c>
       <x:c r="AA8" s="36"/>
       <x:c r="AB8" s="36"/>
       <x:c r="AC8" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #618 DONE (PR #1342 merged, change-kind taxonomy)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4526,25 +4526,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/coverage_report.py</x:v>
       </x:c>
       <x:c r="Q6" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R6" s="36"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R6" s="36" t="str">
+        <x:v>ctrl-vm-2617-4ae45d4e</x:v>
+      </x:c>
       <x:c r="S6" s="36"/>
-      <x:c r="T6" s="36"/>
-      <x:c r="U6" s="36"/>
-      <x:c r="V6" s="36"/>
+      <x:c r="T6" s="36" t="str">
+        <x:v>4069f9fd-ce0e-4efe-8f17-93a636df7f22</x:v>
+      </x:c>
+      <x:c r="U6" s="36" t="str">
+        <x:v>2026-07-03T08:59:32Z</x:v>
+      </x:c>
+      <x:c r="V6" s="36" t="str">
+        <x:v>2026-07-03T08:59:32Z</x:v>
+      </x:c>
       <x:c r="W6" s="36"/>
-      <x:c r="X6" s="36"/>
+      <x:c r="X6" s="36" t="str">
+        <x:v>2026-07-03T08:59:32Z</x:v>
+      </x:c>
       <x:c r="Y6" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z6" s="36" t="str">
-        <x:v>Migrated from GitHub issue #618; not yet claimed.</x:v>
-      </x:c>
-      <x:c r="AA6" s="36"/>
-      <x:c r="AB6" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA6" s="36" t="str">
+        <x:v>Delivered via merged PR #1342: additive change-KIND taxonomy on ci_change_classifier.py + _path_kind, GitHub outputs, src/gui/** coverage-lock test. build.yml gating unchanged. Human-reviewed and merged (authority file).</x:v>
+      </x:c>
+      <x:c r="AB6" s="36" t="str">
+        <x:v>unittest ci_change_classifier+poll_pr_checks+prompt_inventory -&gt; 74 OK; merged to main.</x:v>
+      </x:c>
       <x:c r="AC6" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #618 DONE (PR #1342 merged) (#1355)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4526,25 +4526,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/coverage_report.py</x:v>
       </x:c>
       <x:c r="Q6" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R6" s="36"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R6" s="36" t="str">
+        <x:v>ctrl-vm-2617-4ae45d4e</x:v>
+      </x:c>
       <x:c r="S6" s="36"/>
-      <x:c r="T6" s="36"/>
-      <x:c r="U6" s="36"/>
-      <x:c r="V6" s="36"/>
+      <x:c r="T6" s="36" t="str">
+        <x:v>4069f9fd-ce0e-4efe-8f17-93a636df7f22</x:v>
+      </x:c>
+      <x:c r="U6" s="36" t="str">
+        <x:v>2026-07-03T08:59:32Z</x:v>
+      </x:c>
+      <x:c r="V6" s="36" t="str">
+        <x:v>2026-07-03T08:59:32Z</x:v>
+      </x:c>
       <x:c r="W6" s="36"/>
-      <x:c r="X6" s="36"/>
+      <x:c r="X6" s="36" t="str">
+        <x:v>2026-07-03T08:59:32Z</x:v>
+      </x:c>
       <x:c r="Y6" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z6" s="36" t="str">
-        <x:v>Migrated from GitHub issue #618; not yet claimed.</x:v>
-      </x:c>
-      <x:c r="AA6" s="36"/>
-      <x:c r="AB6" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA6" s="36" t="str">
+        <x:v>Delivered via merged PR #1342: additive change-KIND taxonomy on ci_change_classifier.py + _path_kind, GitHub outputs, src/gui/** coverage-lock test. build.yml gating unchanged. Human-reviewed and merged (authority file).</x:v>
+      </x:c>
+      <x:c r="AB6" s="36" t="str">
+        <x:v>unittest ci_change_classifier+poll_pr_checks+prompt_inventory -&gt; 74 OK; merged to main.</x:v>
+      </x:c>
       <x:c r="AC6" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #614 durable controller transition reconciler (refill slot)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4167,25 +4167,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q2" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R2" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R2" s="36" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-46</x:v>
+      </x:c>
       <x:c r="S2" s="36"/>
-      <x:c r="T2" s="36"/>
-      <x:c r="U2" s="36"/>
-      <x:c r="V2" s="36"/>
-      <x:c r="W2" s="36"/>
+      <x:c r="T2" s="36" t="str">
+        <x:v>94e6906b-988f-4f1a-b318-5d060bd9991a</x:v>
+      </x:c>
+      <x:c r="U2" s="36" t="str">
+        <x:v>2026-07-03T09:10:41Z</x:v>
+      </x:c>
+      <x:c r="V2" s="36" t="str">
+        <x:v>2026-07-03T09:10:41Z</x:v>
+      </x:c>
+      <x:c r="W2" s="36" t="str">
+        <x:v>2026-07-03T12:10:41Z</x:v>
+      </x:c>
       <x:c r="X2" s="36"/>
       <x:c r="Y2" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z2" s="36" t="str">
-        <x:v>Migrated from GitHub issue #614; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-46</x:v>
       </x:c>
       <x:c r="AA2" s="36"/>
       <x:c r="AB2" s="36"/>
       <x:c r="AC2" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #620 mechanical policy consolidation DONE (PR #1354 merged, ctrl-vm-4027)
Queue-state-only change: complete the subagent-7 claim on the migrated
workbook row after PR #1354 squash-merged as f3cf8ac2 with a green build run.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4712,7 +4712,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-queue-controller.md</x:v>
       </x:c>
       <x:c r="Q8" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R8" s="36" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
@@ -4725,20 +4725,24 @@
         <x:v>2026-07-03T05:04:22Z</x:v>
       </x:c>
       <x:c r="V8" s="36" t="str">
-        <x:v>2026-07-03T05:04:22Z</x:v>
-      </x:c>
-      <x:c r="W8" s="36" t="str">
-        <x:v>2026-07-03T07:04:22Z</x:v>
-      </x:c>
-      <x:c r="X8" s="36"/>
+        <x:v>2026-07-03T11:22:28Z</x:v>
+      </x:c>
+      <x:c r="W8" s="36"/>
+      <x:c r="X8" s="36" t="str">
+        <x:v>2026-07-03T11:22:28Z</x:v>
+      </x:c>
       <x:c r="Y8" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z8" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
-      </x:c>
-      <x:c r="AA8" s="36"/>
-      <x:c r="AB8" s="36"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1354 (green CI on updated branch onto green main).</x:v>
+      </x:c>
+      <x:c r="AA8" s="36" t="str">
+        <x:v>Implemented by PR #1354 (squash-merged as f3cf8ac2): scripts/controller_policy.py canonical stdlib-only policy module (SCHEMA_VERSION, PolicyField dataclass with value/type/bounds/enum/description + errors(), POLICY registry, value()/heartbeat_interval_minutes() accessors, canonical QUEUE_STATUSES/QUEUE_PRIORITIES/TARGET_FILE_OVERLAP_POLICIES, validate() with cross-field checks, schemaPayload(), fast-check CLI). scripts/issue_queue.py and scripts/subagent_registry.py derive their legacy constants/CLI defaults from the policy via guarded imports; no numeric value changed. Docs/prompt reference the canonical source.</x:v>
+      </x:c>
+      <x:c r="AB8" s="36" t="str">
+        <x:v>GREEN on PR #1354 CI run 28656339768 (conclusion success, all jobs). tests.test_controller_policy 11 OK; tests.test_issue_queue 46 OK; tests.test_subagent_registry 17 OK; tests.test_prompt_inventory 7 OK; tests.test_worker_report 16 OK; full tests/ discovery 702 OK; black -l 120 clean; 4-space indentation clean; validate_content OK.</x:v>
+      </x:c>
       <x:c r="AC8" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #620 mechanical policy consolidation DONE (PR #1354 merged, ctrl-vm-4027) (#1375)
Queue-state-only change: complete the subagent-7 claim on the migrated
workbook row after PR #1354 squash-merged as f3cf8ac2 with a green build run.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4712,7 +4712,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/prompts/codex-queue-controller.md</x:v>
       </x:c>
       <x:c r="Q8" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R8" s="36" t="str">
         <x:v>controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
@@ -4725,20 +4725,24 @@
         <x:v>2026-07-03T05:04:22Z</x:v>
       </x:c>
       <x:c r="V8" s="36" t="str">
-        <x:v>2026-07-03T05:04:22Z</x:v>
-      </x:c>
-      <x:c r="W8" s="36" t="str">
-        <x:v>2026-07-03T07:04:22Z</x:v>
-      </x:c>
-      <x:c r="X8" s="36"/>
+        <x:v>2026-07-03T11:22:28Z</x:v>
+      </x:c>
+      <x:c r="W8" s="36"/>
+      <x:c r="X8" s="36" t="str">
+        <x:v>2026-07-03T11:22:28Z</x:v>
+      </x:c>
       <x:c r="Y8" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z8" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4027-c0afa077/subagent-7</x:v>
-      </x:c>
-      <x:c r="AA8" s="36"/>
-      <x:c r="AB8" s="36"/>
+        <x:v>Completed by controller ctrl-vm-4027-c0afa077 after squash-merge of PR #1354 (green CI on updated branch onto green main).</x:v>
+      </x:c>
+      <x:c r="AA8" s="36" t="str">
+        <x:v>Implemented by PR #1354 (squash-merged as f3cf8ac2): scripts/controller_policy.py canonical stdlib-only policy module (SCHEMA_VERSION, PolicyField dataclass with value/type/bounds/enum/description + errors(), POLICY registry, value()/heartbeat_interval_minutes() accessors, canonical QUEUE_STATUSES/QUEUE_PRIORITIES/TARGET_FILE_OVERLAP_POLICIES, validate() with cross-field checks, schemaPayload(), fast-check CLI). scripts/issue_queue.py and scripts/subagent_registry.py derive their legacy constants/CLI defaults from the policy via guarded imports; no numeric value changed. Docs/prompt reference the canonical source.</x:v>
+      </x:c>
+      <x:c r="AB8" s="36" t="str">
+        <x:v>GREEN on PR #1354 CI run 28656339768 (conclusion success, all jobs). tests.test_controller_policy 11 OK; tests.test_issue_queue 46 OK; tests.test_subagent_registry 17 OK; tests.test_prompt_inventory 7 OK; tests.test_worker_report 16 OK; full tests/ discovery 702 OK; black -l 120 clean; 4-space indentation clean; validate_content OK.</x:v>
+      </x:c>
       <x:c r="AC8" s="36" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Claim heartbeat batch publication issue
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4899,25 +4899,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q10" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R10" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R10" s="36" t="str">
+        <x:v>controller/ctrl-lis-2-14d26144/subagent-1</x:v>
+      </x:c>
       <x:c r="S10" s="36"/>
-      <x:c r="T10" s="36"/>
-      <x:c r="U10" s="36"/>
-      <x:c r="V10" s="36"/>
-      <x:c r="W10" s="36"/>
+      <x:c r="T10" s="36" t="str">
+        <x:v>d0707cc7-e3ad-4b04-a939-e9e616e61293</x:v>
+      </x:c>
+      <x:c r="U10" s="36" t="str">
+        <x:v>2026-07-06T03:09:28Z</x:v>
+      </x:c>
+      <x:c r="V10" s="36" t="str">
+        <x:v>2026-07-06T03:09:28Z</x:v>
+      </x:c>
+      <x:c r="W10" s="36" t="str">
+        <x:v>2026-07-07T03:09:28Z</x:v>
+      </x:c>
       <x:c r="X10" s="36"/>
       <x:c r="Y10" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z10" s="36" t="str">
-        <x:v>Migrated from GitHub issue #622; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-lis-2-14d26144/subagent-1</x:v>
       </x:c>
       <x:c r="AA10" s="36"/>
       <x:c r="AB10" s="36"/>
       <x:c r="AC10" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim heartbeat batch publication issue (#1419)
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4899,25 +4899,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q10" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R10" s="36"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R10" s="36" t="str">
+        <x:v>controller/ctrl-lis-2-14d26144/subagent-1</x:v>
+      </x:c>
       <x:c r="S10" s="36"/>
-      <x:c r="T10" s="36"/>
-      <x:c r="U10" s="36"/>
-      <x:c r="V10" s="36"/>
-      <x:c r="W10" s="36"/>
+      <x:c r="T10" s="36" t="str">
+        <x:v>d0707cc7-e3ad-4b04-a939-e9e616e61293</x:v>
+      </x:c>
+      <x:c r="U10" s="36" t="str">
+        <x:v>2026-07-06T03:09:28Z</x:v>
+      </x:c>
+      <x:c r="V10" s="36" t="str">
+        <x:v>2026-07-06T03:09:28Z</x:v>
+      </x:c>
+      <x:c r="W10" s="36" t="str">
+        <x:v>2026-07-07T03:09:28Z</x:v>
+      </x:c>
       <x:c r="X10" s="36"/>
       <x:c r="Y10" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z10" s="36" t="str">
-        <x:v>Migrated from GitHub issue #622; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-lis-2-14d26144/subagent-1</x:v>
       </x:c>
       <x:c r="AA10" s="36"/>
       <x:c r="AB10" s="36"/>
       <x:c r="AC10" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Reconcile duplicate #614 row as DONE (delivered by PRs #1349/#1364)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4167,25 +4167,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q2" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R2" s="36"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R2" s="36" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-55</x:v>
+      </x:c>
       <x:c r="S2" s="36"/>
-      <x:c r="T2" s="36"/>
-      <x:c r="U2" s="36"/>
-      <x:c r="V2" s="36"/>
+      <x:c r="T2" s="36" t="str">
+        <x:v>68129181-22e8-4bd4-a4a2-b4b0dafa4e32</x:v>
+      </x:c>
+      <x:c r="U2" s="36" t="str">
+        <x:v>2026-07-08T10:48:53Z</x:v>
+      </x:c>
+      <x:c r="V2" s="36" t="str">
+        <x:v>2026-07-08T10:48:53Z</x:v>
+      </x:c>
       <x:c r="W2" s="36"/>
-      <x:c r="X2" s="36"/>
+      <x:c r="X2" s="36" t="str">
+        <x:v>2026-07-08T10:48:53Z</x:v>
+      </x:c>
       <x:c r="Y2" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z2" s="36" t="str">
-        <x:v>Migrated from GitHub issue #614; not yet claimed.</x:v>
-      </x:c>
-      <x:c r="AA2" s="36"/>
-      <x:c r="AB2" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA2" s="36" t="str">
+        <x:v>Reconciliation record: #614 is already delivered on main. scripts/controller_reconciler.py (snapshot/reconcile/next-action; read-only, deterministic, idempotency keys) landed via the foundation PR #1349 and was completed with the claim_pr_open/claim_pr_merged lifecycle states plus 28 tests in tests/test_controller_reconciler.py via PR #1364 (merged a5542550). This duplicate row in the migrated workbook is closed against those merged PRs; no new implementation was needed.</x:v>
+      </x:c>
+      <x:c r="AB2" s="36" t="str">
+        <x:v>Verified on current main: scripts/controller_reconciler.py and tests/test_controller_reconciler.py exist with claim_pr states present; delivering PRs #1349/#1364 merged; duplicate rows of this issue in other workbooks already DONE.</x:v>
+      </x:c>
       <x:c r="AC2" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Reconcile duplicate #614 row as DONE (delivered by PRs #1349/#1364) (#1442)
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4167,25 +4167,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/issue_queue.py</x:v>
       </x:c>
       <x:c r="Q2" s="36" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R2" s="36"/>
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="R2" s="36" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-55</x:v>
+      </x:c>
       <x:c r="S2" s="36"/>
-      <x:c r="T2" s="36"/>
-      <x:c r="U2" s="36"/>
-      <x:c r="V2" s="36"/>
+      <x:c r="T2" s="36" t="str">
+        <x:v>68129181-22e8-4bd4-a4a2-b4b0dafa4e32</x:v>
+      </x:c>
+      <x:c r="U2" s="36" t="str">
+        <x:v>2026-07-08T10:48:53Z</x:v>
+      </x:c>
+      <x:c r="V2" s="36" t="str">
+        <x:v>2026-07-08T10:48:53Z</x:v>
+      </x:c>
       <x:c r="W2" s="36"/>
-      <x:c r="X2" s="36"/>
+      <x:c r="X2" s="36" t="str">
+        <x:v>2026-07-08T10:48:53Z</x:v>
+      </x:c>
       <x:c r="Y2" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z2" s="36" t="str">
-        <x:v>Migrated from GitHub issue #614; not yet claimed.</x:v>
-      </x:c>
-      <x:c r="AA2" s="36"/>
-      <x:c r="AB2" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA2" s="36" t="str">
+        <x:v>Reconciliation record: #614 is already delivered on main. scripts/controller_reconciler.py (snapshot/reconcile/next-action; read-only, deterministic, idempotency keys) landed via the foundation PR #1349 and was completed with the claim_pr_open/claim_pr_merged lifecycle states plus 28 tests in tests/test_controller_reconciler.py via PR #1364 (merged a5542550). This duplicate row in the migrated workbook is closed against those merged PRs; no new implementation was needed.</x:v>
+      </x:c>
+      <x:c r="AB2" s="36" t="str">
+        <x:v>Verified on current main: scripts/controller_reconciler.py and tests/test_controller_reconciler.py exist with claim_pr states present; delivering PRs #1349/#1364 merged; duplicate rows of this issue in other workbooks already DONE.</x:v>
+      </x:c>
       <x:c r="AC2" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #623 pull-request preflight duplicate and scope guard
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5003,25 +5003,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q11" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R11" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R11" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
+      </x:c>
       <x:c r="S11" s="39"/>
-      <x:c r="T11" s="39"/>
-      <x:c r="U11" s="39"/>
-      <x:c r="V11" s="39"/>
-      <x:c r="W11" s="39"/>
+      <x:c r="T11" s="39" t="str">
+        <x:v>3390230a-45c6-459f-b1fe-f12a2fb31bb2</x:v>
+      </x:c>
+      <x:c r="U11" s="39" t="str">
+        <x:v>2026-07-09T04:30:04Z</x:v>
+      </x:c>
+      <x:c r="V11" s="39" t="str">
+        <x:v>2026-07-09T04:30:04Z</x:v>
+      </x:c>
+      <x:c r="W11" s="39" t="str">
+        <x:v>2026-07-09T06:00:04Z</x:v>
+      </x:c>
       <x:c r="X11" s="39"/>
       <x:c r="Y11" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z11" s="39" t="str">
-        <x:v>Migrated from GitHub issue #623; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
       </x:c>
       <x:c r="AA11" s="39"/>
       <x:c r="AB11" s="39"/>
       <x:c r="AC11" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Claim #623 pull-request preflight duplicate and scope guard (#1452)
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5003,25 +5003,35 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q11" s="39" t="str">
-        <x:v>NOT_STARTED</x:v>
-      </x:c>
-      <x:c r="R11" s="39"/>
+        <x:v>IN_PROGRESS</x:v>
+      </x:c>
+      <x:c r="R11" s="39" t="str">
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
+      </x:c>
       <x:c r="S11" s="39"/>
-      <x:c r="T11" s="39"/>
-      <x:c r="U11" s="39"/>
-      <x:c r="V11" s="39"/>
-      <x:c r="W11" s="39"/>
+      <x:c r="T11" s="39" t="str">
+        <x:v>3390230a-45c6-459f-b1fe-f12a2fb31bb2</x:v>
+      </x:c>
+      <x:c r="U11" s="39" t="str">
+        <x:v>2026-07-09T04:30:04Z</x:v>
+      </x:c>
+      <x:c r="V11" s="39" t="str">
+        <x:v>2026-07-09T04:30:04Z</x:v>
+      </x:c>
+      <x:c r="W11" s="39" t="str">
+        <x:v>2026-07-09T06:00:04Z</x:v>
+      </x:c>
       <x:c r="X11" s="39"/>
       <x:c r="Y11" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z11" s="39" t="str">
-        <x:v>Migrated from GitHub issue #623; not yet claimed.</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
       </x:c>
       <x:c r="AA11" s="39"/>
       <x:c r="AB11" s="39"/>
       <x:c r="AC11" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #623 PR preflight duplicate and scope guard DONE (PR #1454 merged)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5003,7 +5003,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q11" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R11" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
@@ -5016,20 +5016,24 @@
         <x:v>2026-07-09T04:30:04Z</x:v>
       </x:c>
       <x:c r="V11" s="39" t="str">
-        <x:v>2026-07-09T04:30:04Z</x:v>
-      </x:c>
-      <x:c r="W11" s="39" t="str">
-        <x:v>2026-07-09T06:00:04Z</x:v>
-      </x:c>
-      <x:c r="X11" s="39"/>
+        <x:v>2026-07-09T05:08:25Z</x:v>
+      </x:c>
+      <x:c r="W11" s="39"/>
+      <x:c r="X11" s="39" t="str">
+        <x:v>2026-07-09T05:08:25Z</x:v>
+      </x:c>
       <x:c r="Y11" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z11" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
-      </x:c>
-      <x:c r="AA11" s="39"/>
-      <x:c r="AB11" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA11" s="39" t="str">
+        <x:v>Read-only PR preflight in pr_review_audit.py: deterministic verdict taxonomy (allow/allow_replacement/reject_duplicate_open/already_delivered/cannot_verify fail-closed), advisory-only scope/title warnings, JSON in/out with shell-gateable exit codes, issue_queue payload builder, controller docs. Both Codex findings fixed (object-shaped snapshots routed through loadRecords + doc example branches on nonzero exit). 240 tests green. Delivered by PR #1454 (merged).</x:v>
+      </x:c>
+      <x:c r="AB11" s="39" t="str">
+        <x:v>PR #1454 CI green on fix commit 6c17063a (all required lanes); squash-merged to main at efd8c03b.</x:v>
+      </x:c>
       <x:c r="AC11" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Mark #623 PR preflight duplicate and scope guard DONE (PR #1454 merged) (#1457)
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -5003,7 +5003,7 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/scripts/poll_pr_checks.py</x:v>
       </x:c>
       <x:c r="Q11" s="39" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R11" s="39" t="str">
         <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
@@ -5016,20 +5016,24 @@
         <x:v>2026-07-09T04:30:04Z</x:v>
       </x:c>
       <x:c r="V11" s="39" t="str">
-        <x:v>2026-07-09T04:30:04Z</x:v>
-      </x:c>
-      <x:c r="W11" s="39" t="str">
-        <x:v>2026-07-09T06:00:04Z</x:v>
-      </x:c>
-      <x:c r="X11" s="39"/>
+        <x:v>2026-07-09T05:08:25Z</x:v>
+      </x:c>
+      <x:c r="W11" s="39"/>
+      <x:c r="X11" s="39" t="str">
+        <x:v>2026-07-09T05:08:25Z</x:v>
+      </x:c>
       <x:c r="Y11" s="39" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z11" s="39" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-60</x:v>
-      </x:c>
-      <x:c r="AA11" s="39"/>
-      <x:c r="AB11" s="39"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA11" s="39" t="str">
+        <x:v>Read-only PR preflight in pr_review_audit.py: deterministic verdict taxonomy (allow/allow_replacement/reject_duplicate_open/already_delivered/cannot_verify fail-closed), advisory-only scope/title warnings, JSON in/out with shell-gateable exit codes, issue_queue payload builder, controller docs. Both Codex findings fixed (object-shaped snapshots routed through loadRecords + doc example branches on nonzero exit). 240 tests green. Delivered by PR #1454 (merged).</x:v>
+      </x:c>
+      <x:c r="AB11" s="39" t="str">
+        <x:v>PR #1454 CI green on fix commit 6c17063a (all required lanes); squash-merged to main at efd8c03b.</x:v>
+      </x:c>
       <x:c r="AC11" s="39" t="n">
         <x:v>1</x:v>
       </x:c>

</xml_diff>

<commit_message>
Reclaim stale #622 heartbeat automation claim and re-claim (lease expired 6 days)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4916,32 +4916,32 @@
         <x:v>IN_PROGRESS</x:v>
       </x:c>
       <x:c r="R10" s="36" t="str">
-        <x:v>controller/ctrl-lis-2-14d26144/subagent-1</x:v>
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
       </x:c>
       <x:c r="S10" s="36"/>
       <x:c r="T10" s="36" t="str">
-        <x:v>d0707cc7-e3ad-4b04-a939-e9e616e61293</x:v>
+        <x:v>0d2a37d1-1e85-4dde-aca2-7b95984e8786</x:v>
       </x:c>
       <x:c r="U10" s="36" t="str">
-        <x:v>2026-07-06T03:09:28Z</x:v>
+        <x:v>2026-07-13T04:33:43Z</x:v>
       </x:c>
       <x:c r="V10" s="36" t="str">
-        <x:v>2026-07-06T03:09:28Z</x:v>
+        <x:v>2026-07-13T04:33:43Z</x:v>
       </x:c>
       <x:c r="W10" s="36" t="str">
-        <x:v>2026-07-07T03:09:28Z</x:v>
+        <x:v>2026-07-13T06:03:43Z</x:v>
       </x:c>
       <x:c r="X10" s="36"/>
       <x:c r="Y10" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z10" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-lis-2-14d26144/subagent-1</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
       </x:c>
       <x:c r="AA10" s="36"/>
       <x:c r="AB10" s="36"/>
       <x:c r="AC10" s="36" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Reclaim stale #622 heartbeat automation claim and re-claim (lease expired 6 days) (#1460)
Claude-Session: https://claude.ai/code/session_01CdodZrjPToZ48BkaoAfmPn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4916,32 +4916,32 @@
         <x:v>IN_PROGRESS</x:v>
       </x:c>
       <x:c r="R10" s="36" t="str">
-        <x:v>controller/ctrl-lis-2-14d26144/subagent-1</x:v>
+        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
       </x:c>
       <x:c r="S10" s="36"/>
       <x:c r="T10" s="36" t="str">
-        <x:v>d0707cc7-e3ad-4b04-a939-e9e616e61293</x:v>
+        <x:v>0d2a37d1-1e85-4dde-aca2-7b95984e8786</x:v>
       </x:c>
       <x:c r="U10" s="36" t="str">
-        <x:v>2026-07-06T03:09:28Z</x:v>
+        <x:v>2026-07-13T04:33:43Z</x:v>
       </x:c>
       <x:c r="V10" s="36" t="str">
-        <x:v>2026-07-06T03:09:28Z</x:v>
+        <x:v>2026-07-13T04:33:43Z</x:v>
       </x:c>
       <x:c r="W10" s="36" t="str">
-        <x:v>2026-07-07T03:09:28Z</x:v>
+        <x:v>2026-07-13T06:03:43Z</x:v>
       </x:c>
       <x:c r="X10" s="36"/>
       <x:c r="Y10" s="36" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z10" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-lis-2-14d26144/subagent-1</x:v>
+        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
       </x:c>
       <x:c r="AA10" s="36"/>
       <x:c r="AB10" s="36"/>
       <x:c r="AC10" s="36" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #622 automate heartbeat scheduling DONE (PR #1462 merged, reclaimed, ctrl-vm-4027)
Reclaimed the expired ctrl-vm-4039 claim and marked DONE after landing the additive
scheduler implementation in PR #1462.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4913,35 +4913,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q10" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R10" s="36" t="str">
-        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-27</x:v>
       </x:c>
       <x:c r="S10" s="36"/>
       <x:c r="T10" s="36" t="str">
-        <x:v>0d2a37d1-1e85-4dde-aca2-7b95984e8786</x:v>
+        <x:v>ff361dae-b4dc-4ead-9003-4a7816f2ddcf</x:v>
       </x:c>
       <x:c r="U10" s="36" t="str">
-        <x:v>2026-07-13T04:33:43Z</x:v>
+        <x:v>2026-07-19T08:51:56Z</x:v>
       </x:c>
       <x:c r="V10" s="36" t="str">
-        <x:v>2026-07-13T04:33:43Z</x:v>
-      </x:c>
-      <x:c r="W10" s="36" t="str">
-        <x:v>2026-07-13T06:03:43Z</x:v>
-      </x:c>
-      <x:c r="X10" s="36"/>
+        <x:v>2026-07-19T08:52:08Z</x:v>
+      </x:c>
+      <x:c r="W10" s="36"/>
+      <x:c r="X10" s="36" t="str">
+        <x:v>2026-07-19T08:52:08Z</x:v>
+      </x:c>
       <x:c r="Y10" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z10" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
-      </x:c>
-      <x:c r="AA10" s="36"/>
-      <x:c r="AB10" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA10" s="36" t="str">
+        <x:v>Landed the reclaimed #622 implementation (PR #1462): scripts/heartbeat_scheduler.py adds a pure scheduler deriving not_due/due_soon/due/overdue/recovery_required states solely from issue_queue.claimTimingHealth() and one captured UTC timestamp, plus worker-poll evidence validation (identity/liveness/freshness), read-only planning + apply --dry-run, and atomic multi-claim publication under the workbook lock (prevalidate all, one shared timestamp, max(existing,now+lease) preservation, single atomicSave, byte restoration on failure). Existing single-claim heartbeat API/CLI unchanged. Additive tooling only (no build.yml/AGENTS.md changes).</x:v>
+      </x:c>
+      <x:c r="AB10" s="36" t="str">
+        <x:v>CI green on PR #1462 (rebased onto current main): validate/export/linux-fast/linux/windows-deps/windows all success (linux-coverage skipped, no src). tests/test_heartbeat_scheduler.py covers due/overdue boundaries, identity/liveness evidence, duplicate/mixed-validity all-or-nothing batches, lease preservation, single-save multi-row, byte preservation, CLI immutability. Squash-merged to main as 83e47380.</x:v>
+      </x:c>
       <x:c r="AC10" s="36" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">

</xml_diff>

<commit_message>
Mark #622 automate heartbeat scheduling DONE (PR #1462 merged, reclaimed, ctrl-vm-4027) (#1475)
Reclaimed the expired ctrl-vm-4039 claim and marked DONE after landing the additive
scheduler implementation in PR #1462.


Claude-Session: https://claude.ai/code/session_01WctWHcx4zSPNJDdKzUvK3b

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
+++ b/planning/fall_of_nouraajd_github_issues_implementation_workbook_migrated.xlsx
@@ -4913,35 +4913,39 @@
 https://raw.githubusercontent.com/lisu188/fall-of-nouraajd/main/docs/codex-agent-queue.md</x:v>
       </x:c>
       <x:c r="Q10" s="36" t="str">
-        <x:v>IN_PROGRESS</x:v>
+        <x:v>DONE</x:v>
       </x:c>
       <x:c r="R10" s="36" t="str">
-        <x:v>controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
+        <x:v>controller/ctrl-vm-4027-c0afa077/subagent-27</x:v>
       </x:c>
       <x:c r="S10" s="36"/>
       <x:c r="T10" s="36" t="str">
-        <x:v>0d2a37d1-1e85-4dde-aca2-7b95984e8786</x:v>
+        <x:v>ff361dae-b4dc-4ead-9003-4a7816f2ddcf</x:v>
       </x:c>
       <x:c r="U10" s="36" t="str">
-        <x:v>2026-07-13T04:33:43Z</x:v>
+        <x:v>2026-07-19T08:51:56Z</x:v>
       </x:c>
       <x:c r="V10" s="36" t="str">
-        <x:v>2026-07-13T04:33:43Z</x:v>
-      </x:c>
-      <x:c r="W10" s="36" t="str">
-        <x:v>2026-07-13T06:03:43Z</x:v>
-      </x:c>
-      <x:c r="X10" s="36"/>
+        <x:v>2026-07-19T08:52:08Z</x:v>
+      </x:c>
+      <x:c r="W10" s="36"/>
+      <x:c r="X10" s="36" t="str">
+        <x:v>2026-07-19T08:52:08Z</x:v>
+      </x:c>
       <x:c r="Y10" s="36" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="Z10" s="36" t="str">
-        <x:v>Claimed by controller/ctrl-vm-4039-a70f65a5/subagent-63</x:v>
-      </x:c>
-      <x:c r="AA10" s="36"/>
-      <x:c r="AB10" s="36"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="AA10" s="36" t="str">
+        <x:v>Landed the reclaimed #622 implementation (PR #1462): scripts/heartbeat_scheduler.py adds a pure scheduler deriving not_due/due_soon/due/overdue/recovery_required states solely from issue_queue.claimTimingHealth() and one captured UTC timestamp, plus worker-poll evidence validation (identity/liveness/freshness), read-only planning + apply --dry-run, and atomic multi-claim publication under the workbook lock (prevalidate all, one shared timestamp, max(existing,now+lease) preservation, single atomicSave, byte restoration on failure). Existing single-claim heartbeat API/CLI unchanged. Additive tooling only (no build.yml/AGENTS.md changes).</x:v>
+      </x:c>
+      <x:c r="AB10" s="36" t="str">
+        <x:v>CI green on PR #1462 (rebased onto current main): validate/export/linux-fast/linux/windows-deps/windows all success (linux-coverage skipped, no src). tests/test_heartbeat_scheduler.py covers due/overdue boundaries, identity/liveness evidence, duplicate/mixed-validity all-or-nothing batches, lease preservation, single-save multi-row, byte preservation, CLI immutability. Squash-merged to main as 83e47380.</x:v>
+      </x:c>
       <x:c r="AC10" s="36" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">

</xml_diff>